<commit_message>
Update MLF data 2026-10-05
</commit_message>
<xml_diff>
--- a/outputs/NSW_mlf.xlsx
+++ b/outputs/NSW_mlf.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -725,27 +725,25 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>White Rock Wind Farm</t>
+          <t>White Rock Solar Farm</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>175</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -788,25 +786,27 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>White Rock Solar Farm</t>
+          <t>White Rock Wind Farm</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>22</v>
+        <v>175</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="H5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -1748,12 +1748,12 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Junee Solar Farm</t>
+          <t>West Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1762,19 +1762,15 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr"/>
       <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="n">
-        <v>0.9645</v>
-      </c>
-      <c r="K21" s="5" t="n">
-        <v>0.8799</v>
-      </c>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -1805,12 +1801,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Sebastopol Solar Farm</t>
+          <t>Junee Solar Farm</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1819,14 +1815,16 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>110</v>
+        <v>36</v>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
       <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr"/>
       <c r="H22" s="5" t="inlineStr"/>
       <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="n">
+        <v>0.9645</v>
+      </c>
       <c r="K22" s="5" t="n">
         <v>0.8799</v>
       </c>
@@ -1860,12 +1858,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>West Wyalong Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1874,7 +1872,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1913,12 +1911,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>Sebastopol Solar Farm</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1927,7 +1925,7 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>62</v>
+        <v>110</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
@@ -1935,7 +1933,9 @@
       <c r="H24" s="5" t="inlineStr"/>
       <c r="I24" s="5" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr"/>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="n">
+        <v>0.8799</v>
+      </c>
       <c r="L24" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -2113,7 +2113,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -2166,7 +2166,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -2219,12 +2219,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>CRWASF1</t>
+          <t>MULWASF1</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Corowa Solar Farm</t>
+          <t>Mulwala Solar Farm</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2233,31 +2233,21 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr"/>
       <c r="H30" s="5" t="inlineStr"/>
       <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="n">
-        <v>0.9497</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>0.8813</v>
-      </c>
-      <c r="L30" s="5" t="n">
-        <v>0.9242</v>
-      </c>
-      <c r="M30" s="5" t="n">
-        <v>0.9365</v>
-      </c>
-      <c r="N30" s="5" t="n">
-        <v>0.8979</v>
-      </c>
+      <c r="J30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr"/>
+      <c r="M30" s="5" t="inlineStr"/>
+      <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr"/>
       <c r="P30" s="5" t="n">
-        <v>0.9355</v>
+        <v>0.9345</v>
       </c>
       <c r="Q30" s="5" t="inlineStr"/>
       <c r="R30" s="5" t="n">
@@ -2265,10 +2255,10 @@
       </c>
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="n">
-        <v>-0.0443</v>
+        <v>-0.0433</v>
       </c>
       <c r="U30" s="6" t="n">
-        <v>-4.74</v>
+        <v>-4.63</v>
       </c>
       <c r="V30" s="5" t="inlineStr"/>
       <c r="W30" s="6" t="inlineStr"/>
@@ -2276,12 +2266,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>MULWASF1</t>
+          <t>CRWASF1</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Mulwala Solar Farm</t>
+          <t>Corowa Solar Farm</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2290,21 +2280,31 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr"/>
       <c r="H31" s="5" t="inlineStr"/>
       <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
-      <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr"/>
-      <c r="M31" s="5" t="inlineStr"/>
-      <c r="N31" s="5" t="inlineStr"/>
+      <c r="J31" s="5" t="n">
+        <v>0.9497</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>0.9365</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>0.8979</v>
+      </c>
       <c r="O31" s="5" t="inlineStr"/>
       <c r="P31" s="5" t="n">
-        <v>0.9345</v>
+        <v>0.9355</v>
       </c>
       <c r="Q31" s="5" t="inlineStr"/>
       <c r="R31" s="5" t="n">
@@ -2312,10 +2312,10 @@
       </c>
       <c r="S31" s="5" t="inlineStr"/>
       <c r="T31" s="5" t="n">
-        <v>-0.0433</v>
+        <v>-0.0443</v>
       </c>
       <c r="U31" s="6" t="n">
-        <v>-4.63</v>
+        <v>-4.74</v>
       </c>
       <c r="V31" s="5" t="inlineStr"/>
       <c r="W31" s="6" t="inlineStr"/>
@@ -2781,7 +2781,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>NESBESS1</t>
+          <t>NESBESS2</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NESBESS2</t>
+          <t>NESBESS1</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -3013,7 +3013,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -3080,7 +3080,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -3147,7 +3147,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -3214,7 +3214,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -3399,12 +3399,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Nevertire Solar Farm</t>
+          <t xml:space="preserve">Wellington Solar Farm </t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3413,15 +3413,13 @@
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>132</v>
+        <v>216</v>
       </c>
       <c r="E50" s="5" t="inlineStr"/>
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr"/>
       <c r="H50" s="5" t="inlineStr"/>
-      <c r="I50" s="5" t="n">
-        <v>0.9582000000000001</v>
-      </c>
+      <c r="I50" s="5" t="inlineStr"/>
       <c r="J50" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -3458,12 +3456,12 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
+          <t>NASF1</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>South Keswick Solar Farm</t>
+          <t>Narromine Solar Farm</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3472,7 +3470,7 @@
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
       <c r="F51" s="5" t="inlineStr"/>
@@ -3521,12 +3519,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Narromine Solar Farm</t>
+          <t>Nevertire Solar Farm</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3535,16 +3533,12 @@
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>10</v>
+        <v>132</v>
       </c>
       <c r="E52" s="5" t="inlineStr"/>
       <c r="F52" s="5" t="inlineStr"/>
-      <c r="G52" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="H52" s="5" t="n">
-        <v>0.9708</v>
-      </c>
+      <c r="G52" s="5" t="inlineStr"/>
+      <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="n">
         <v>0.9582000000000001</v>
       </c>
@@ -3651,12 +3645,12 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wellington Solar Farm </t>
+          <t>South Keswick Solar Farm</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -3665,13 +3659,19 @@
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>216</v>
+        <v>15</v>
       </c>
       <c r="E54" s="5" t="inlineStr"/>
       <c r="F54" s="5" t="inlineStr"/>
-      <c r="G54" s="5" t="inlineStr"/>
-      <c r="H54" s="5" t="inlineStr"/>
-      <c r="I54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="H54" s="5" t="n">
+        <v>0.9708</v>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="J54" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -3940,12 +3940,12 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>STUBSF1</t>
+          <t>STUBSF2</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Stubbo Solar Farm 1</t>
+          <t>Stubbo Solar Farm 2</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3954,7 +3954,7 @@
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E59" s="5" t="inlineStr"/>
       <c r="F59" s="5" t="inlineStr"/>
@@ -3989,12 +3989,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>STUBSF2</t>
+          <t>STUBSF1</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Stubbo Solar Farm 2</t>
+          <t>Stubbo Solar Farm 1</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -4003,7 +4003,7 @@
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="E60" s="5" t="inlineStr"/>
       <c r="F60" s="5" t="inlineStr"/>
@@ -4491,12 +4491,12 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Gunning Wind Farm</t>
+          <t>Cullerin Range Wind Farm</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>46.5</v>
+        <v>30</v>
       </c>
       <c r="E68" s="5" t="n">
         <v>0.9742</v>
@@ -4558,12 +4558,12 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Cullerin Range Wind Farm</t>
+          <t>Gunning Wind Farm</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -4572,7 +4572,7 @@
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>30</v>
+        <v>46.5</v>
       </c>
       <c r="E69" s="5" t="n">
         <v>0.9742</v>
@@ -5238,7 +5238,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>BW03</t>
+          <t>BW04</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>BW04</t>
+          <t>BW03</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -5372,7 +5372,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>BW01</t>
+          <t>BW02</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -5439,7 +5439,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>BW02</t>
+          <t>BW01</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -5506,30 +5506,26 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>GULLRSF1</t>
+          <t>GULLRWF2</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Gullen Range Solar Farm</t>
+          <t>Gullen Range Wind Farm</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D85" s="4" t="n">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="E85" s="5" t="inlineStr"/>
       <c r="F85" s="5" t="inlineStr"/>
-      <c r="G85" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="H85" s="5" t="n">
-        <v>0.9959</v>
-      </c>
+      <c r="G85" s="5" t="inlineStr"/>
+      <c r="H85" s="5" t="inlineStr"/>
       <c r="I85" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -5569,7 +5565,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF2</t>
+          <t>GULLRWF1</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -5583,12 +5579,20 @@
         </is>
       </c>
       <c r="D86" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="E86" s="5" t="inlineStr"/>
-      <c r="F86" s="5" t="inlineStr"/>
-      <c r="G86" s="5" t="inlineStr"/>
-      <c r="H86" s="5" t="inlineStr"/>
+        <v>165</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="F86" s="5" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="G86" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="H86" s="5" t="n">
+        <v>0.9959</v>
+      </c>
       <c r="I86" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -5628,28 +5632,24 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF1</t>
+          <t>GULLRSF1</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Gullen Range Wind Farm</t>
+          <t>Gullen Range Solar Farm</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D87" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="E87" s="5" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="F87" s="5" t="n">
-        <v>0.9909</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E87" s="5" t="inlineStr"/>
+      <c r="F87" s="5" t="inlineStr"/>
       <c r="G87" s="5" t="n">
         <v>1.001</v>
       </c>
@@ -6120,12 +6120,12 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Wind Farm</t>
+          <t>Capital Wind Farm</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -6134,7 +6134,7 @@
         </is>
       </c>
       <c r="D95" s="4" t="n">
-        <v>48.3</v>
+        <v>140</v>
       </c>
       <c r="E95" s="5" t="n">
         <v>0.9748</v>
@@ -6187,12 +6187,12 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Capital Wind Farm</t>
+          <t>Woodlawn Wind Farm</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -6201,7 +6201,7 @@
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>140</v>
+        <v>48.3</v>
       </c>
       <c r="E96" s="5" t="n">
         <v>0.9748</v>
@@ -6520,12 +6520,12 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MPNL1</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Mt Piper Power Station</t>
+          <t>MT PIPER POWER STATION</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -6534,7 +6534,7 @@
         </is>
       </c>
       <c r="D101" s="4" t="n">
-        <v>700</v>
+        <v>25</v>
       </c>
       <c r="E101" s="5" t="n">
         <v>0.9744</v>
@@ -6654,12 +6654,12 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>MPNL1</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>MT PIPER POWER STATION</t>
+          <t>Mt Piper Power Station</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -6668,7 +6668,7 @@
         </is>
       </c>
       <c r="D103" s="4" t="n">
-        <v>25</v>
+        <v>700</v>
       </c>
       <c r="E103" s="5" t="n">
         <v>0.9744</v>
@@ -6914,7 +6914,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -6977,17 +6977,17 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
+          <t>TUMUT2</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr"/>
       <c r="D108" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E108" s="5" t="n">
         <v>0.9768</v>
@@ -7040,17 +7040,17 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-2</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
+          <t>TUMUT2</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr"/>
       <c r="D109" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E109" s="5" t="n">
         <v>0.9768</v>
@@ -7103,17 +7103,17 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
+          <t>TUMUT2</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr"/>
       <c r="D110" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E110" s="5" t="n">
         <v>0.9768</v>
@@ -7166,17 +7166,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-2</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
+          <t>TUMUT1</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr"/>
       <c r="D111" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E111" s="5" t="n">
         <v>0.9768</v>
@@ -7229,17 +7229,17 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
+          <t>TUMUT1</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr"/>
       <c r="D112" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E112" s="5" t="n">
         <v>0.9768</v>
@@ -7292,17 +7292,17 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
+          <t>TUMUT1</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr"/>
       <c r="D113" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E113" s="5" t="n">
         <v>0.9768</v>
@@ -7482,17 +7482,13 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Eraring Battery Energy Storage System 2</t>
-        </is>
-      </c>
-      <c r="C116" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="D116" s="4" t="n">
-        <v>351</v>
-      </c>
+          <t>ERBESS2</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="n">
+        <v/>
+      </c>
+      <c r="D116" s="3" t="inlineStr"/>
       <c r="E116" s="5" t="inlineStr"/>
       <c r="F116" s="5" t="inlineStr"/>
       <c r="G116" s="5" t="inlineStr"/>
@@ -7705,7 +7701,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -7839,7 +7835,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -7965,12 +7961,12 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>HEZ1</t>
+          <t>ER01</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>Hunter Economic Zone</t>
+          <t>Eraring Power Station</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -7979,29 +7975,41 @@
         </is>
       </c>
       <c r="D124" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="E124" s="5" t="inlineStr"/>
-      <c r="F124" s="5" t="inlineStr"/>
-      <c r="G124" s="5" t="inlineStr"/>
-      <c r="H124" s="5" t="inlineStr"/>
-      <c r="I124" s="5" t="inlineStr"/>
-      <c r="J124" s="5" t="inlineStr"/>
+        <v>720</v>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="F124" s="5" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="G124" s="5" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="H124" s="5" t="n">
+        <v>0.9828</v>
+      </c>
+      <c r="I124" s="5" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="J124" s="5" t="n">
+        <v>0.9835</v>
+      </c>
       <c r="K124" s="5" t="n">
-        <v>0.9897</v>
+        <v>0.9849</v>
       </c>
       <c r="L124" s="5" t="n">
-        <v>0.992</v>
+        <v>0.9865</v>
       </c>
       <c r="M124" s="5" t="n">
-        <v>0.9899</v>
+        <v>0.9848</v>
       </c>
       <c r="N124" s="5" t="n">
-        <v>0.9896</v>
+        <v>0.9855</v>
       </c>
       <c r="O124" s="5" t="inlineStr"/>
       <c r="P124" s="5" t="n">
-        <v>0.9931</v>
+        <v>0.9846</v>
       </c>
       <c r="Q124" s="5" t="inlineStr"/>
       <c r="R124" s="5" t="n">
@@ -8009,10 +8017,10 @@
       </c>
       <c r="S124" s="5" t="inlineStr"/>
       <c r="T124" s="5" t="n">
-        <v>-0.01</v>
+        <v>-0.0015</v>
       </c>
       <c r="U124" s="6" t="n">
-        <v>-1.01</v>
+        <v>-0.15</v>
       </c>
       <c r="V124" s="5" t="inlineStr"/>
       <c r="W124" s="6" t="inlineStr"/>
@@ -8020,7 +8028,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -8034,7 +8042,7 @@
         </is>
       </c>
       <c r="D125" s="4" t="n">
-        <v>41.5</v>
+        <v>720</v>
       </c>
       <c r="E125" s="5" t="n">
         <v>0.9856</v>
@@ -8087,7 +8095,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -8101,7 +8109,7 @@
         </is>
       </c>
       <c r="D126" s="4" t="n">
-        <v>720</v>
+        <v>41.5</v>
       </c>
       <c r="E126" s="5" t="n">
         <v>0.9856</v>
@@ -8154,12 +8162,12 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
+          <t>HEZ1</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>Eraring Power Station</t>
+          <t>Hunter Economic Zone</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -8168,41 +8176,29 @@
         </is>
       </c>
       <c r="D127" s="4" t="n">
-        <v>720</v>
-      </c>
-      <c r="E127" s="5" t="n">
-        <v>0.9856</v>
-      </c>
-      <c r="F127" s="5" t="n">
-        <v>0.9829</v>
-      </c>
-      <c r="G127" s="5" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="H127" s="5" t="n">
-        <v>0.9828</v>
-      </c>
-      <c r="I127" s="5" t="n">
-        <v>0.9836</v>
-      </c>
-      <c r="J127" s="5" t="n">
-        <v>0.9835</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="E127" s="5" t="inlineStr"/>
+      <c r="F127" s="5" t="inlineStr"/>
+      <c r="G127" s="5" t="inlineStr"/>
+      <c r="H127" s="5" t="inlineStr"/>
+      <c r="I127" s="5" t="inlineStr"/>
+      <c r="J127" s="5" t="inlineStr"/>
       <c r="K127" s="5" t="n">
-        <v>0.9849</v>
+        <v>0.9897</v>
       </c>
       <c r="L127" s="5" t="n">
-        <v>0.9865</v>
+        <v>0.992</v>
       </c>
       <c r="M127" s="5" t="n">
-        <v>0.9848</v>
+        <v>0.9899</v>
       </c>
       <c r="N127" s="5" t="n">
-        <v>0.9855</v>
+        <v>0.9896</v>
       </c>
       <c r="O127" s="5" t="inlineStr"/>
       <c r="P127" s="5" t="n">
-        <v>0.9846</v>
+        <v>0.9931</v>
       </c>
       <c r="Q127" s="5" t="inlineStr"/>
       <c r="R127" s="5" t="n">
@@ -8210,10 +8206,10 @@
       </c>
       <c r="S127" s="5" t="inlineStr"/>
       <c r="T127" s="5" t="n">
-        <v>-0.0015</v>
+        <v>-0.01</v>
       </c>
       <c r="U127" s="6" t="n">
-        <v>-0.15</v>
+        <v>-1.01</v>
       </c>
       <c r="V127" s="5" t="inlineStr"/>
       <c r="W127" s="6" t="inlineStr"/>
@@ -8607,7 +8603,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -8674,7 +8670,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -8741,7 +8737,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -8808,7 +8804,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -8875,7 +8871,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -9122,17 +9118,13 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Williamsdale BESS</t>
-        </is>
-      </c>
-      <c r="C142" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="D142" s="4" t="n">
-        <v>262</v>
-      </c>
+          <t>WILLBESS</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="n">
+        <v/>
+      </c>
+      <c r="D142" s="3" t="inlineStr"/>
       <c r="E142" s="5" t="inlineStr"/>
       <c r="F142" s="5" t="inlineStr"/>
       <c r="G142" s="5" t="inlineStr"/>
@@ -9223,12 +9215,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>JNDABNE1</t>
+          <t>BROWNMT</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Jindabyne Small Hydro Power Station</t>
+          <t>Brown Mountain Hydro Power Station</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -9237,7 +9229,7 @@
         </is>
       </c>
       <c r="D144" s="4" t="n">
-        <v>1.1</v>
+        <v>5</v>
       </c>
       <c r="E144" s="5" t="n">
         <v>0.9762999999999999</v>
@@ -9290,12 +9282,12 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>BROWNMT</t>
+          <t>JNDABNE1</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Brown Mountain Hydro Power Station</t>
+          <t>Jindabyne Small Hydro Power Station</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -9304,7 +9296,7 @@
         </is>
       </c>
       <c r="D145" s="4" t="n">
-        <v>5</v>
+        <v>1.1</v>
       </c>
       <c r="E145" s="5" t="n">
         <v>0.9762999999999999</v>
@@ -9491,12 +9483,12 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>SHOAL1</t>
+          <t>WESTILL1</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Shoalhaven Starches Cogeneration Plant</t>
+          <t>West Illawarra Leagues Club Plant</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -9505,16 +9497,32 @@
         </is>
       </c>
       <c r="D148" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="E148" s="5" t="inlineStr"/>
-      <c r="F148" s="5" t="inlineStr"/>
-      <c r="G148" s="5" t="inlineStr"/>
-      <c r="H148" s="5" t="inlineStr"/>
-      <c r="I148" s="5" t="inlineStr"/>
-      <c r="J148" s="5" t="inlineStr"/>
-      <c r="K148" s="5" t="inlineStr"/>
-      <c r="L148" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E148" s="5" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="F148" s="5" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="G148" s="5" t="n">
+        <v>1.0023</v>
+      </c>
+      <c r="H148" s="5" t="n">
+        <v>1.0037</v>
+      </c>
+      <c r="I148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="J148" s="5" t="n">
+        <v>0.9967</v>
+      </c>
+      <c r="K148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="L148" s="5" t="n">
+        <v>0.9933999999999999</v>
+      </c>
       <c r="M148" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -9542,12 +9550,12 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>WESTILL1</t>
+          <t>SHOAL1</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>West Illawarra Leagues Club Plant</t>
+          <t>Shoalhaven Starches Cogeneration Plant</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -9556,32 +9564,16 @@
         </is>
       </c>
       <c r="D149" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E149" s="5" t="n">
-        <v>0.9916</v>
-      </c>
-      <c r="F149" s="5" t="n">
-        <v>0.9986</v>
-      </c>
-      <c r="G149" s="5" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="H149" s="5" t="n">
-        <v>1.0037</v>
-      </c>
-      <c r="I149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="J149" s="5" t="n">
-        <v>0.9967</v>
-      </c>
-      <c r="K149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="L149" s="5" t="n">
-        <v>0.9933999999999999</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E149" s="5" t="inlineStr"/>
+      <c r="F149" s="5" t="inlineStr"/>
+      <c r="G149" s="5" t="inlineStr"/>
+      <c r="H149" s="5" t="inlineStr"/>
+      <c r="I149" s="5" t="inlineStr"/>
+      <c r="J149" s="5" t="inlineStr"/>
+      <c r="K149" s="5" t="inlineStr"/>
+      <c r="L149" s="5" t="inlineStr"/>
       <c r="M149" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -9802,12 +9794,12 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>Wyangala B Power Station</t>
+          <t>Wyangala A Power Station</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
@@ -9816,7 +9808,7 @@
         </is>
       </c>
       <c r="D153" s="4" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E153" s="5" t="n">
         <v>1.0099</v>
@@ -9869,12 +9861,12 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>Wyangala A Power Station</t>
+          <t>Wyangala B Power Station</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -9883,7 +9875,7 @@
         </is>
       </c>
       <c r="D154" s="4" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E154" s="5" t="n">
         <v>1.0099</v>
@@ -10549,7 +10541,7 @@
         </is>
       </c>
       <c r="D164" s="4" t="n">
-        <v>4.492</v>
+        <v>6.738</v>
       </c>
       <c r="E164" s="5" t="n">
         <v>1.0021</v>
@@ -10602,12 +10594,12 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>SMTHBES1</t>
+          <t>WALGRV1</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Smithfield Battery Energy Storage System, Units 1 - 36</t>
+          <t>Wallgrove BESS 1</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -10616,7 +10608,7 @@
         </is>
       </c>
       <c r="D165" s="4" t="n">
-        <v>69.40000000000001</v>
+        <v>50</v>
       </c>
       <c r="E165" s="5" t="inlineStr"/>
       <c r="F165" s="5" t="inlineStr"/>
@@ -10627,25 +10619,29 @@
       <c r="K165" s="5" t="inlineStr"/>
       <c r="L165" s="5" t="inlineStr"/>
       <c r="M165" s="5" t="inlineStr"/>
-      <c r="N165" s="5" t="inlineStr"/>
-      <c r="O165" s="5" t="inlineStr"/>
+      <c r="N165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="O165" s="5" t="n">
+        <v>1.0009</v>
+      </c>
       <c r="P165" s="5" t="n">
-        <v>1.0016</v>
+        <v>1.0018</v>
       </c>
       <c r="Q165" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0015</v>
       </c>
       <c r="R165" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="S165" s="5" t="n">
-        <v>1.0019</v>
+        <v>1.0017</v>
       </c>
       <c r="T165" s="5" t="n">
-        <v>0.0001</v>
+        <v>-0.0001</v>
       </c>
       <c r="U165" s="6" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="V165" s="5" t="n">
         <v>0.0002</v>
@@ -10657,12 +10653,12 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>WALGRV1</t>
+          <t>SMTHBES1</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>Wallgrove BESS 1</t>
+          <t>Smithfield Battery Energy Storage System, Units 1 - 36</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -10671,7 +10667,7 @@
         </is>
       </c>
       <c r="D166" s="4" t="n">
-        <v>50</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="E166" s="5" t="inlineStr"/>
       <c r="F166" s="5" t="inlineStr"/>
@@ -10682,29 +10678,25 @@
       <c r="K166" s="5" t="inlineStr"/>
       <c r="L166" s="5" t="inlineStr"/>
       <c r="M166" s="5" t="inlineStr"/>
-      <c r="N166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="O166" s="5" t="n">
-        <v>1.0009</v>
-      </c>
+      <c r="N166" s="5" t="inlineStr"/>
+      <c r="O166" s="5" t="inlineStr"/>
       <c r="P166" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0016</v>
       </c>
       <c r="Q166" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0017</v>
       </c>
       <c r="R166" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="S166" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0019</v>
       </c>
       <c r="T166" s="5" t="n">
-        <v>-0.0001</v>
+        <v>0.0001</v>
       </c>
       <c r="U166" s="6" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="V166" s="5" t="n">
         <v>0.0002</v>
@@ -10783,21 +10775,21 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>Taralga Wind Farm</t>
+          <t>Woodlawn Bioreactor Energy Generation Station</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D168" s="4" t="n">
-        <v>106.8</v>
+        <v>7</v>
       </c>
       <c r="E168" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -10850,21 +10842,21 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Bioreactor Energy Generation Station</t>
+          <t>Taralga Wind Farm</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D169" s="4" t="n">
-        <v>7</v>
+        <v>106.8</v>
       </c>
       <c r="E169" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -11035,7 +11027,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -11098,7 +11090,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -11161,7 +11153,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -11224,7 +11216,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -11287,7 +11279,7 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -11350,7 +11342,7 @@
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -11636,12 +11628,12 @@
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
+          <t>AGLSITA1</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>West Nowra Landfill Gas Power Generation Facility</t>
+          <t>AGL KEMPS CREEK</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
@@ -11652,26 +11644,24 @@
       <c r="D183" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E183" s="5" t="n">
-        <v>0.9916</v>
-      </c>
+      <c r="E183" s="5" t="inlineStr"/>
       <c r="F183" s="5" t="n">
-        <v>0.9986</v>
+        <v>1.0019</v>
       </c>
       <c r="G183" s="5" t="n">
-        <v>1.0023</v>
+        <v>1.0022</v>
       </c>
       <c r="H183" s="5" t="n">
-        <v>1.0037</v>
+        <v>1.0024</v>
       </c>
       <c r="I183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0009</v>
       </c>
       <c r="J183" s="5" t="n">
-        <v>0.9967</v>
+        <v>1.0012</v>
       </c>
       <c r="K183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0015</v>
       </c>
       <c r="L183" s="5" t="inlineStr"/>
       <c r="M183" s="5" t="inlineStr"/>
@@ -11689,12 +11679,12 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>AGLNOW1</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>TERALBA POWER STATION</t>
+          <t>West Nowra Landfill Gas Power Generation Facility</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
@@ -11703,28 +11693,28 @@
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>0.9926</v>
+        <v>0.9916</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9986</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>0.9892</v>
+        <v>1.0023</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>0.9901</v>
+        <v>1.0037</v>
       </c>
       <c r="I184" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9929</v>
       </c>
       <c r="J184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9967</v>
       </c>
       <c r="K184" s="5" t="n">
-        <v>0.9917</v>
+        <v>0.9929</v>
       </c>
       <c r="L184" s="5" t="inlineStr"/>
       <c r="M184" s="5" t="inlineStr"/>
@@ -11742,42 +11732,42 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Liddell Power Station</t>
+          <t>Kincumber Landfill Site</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Fossil</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="I185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="J185" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="L185" s="5" t="inlineStr"/>
       <c r="M185" s="5" t="inlineStr"/>
@@ -11795,42 +11785,42 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>Kincumber Landfill Site</t>
+          <t>Liddell Power Station</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Fossil</t>
         </is>
       </c>
       <c r="D186" s="4" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9676</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9593</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9509</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9537</v>
       </c>
       <c r="I186" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9593</v>
       </c>
       <c r="J186" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9631</v>
       </c>
       <c r="K186" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9628</v>
       </c>
       <c r="L186" s="5" t="inlineStr"/>
       <c r="M186" s="5" t="inlineStr"/>
@@ -11897,12 +11887,12 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>Woy Woy Landfill Site</t>
+          <t>TERALBA POWER STATION</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -11911,28 +11901,28 @@
         </is>
       </c>
       <c r="D188" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9926</v>
       </c>
       <c r="F188" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9907</v>
       </c>
       <c r="G188" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9892</v>
       </c>
       <c r="H188" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9901</v>
       </c>
       <c r="I188" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="J188" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9907</v>
       </c>
       <c r="K188" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9917</v>
       </c>
       <c r="L188" s="5" t="inlineStr"/>
       <c r="M188" s="5" t="inlineStr"/>
@@ -11950,12 +11940,12 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>AGLSITA1</t>
+          <t>WOYWOY1</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>AGL KEMPS CREEK</t>
+          <t>Woy Woy Landfill Site</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
@@ -11966,24 +11956,26 @@
       <c r="D189" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E189" s="5" t="inlineStr"/>
+      <c r="E189" s="5" t="n">
+        <v>1.0017</v>
+      </c>
       <c r="F189" s="5" t="n">
+        <v>1.0015</v>
+      </c>
+      <c r="G189" s="5" t="n">
+        <v>1.0008</v>
+      </c>
+      <c r="H189" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="I189" s="5" t="n">
+        <v>1.0036</v>
+      </c>
+      <c r="J189" s="5" t="n">
         <v>1.0019</v>
       </c>
-      <c r="G189" s="5" t="n">
-        <v>1.0022</v>
-      </c>
-      <c r="H189" s="5" t="n">
-        <v>1.0024</v>
-      </c>
-      <c r="I189" s="5" t="n">
-        <v>1.0009</v>
-      </c>
-      <c r="J189" s="5" t="n">
-        <v>1.0012</v>
-      </c>
       <c r="K189" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0037</v>
       </c>
       <c r="L189" s="5" t="inlineStr"/>
       <c r="M189" s="5" t="inlineStr"/>
@@ -12001,7 +11993,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>LD04</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -12056,7 +12048,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD04</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
@@ -12111,7 +12103,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -12166,12 +12158,12 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>WALGRVG1</t>
+          <t>QBYNBG1</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>Wallgrove BESS 1</t>
+          <t>Queanbeyan BESS</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
@@ -12180,7 +12172,7 @@
         </is>
       </c>
       <c r="D193" s="4" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E193" s="5" t="inlineStr"/>
       <c r="F193" s="5" t="inlineStr"/>
@@ -12188,17 +12180,15 @@
       <c r="H193" s="5" t="inlineStr"/>
       <c r="I193" s="5" t="inlineStr"/>
       <c r="J193" s="5" t="inlineStr"/>
-      <c r="K193" s="5" t="n">
-        <v>1.0011</v>
-      </c>
+      <c r="K193" s="5" t="inlineStr"/>
       <c r="L193" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9752</v>
       </c>
       <c r="M193" s="5" t="n">
-        <v>1.001</v>
+        <v>0.979</v>
       </c>
       <c r="N193" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9571</v>
       </c>
       <c r="O193" s="5" t="inlineStr"/>
       <c r="P193" s="5" t="inlineStr"/>
@@ -12213,12 +12203,12 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>DPNTBG1</t>
+          <t>BHBG1</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>Darlington Point Energy Storage System</t>
+          <t>Broken Hill Battery Energy Storage System</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
@@ -12227,7 +12217,7 @@
         </is>
       </c>
       <c r="D194" s="4" t="n">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="E194" s="5" t="inlineStr"/>
       <c r="F194" s="5" t="inlineStr"/>
@@ -12236,14 +12226,12 @@
       <c r="I194" s="5" t="inlineStr"/>
       <c r="J194" s="5" t="inlineStr"/>
       <c r="K194" s="5" t="inlineStr"/>
-      <c r="L194" s="5" t="n">
-        <v>0.9402</v>
-      </c>
+      <c r="L194" s="5" t="inlineStr"/>
       <c r="M194" s="5" t="n">
-        <v>0.9089</v>
+        <v>0.8671</v>
       </c>
       <c r="N194" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.8423</v>
       </c>
       <c r="O194" s="5" t="inlineStr"/>
       <c r="P194" s="5" t="inlineStr"/>
@@ -12258,21 +12246,21 @@
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>MLLFGEF1</t>
+          <t>CAPBES1G</t>
         </is>
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>Mugga Lane Landfill Gas To Energy Facility</t>
+          <t>Capital Battery</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Battery</t>
         </is>
       </c>
       <c r="D195" s="4" t="n">
-        <v>4</v>
+        <v>125</v>
       </c>
       <c r="E195" s="5" t="inlineStr"/>
       <c r="F195" s="5" t="inlineStr"/>
@@ -12280,17 +12268,13 @@
       <c r="H195" s="5" t="inlineStr"/>
       <c r="I195" s="5" t="inlineStr"/>
       <c r="J195" s="5" t="inlineStr"/>
-      <c r="K195" s="5" t="n">
-        <v>0.9683</v>
-      </c>
-      <c r="L195" s="5" t="n">
-        <v>0.9687</v>
-      </c>
+      <c r="K195" s="5" t="inlineStr"/>
+      <c r="L195" s="5" t="inlineStr"/>
       <c r="M195" s="5" t="n">
-        <v>0.9663</v>
+        <v>0.9704</v>
       </c>
       <c r="N195" s="5" t="n">
-        <v>0.9567</v>
+        <v>0.9337</v>
       </c>
       <c r="O195" s="5" t="inlineStr"/>
       <c r="P195" s="5" t="inlineStr"/>
@@ -12305,12 +12289,12 @@
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
         <is>
-          <t>BHBG1</t>
+          <t>WALGRVG1</t>
         </is>
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>Broken Hill Battery Energy Storage System</t>
+          <t>Wallgrove BESS 1</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
@@ -12319,7 +12303,7 @@
         </is>
       </c>
       <c r="D196" s="4" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="E196" s="5" t="inlineStr"/>
       <c r="F196" s="5" t="inlineStr"/>
@@ -12327,13 +12311,17 @@
       <c r="H196" s="5" t="inlineStr"/>
       <c r="I196" s="5" t="inlineStr"/>
       <c r="J196" s="5" t="inlineStr"/>
-      <c r="K196" s="5" t="inlineStr"/>
-      <c r="L196" s="5" t="inlineStr"/>
+      <c r="K196" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="L196" s="5" t="n">
+        <v>1.001</v>
+      </c>
       <c r="M196" s="5" t="n">
-        <v>0.8671</v>
+        <v>1.001</v>
       </c>
       <c r="N196" s="5" t="n">
-        <v>0.8423</v>
+        <v>1.001</v>
       </c>
       <c r="O196" s="5" t="inlineStr"/>
       <c r="P196" s="5" t="inlineStr"/>
@@ -12348,12 +12336,12 @@
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
         <is>
-          <t>RESS1G</t>
+          <t>DPNTBG1</t>
         </is>
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>Riverina BESS 1</t>
+          <t>Darlington Point Energy Storage System</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
@@ -12362,7 +12350,7 @@
         </is>
       </c>
       <c r="D197" s="4" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="E197" s="5" t="inlineStr"/>
       <c r="F197" s="5" t="inlineStr"/>
@@ -12372,13 +12360,13 @@
       <c r="J197" s="5" t="inlineStr"/>
       <c r="K197" s="5" t="inlineStr"/>
       <c r="L197" s="5" t="n">
-        <v>0.9286</v>
+        <v>0.9402</v>
       </c>
       <c r="M197" s="5" t="n">
         <v>0.9089</v>
       </c>
       <c r="N197" s="5" t="n">
-        <v>0.8702</v>
+        <v>0.9048</v>
       </c>
       <c r="O197" s="5" t="inlineStr"/>
       <c r="P197" s="5" t="inlineStr"/>
@@ -12393,21 +12381,21 @@
     <row r="198">
       <c r="A198" s="3" t="inlineStr">
         <is>
-          <t>RIVNBG2</t>
+          <t>MLLFGEF1</t>
         </is>
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>Riverina Energy Storage System 2</t>
+          <t>Mugga Lane Landfill Gas To Energy Facility</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D198" s="4" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E198" s="5" t="inlineStr"/>
       <c r="F198" s="5" t="inlineStr"/>
@@ -12415,15 +12403,17 @@
       <c r="H198" s="5" t="inlineStr"/>
       <c r="I198" s="5" t="inlineStr"/>
       <c r="J198" s="5" t="inlineStr"/>
-      <c r="K198" s="5" t="inlineStr"/>
+      <c r="K198" s="5" t="n">
+        <v>0.9683</v>
+      </c>
       <c r="L198" s="5" t="n">
-        <v>0.9058</v>
+        <v>0.9687</v>
       </c>
       <c r="M198" s="5" t="n">
-        <v>0.9106</v>
+        <v>0.9663</v>
       </c>
       <c r="N198" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.9567</v>
       </c>
       <c r="O198" s="5" t="inlineStr"/>
       <c r="P198" s="5" t="inlineStr"/>
@@ -12438,12 +12428,12 @@
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
         <is>
-          <t>QBYNBG1</t>
+          <t>RESS1G</t>
         </is>
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>Queanbeyan BESS</t>
+          <t>Riverina BESS 1</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
@@ -12452,7 +12442,7 @@
         </is>
       </c>
       <c r="D199" s="4" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="E199" s="5" t="inlineStr"/>
       <c r="F199" s="5" t="inlineStr"/>
@@ -12462,13 +12452,13 @@
       <c r="J199" s="5" t="inlineStr"/>
       <c r="K199" s="5" t="inlineStr"/>
       <c r="L199" s="5" t="n">
-        <v>0.9752</v>
+        <v>0.9286</v>
       </c>
       <c r="M199" s="5" t="n">
-        <v>0.979</v>
+        <v>0.9089</v>
       </c>
       <c r="N199" s="5" t="n">
-        <v>0.9571</v>
+        <v>0.8702</v>
       </c>
       <c r="O199" s="5" t="inlineStr"/>
       <c r="P199" s="5" t="inlineStr"/>
@@ -12483,12 +12473,12 @@
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
         <is>
-          <t>CAPBES1G</t>
+          <t>RIVNBG2</t>
         </is>
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>Capital Battery</t>
+          <t>Riverina Energy Storage System 2</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
@@ -12497,7 +12487,7 @@
         </is>
       </c>
       <c r="D200" s="4" t="n">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="E200" s="5" t="inlineStr"/>
       <c r="F200" s="5" t="inlineStr"/>
@@ -12506,12 +12496,14 @@
       <c r="I200" s="5" t="inlineStr"/>
       <c r="J200" s="5" t="inlineStr"/>
       <c r="K200" s="5" t="inlineStr"/>
-      <c r="L200" s="5" t="inlineStr"/>
+      <c r="L200" s="5" t="n">
+        <v>0.9058</v>
+      </c>
       <c r="M200" s="5" t="n">
-        <v>0.9704</v>
+        <v>0.9106</v>
       </c>
       <c r="N200" s="5" t="n">
-        <v>0.9337</v>
+        <v>0.9048</v>
       </c>
       <c r="O200" s="5" t="inlineStr"/>
       <c r="P200" s="5" t="inlineStr"/>
@@ -12775,14 +12767,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr"/>
       <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -12817,12 +12807,14 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="E5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -13441,7 +13433,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr"/>
@@ -13449,12 +13441,8 @@
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="5" t="n">
-        <v>0.9645</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>0.8799</v>
-      </c>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
       <c r="I21" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -13477,7 +13465,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr"/>
@@ -13485,7 +13473,9 @@
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr"/>
       <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="n">
+        <v>0.9645</v>
+      </c>
       <c r="H22" s="5" t="n">
         <v>0.8799</v>
       </c>
@@ -13511,7 +13501,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr"/>
@@ -13543,7 +13533,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr"/>
@@ -13552,7 +13542,9 @@
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="n">
+        <v>0.8799</v>
+      </c>
       <c r="I24" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -13659,7 +13651,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr"/>
@@ -13691,7 +13683,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr"/>
@@ -13723,7 +13715,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>CRWASF1</t>
+          <t>MULWASF1</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr"/>
@@ -13731,24 +13723,14 @@
       <c r="D30" s="5" t="inlineStr"/>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="n">
-        <v>0.9497</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>0.8813</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>0.9242</v>
-      </c>
-      <c r="J30" s="5" t="n">
-        <v>0.9365</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>0.8979</v>
-      </c>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="inlineStr"/>
       <c r="L30" s="5" t="inlineStr"/>
       <c r="M30" s="5" t="n">
-        <v>0.9355</v>
+        <v>0.9345</v>
       </c>
       <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="n">
@@ -13759,7 +13741,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>MULWASF1</t>
+          <t>CRWASF1</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr"/>
@@ -13767,14 +13749,24 @@
       <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr"/>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
-      <c r="K31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="n">
+        <v>0.9497</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0.9365</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.8979</v>
+      </c>
       <c r="L31" s="5" t="inlineStr"/>
       <c r="M31" s="5" t="n">
-        <v>0.9345</v>
+        <v>0.9355</v>
       </c>
       <c r="N31" s="5" t="inlineStr"/>
       <c r="O31" s="5" t="n">
@@ -14071,7 +14063,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>NESBESS1</t>
+          <t>NESBESS2</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr"/>
@@ -14101,7 +14093,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NESBESS2</t>
+          <t>NESBESS1</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr"/>
@@ -14211,7 +14203,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
@@ -14257,7 +14249,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
@@ -14303,7 +14295,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
@@ -14349,7 +14341,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
@@ -14471,16 +14463,14 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr"/>
       <c r="C50" s="5" t="inlineStr"/>
       <c r="D50" s="5" t="inlineStr"/>
       <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="n">
-        <v>0.9582000000000001</v>
-      </c>
+      <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -14509,7 +14499,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
+          <t>NASF1</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr"/>
@@ -14551,17 +14541,13 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr"/>
       <c r="C52" s="5" t="inlineStr"/>
-      <c r="D52" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="E52" s="5" t="n">
-        <v>0.9708</v>
-      </c>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr"/>
       <c r="F52" s="5" t="n">
         <v>0.9582000000000001</v>
       </c>
@@ -14639,14 +14625,20 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr"/>
       <c r="C54" s="5" t="inlineStr"/>
-      <c r="D54" s="5" t="inlineStr"/>
-      <c r="E54" s="5" t="inlineStr"/>
-      <c r="F54" s="5" t="inlineStr"/>
+      <c r="D54" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>0.9708</v>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="G54" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -14823,7 +14815,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>STUBSF1</t>
+          <t>STUBSF2</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr"/>
@@ -14851,7 +14843,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>STUBSF2</t>
+          <t>STUBSF1</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr"/>
@@ -15181,7 +15173,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B68" s="5" t="n">
@@ -15227,7 +15219,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B69" s="5" t="n">
@@ -15655,7 +15647,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>BW03</t>
+          <t>BW04</t>
         </is>
       </c>
       <c r="B81" s="5" t="n">
@@ -15701,7 +15693,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>BW04</t>
+          <t>BW03</t>
         </is>
       </c>
       <c r="B82" s="5" t="n">
@@ -15747,7 +15739,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>BW01</t>
+          <t>BW02</t>
         </is>
       </c>
       <c r="B83" s="5" t="n">
@@ -15793,7 +15785,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>BW02</t>
+          <t>BW01</t>
         </is>
       </c>
       <c r="B84" s="5" t="n">
@@ -15839,17 +15831,13 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>GULLRSF1</t>
+          <t>GULLRWF2</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr"/>
       <c r="C85" s="5" t="inlineStr"/>
-      <c r="D85" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="E85" s="5" t="n">
-        <v>0.9959</v>
-      </c>
+      <c r="D85" s="5" t="inlineStr"/>
+      <c r="E85" s="5" t="inlineStr"/>
       <c r="F85" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -15881,13 +15869,21 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF2</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="inlineStr"/>
-      <c r="C86" s="5" t="inlineStr"/>
-      <c r="D86" s="5" t="inlineStr"/>
-      <c r="E86" s="5" t="inlineStr"/>
+          <t>GULLRWF1</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="C86" s="5" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="D86" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v>0.9959</v>
+      </c>
       <c r="F86" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -15919,15 +15915,11 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF1</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="C87" s="5" t="n">
-        <v>0.9909</v>
-      </c>
+          <t>GULLRSF1</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr"/>
+      <c r="C87" s="5" t="inlineStr"/>
       <c r="D87" s="5" t="n">
         <v>1.001</v>
       </c>
@@ -16239,7 +16231,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B95" s="5" t="n">
@@ -16285,7 +16277,7 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B96" s="5" t="n">
@@ -16513,7 +16505,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MPNL1</t>
         </is>
       </c>
       <c r="B101" s="5" t="n">
@@ -16605,7 +16597,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>MPNL1</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B103" s="5" t="n">
@@ -16777,7 +16769,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B107" s="5" t="n">
@@ -16823,7 +16815,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B108" s="5" t="n">
@@ -16869,7 +16861,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-2</t>
         </is>
       </c>
       <c r="B109" s="5" t="n">
@@ -16915,7 +16907,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B110" s="5" t="n">
@@ -16961,7 +16953,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-2</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B111" s="5" t="n">
@@ -17007,7 +16999,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B112" s="5" t="n">
@@ -17053,7 +17045,7 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B113" s="5" t="n">
@@ -17319,7 +17311,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B120" s="5" t="n">
@@ -17411,7 +17403,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B122" s="5" t="n">
@@ -17491,30 +17483,42 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>HEZ1</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="inlineStr"/>
-      <c r="C124" s="5" t="inlineStr"/>
-      <c r="D124" s="5" t="inlineStr"/>
-      <c r="E124" s="5" t="inlineStr"/>
-      <c r="F124" s="5" t="inlineStr"/>
-      <c r="G124" s="5" t="inlineStr"/>
+          <t>ER01</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="C124" s="5" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="D124" s="5" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>0.9828</v>
+      </c>
+      <c r="F124" s="5" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="G124" s="5" t="n">
+        <v>0.9835</v>
+      </c>
       <c r="H124" s="5" t="n">
-        <v>0.9897</v>
+        <v>0.9849</v>
       </c>
       <c r="I124" s="5" t="n">
-        <v>0.992</v>
+        <v>0.9865</v>
       </c>
       <c r="J124" s="5" t="n">
-        <v>0.9899</v>
+        <v>0.9848</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>0.9896</v>
+        <v>0.9855</v>
       </c>
       <c r="L124" s="5" t="inlineStr"/>
       <c r="M124" s="5" t="n">
-        <v>0.9931</v>
+        <v>0.9846</v>
       </c>
       <c r="N124" s="5" t="inlineStr"/>
       <c r="O124" s="5" t="n">
@@ -17525,7 +17529,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B125" s="5" t="n">
@@ -17571,7 +17575,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B126" s="5" t="n">
@@ -17617,42 +17621,30 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="n">
-        <v>0.9856</v>
-      </c>
-      <c r="C127" s="5" t="n">
-        <v>0.9829</v>
-      </c>
-      <c r="D127" s="5" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="E127" s="5" t="n">
-        <v>0.9828</v>
-      </c>
-      <c r="F127" s="5" t="n">
-        <v>0.9836</v>
-      </c>
-      <c r="G127" s="5" t="n">
-        <v>0.9835</v>
-      </c>
+          <t>HEZ1</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr"/>
+      <c r="C127" s="5" t="inlineStr"/>
+      <c r="D127" s="5" t="inlineStr"/>
+      <c r="E127" s="5" t="inlineStr"/>
+      <c r="F127" s="5" t="inlineStr"/>
+      <c r="G127" s="5" t="inlineStr"/>
       <c r="H127" s="5" t="n">
-        <v>0.9849</v>
+        <v>0.9897</v>
       </c>
       <c r="I127" s="5" t="n">
-        <v>0.9865</v>
+        <v>0.992</v>
       </c>
       <c r="J127" s="5" t="n">
-        <v>0.9848</v>
+        <v>0.9899</v>
       </c>
       <c r="K127" s="5" t="n">
-        <v>0.9855</v>
+        <v>0.9896</v>
       </c>
       <c r="L127" s="5" t="inlineStr"/>
       <c r="M127" s="5" t="n">
-        <v>0.9846</v>
+        <v>0.9931</v>
       </c>
       <c r="N127" s="5" t="inlineStr"/>
       <c r="O127" s="5" t="n">
@@ -17915,7 +17907,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B134" s="5" t="n">
@@ -17961,7 +17953,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B135" s="5" t="n">
@@ -18007,7 +17999,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B136" s="5" t="n">
@@ -18053,7 +18045,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B137" s="5" t="n">
@@ -18099,7 +18091,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B138" s="5" t="n">
@@ -18321,7 +18313,7 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>JNDABNE1</t>
+          <t>BROWNMT</t>
         </is>
       </c>
       <c r="B144" s="5" t="n">
@@ -18367,7 +18359,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>BROWNMT</t>
+          <t>JNDABNE1</t>
         </is>
       </c>
       <c r="B145" s="5" t="n">
@@ -18505,17 +18497,33 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>SHOAL1</t>
-        </is>
-      </c>
-      <c r="B148" s="5" t="inlineStr"/>
-      <c r="C148" s="5" t="inlineStr"/>
-      <c r="D148" s="5" t="inlineStr"/>
-      <c r="E148" s="5" t="inlineStr"/>
-      <c r="F148" s="5" t="inlineStr"/>
-      <c r="G148" s="5" t="inlineStr"/>
-      <c r="H148" s="5" t="inlineStr"/>
-      <c r="I148" s="5" t="inlineStr"/>
+          <t>WESTILL1</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="C148" s="5" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="D148" s="5" t="n">
+        <v>1.0023</v>
+      </c>
+      <c r="E148" s="5" t="n">
+        <v>1.0037</v>
+      </c>
+      <c r="F148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="G148" s="5" t="n">
+        <v>0.9967</v>
+      </c>
+      <c r="H148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="I148" s="5" t="n">
+        <v>0.9933999999999999</v>
+      </c>
       <c r="J148" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -18535,33 +18543,17 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>WESTILL1</t>
-        </is>
-      </c>
-      <c r="B149" s="5" t="n">
-        <v>0.9916</v>
-      </c>
-      <c r="C149" s="5" t="n">
-        <v>0.9986</v>
-      </c>
-      <c r="D149" s="5" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="E149" s="5" t="n">
-        <v>1.0037</v>
-      </c>
-      <c r="F149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="G149" s="5" t="n">
-        <v>0.9967</v>
-      </c>
-      <c r="H149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="I149" s="5" t="n">
-        <v>0.9933999999999999</v>
-      </c>
+          <t>SHOAL1</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr"/>
+      <c r="C149" s="5" t="inlineStr"/>
+      <c r="D149" s="5" t="inlineStr"/>
+      <c r="E149" s="5" t="inlineStr"/>
+      <c r="F149" s="5" t="inlineStr"/>
+      <c r="G149" s="5" t="inlineStr"/>
+      <c r="H149" s="5" t="inlineStr"/>
+      <c r="I149" s="5" t="inlineStr"/>
       <c r="J149" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -18707,7 +18699,7 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B153" s="5" t="n">
@@ -18753,7 +18745,7 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B154" s="5" t="n">
@@ -19259,7 +19251,7 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>SMTHBES1</t>
+          <t>WALGRV1</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr"/>
@@ -19271,25 +19263,29 @@
       <c r="H165" s="5" t="inlineStr"/>
       <c r="I165" s="5" t="inlineStr"/>
       <c r="J165" s="5" t="inlineStr"/>
-      <c r="K165" s="5" t="inlineStr"/>
-      <c r="L165" s="5" t="inlineStr"/>
+      <c r="K165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="L165" s="5" t="n">
+        <v>1.0009</v>
+      </c>
       <c r="M165" s="5" t="n">
-        <v>1.0016</v>
+        <v>1.0018</v>
       </c>
       <c r="N165" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0015</v>
       </c>
       <c r="O165" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="P165" s="5" t="n">
-        <v>1.0019</v>
+        <v>1.0017</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>WALGRV1</t>
+          <t>SMTHBES1</t>
         </is>
       </c>
       <c r="B166" s="5" t="inlineStr"/>
@@ -19301,23 +19297,19 @@
       <c r="H166" s="5" t="inlineStr"/>
       <c r="I166" s="5" t="inlineStr"/>
       <c r="J166" s="5" t="inlineStr"/>
-      <c r="K166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="L166" s="5" t="n">
-        <v>1.0009</v>
-      </c>
+      <c r="K166" s="5" t="inlineStr"/>
+      <c r="L166" s="5" t="inlineStr"/>
       <c r="M166" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0016</v>
       </c>
       <c r="N166" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0017</v>
       </c>
       <c r="O166" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="P166" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0019</v>
       </c>
     </row>
     <row r="167">
@@ -19369,7 +19361,7 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B168" s="5" t="n">
@@ -19415,7 +19407,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B169" s="5" t="n">
@@ -19537,7 +19529,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B172" s="5" t="n">
@@ -19583,7 +19575,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B173" s="5" t="n">
@@ -19629,7 +19621,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B174" s="5" t="n">
@@ -19675,7 +19667,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B175" s="5" t="n">
@@ -19721,7 +19713,7 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B176" s="5" t="n">
@@ -19767,7 +19759,7 @@
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B177" s="5" t="n">
@@ -19955,29 +19947,27 @@
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
-        </is>
-      </c>
-      <c r="B183" s="5" t="n">
-        <v>0.9916</v>
-      </c>
+          <t>AGLSITA1</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr"/>
       <c r="C183" s="5" t="n">
-        <v>0.9986</v>
+        <v>1.0019</v>
       </c>
       <c r="D183" s="5" t="n">
-        <v>1.0023</v>
+        <v>1.0022</v>
       </c>
       <c r="E183" s="5" t="n">
-        <v>1.0037</v>
+        <v>1.0024</v>
       </c>
       <c r="F183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0009</v>
       </c>
       <c r="G183" s="5" t="n">
-        <v>0.9967</v>
+        <v>1.0012</v>
       </c>
       <c r="H183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0015</v>
       </c>
       <c r="I183" s="5" t="inlineStr"/>
       <c r="J183" s="5" t="inlineStr"/>
@@ -19991,29 +19981,29 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>AGLNOW1</t>
         </is>
       </c>
       <c r="B184" s="5" t="n">
-        <v>0.9926</v>
+        <v>0.9916</v>
       </c>
       <c r="C184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9986</v>
       </c>
       <c r="D184" s="5" t="n">
-        <v>0.9892</v>
+        <v>1.0023</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>0.9901</v>
+        <v>1.0037</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9929</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9967</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>0.9917</v>
+        <v>0.9929</v>
       </c>
       <c r="I184" s="5" t="inlineStr"/>
       <c r="J184" s="5" t="inlineStr"/>
@@ -20027,29 +20017,29 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B185" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="C185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="D185" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="I185" s="5" t="inlineStr"/>
       <c r="J185" s="5" t="inlineStr"/>
@@ -20063,29 +20053,29 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B186" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9676</v>
       </c>
       <c r="C186" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9593</v>
       </c>
       <c r="D186" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9509</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9537</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9593</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9631</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9628</v>
       </c>
       <c r="I186" s="5" t="inlineStr"/>
       <c r="J186" s="5" t="inlineStr"/>
@@ -20135,29 +20125,29 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B188" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9926</v>
       </c>
       <c r="C188" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9907</v>
       </c>
       <c r="D188" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9892</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9901</v>
       </c>
       <c r="F188" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="G188" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9907</v>
       </c>
       <c r="H188" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9917</v>
       </c>
       <c r="I188" s="5" t="inlineStr"/>
       <c r="J188" s="5" t="inlineStr"/>
@@ -20171,27 +20161,29 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>AGLSITA1</t>
-        </is>
-      </c>
-      <c r="B189" s="5" t="inlineStr"/>
+          <t>WOYWOY1</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="n">
+        <v>1.0017</v>
+      </c>
       <c r="C189" s="5" t="n">
+        <v>1.0015</v>
+      </c>
+      <c r="D189" s="5" t="n">
+        <v>1.0008</v>
+      </c>
+      <c r="E189" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="F189" s="5" t="n">
+        <v>1.0036</v>
+      </c>
+      <c r="G189" s="5" t="n">
         <v>1.0019</v>
       </c>
-      <c r="D189" s="5" t="n">
-        <v>1.0022</v>
-      </c>
-      <c r="E189" s="5" t="n">
-        <v>1.0024</v>
-      </c>
-      <c r="F189" s="5" t="n">
-        <v>1.0009</v>
-      </c>
-      <c r="G189" s="5" t="n">
-        <v>1.0012</v>
-      </c>
       <c r="H189" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0037</v>
       </c>
       <c r="I189" s="5" t="inlineStr"/>
       <c r="J189" s="5" t="inlineStr"/>
@@ -20205,7 +20197,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>LD04</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B190" s="5" t="n">
@@ -20243,7 +20235,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD04</t>
         </is>
       </c>
       <c r="B191" s="5" t="n">
@@ -20281,7 +20273,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B192" s="5" t="n">
@@ -20319,7 +20311,7 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>WALGRVG1</t>
+          <t>QBYNBG1</t>
         </is>
       </c>
       <c r="B193" s="5" t="inlineStr"/>
@@ -20328,17 +20320,15 @@
       <c r="E193" s="5" t="inlineStr"/>
       <c r="F193" s="5" t="inlineStr"/>
       <c r="G193" s="5" t="inlineStr"/>
-      <c r="H193" s="5" t="n">
-        <v>1.0011</v>
-      </c>
+      <c r="H193" s="5" t="inlineStr"/>
       <c r="I193" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9752</v>
       </c>
       <c r="J193" s="5" t="n">
-        <v>1.001</v>
+        <v>0.979</v>
       </c>
       <c r="K193" s="5" t="n">
-        <v>1.001</v>
+        <v>0.9571</v>
       </c>
       <c r="L193" s="5" t="inlineStr"/>
       <c r="M193" s="5" t="inlineStr"/>
@@ -20349,7 +20339,7 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>DPNTBG1</t>
+          <t>BHBG1</t>
         </is>
       </c>
       <c r="B194" s="5" t="inlineStr"/>
@@ -20359,14 +20349,12 @@
       <c r="F194" s="5" t="inlineStr"/>
       <c r="G194" s="5" t="inlineStr"/>
       <c r="H194" s="5" t="inlineStr"/>
-      <c r="I194" s="5" t="n">
-        <v>0.9402</v>
-      </c>
+      <c r="I194" s="5" t="inlineStr"/>
       <c r="J194" s="5" t="n">
-        <v>0.9089</v>
+        <v>0.8671</v>
       </c>
       <c r="K194" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.8423</v>
       </c>
       <c r="L194" s="5" t="inlineStr"/>
       <c r="M194" s="5" t="inlineStr"/>
@@ -20377,7 +20365,7 @@
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>MLLFGEF1</t>
+          <t>CAPBES1G</t>
         </is>
       </c>
       <c r="B195" s="5" t="inlineStr"/>
@@ -20386,17 +20374,13 @@
       <c r="E195" s="5" t="inlineStr"/>
       <c r="F195" s="5" t="inlineStr"/>
       <c r="G195" s="5" t="inlineStr"/>
-      <c r="H195" s="5" t="n">
-        <v>0.9683</v>
-      </c>
-      <c r="I195" s="5" t="n">
-        <v>0.9687</v>
-      </c>
+      <c r="H195" s="5" t="inlineStr"/>
+      <c r="I195" s="5" t="inlineStr"/>
       <c r="J195" s="5" t="n">
-        <v>0.9663</v>
+        <v>0.9704</v>
       </c>
       <c r="K195" s="5" t="n">
-        <v>0.9567</v>
+        <v>0.9337</v>
       </c>
       <c r="L195" s="5" t="inlineStr"/>
       <c r="M195" s="5" t="inlineStr"/>
@@ -20407,7 +20391,7 @@
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
         <is>
-          <t>BHBG1</t>
+          <t>WALGRVG1</t>
         </is>
       </c>
       <c r="B196" s="5" t="inlineStr"/>
@@ -20416,13 +20400,17 @@
       <c r="E196" s="5" t="inlineStr"/>
       <c r="F196" s="5" t="inlineStr"/>
       <c r="G196" s="5" t="inlineStr"/>
-      <c r="H196" s="5" t="inlineStr"/>
-      <c r="I196" s="5" t="inlineStr"/>
+      <c r="H196" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="I196" s="5" t="n">
+        <v>1.001</v>
+      </c>
       <c r="J196" s="5" t="n">
-        <v>0.8671</v>
+        <v>1.001</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>0.8423</v>
+        <v>1.001</v>
       </c>
       <c r="L196" s="5" t="inlineStr"/>
       <c r="M196" s="5" t="inlineStr"/>
@@ -20433,7 +20421,7 @@
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
         <is>
-          <t>RESS1G</t>
+          <t>DPNTBG1</t>
         </is>
       </c>
       <c r="B197" s="5" t="inlineStr"/>
@@ -20444,13 +20432,13 @@
       <c r="G197" s="5" t="inlineStr"/>
       <c r="H197" s="5" t="inlineStr"/>
       <c r="I197" s="5" t="n">
-        <v>0.9286</v>
+        <v>0.9402</v>
       </c>
       <c r="J197" s="5" t="n">
         <v>0.9089</v>
       </c>
       <c r="K197" s="5" t="n">
-        <v>0.8702</v>
+        <v>0.9048</v>
       </c>
       <c r="L197" s="5" t="inlineStr"/>
       <c r="M197" s="5" t="inlineStr"/>
@@ -20461,7 +20449,7 @@
     <row r="198">
       <c r="A198" s="3" t="inlineStr">
         <is>
-          <t>RIVNBG2</t>
+          <t>MLLFGEF1</t>
         </is>
       </c>
       <c r="B198" s="5" t="inlineStr"/>
@@ -20470,15 +20458,17 @@
       <c r="E198" s="5" t="inlineStr"/>
       <c r="F198" s="5" t="inlineStr"/>
       <c r="G198" s="5" t="inlineStr"/>
-      <c r="H198" s="5" t="inlineStr"/>
+      <c r="H198" s="5" t="n">
+        <v>0.9683</v>
+      </c>
       <c r="I198" s="5" t="n">
-        <v>0.9058</v>
+        <v>0.9687</v>
       </c>
       <c r="J198" s="5" t="n">
-        <v>0.9106</v>
+        <v>0.9663</v>
       </c>
       <c r="K198" s="5" t="n">
-        <v>0.9048</v>
+        <v>0.9567</v>
       </c>
       <c r="L198" s="5" t="inlineStr"/>
       <c r="M198" s="5" t="inlineStr"/>
@@ -20489,7 +20479,7 @@
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
         <is>
-          <t>QBYNBG1</t>
+          <t>RESS1G</t>
         </is>
       </c>
       <c r="B199" s="5" t="inlineStr"/>
@@ -20500,13 +20490,13 @@
       <c r="G199" s="5" t="inlineStr"/>
       <c r="H199" s="5" t="inlineStr"/>
       <c r="I199" s="5" t="n">
-        <v>0.9752</v>
+        <v>0.9286</v>
       </c>
       <c r="J199" s="5" t="n">
-        <v>0.979</v>
+        <v>0.9089</v>
       </c>
       <c r="K199" s="5" t="n">
-        <v>0.9571</v>
+        <v>0.8702</v>
       </c>
       <c r="L199" s="5" t="inlineStr"/>
       <c r="M199" s="5" t="inlineStr"/>
@@ -20517,7 +20507,7 @@
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
         <is>
-          <t>CAPBES1G</t>
+          <t>RIVNBG2</t>
         </is>
       </c>
       <c r="B200" s="5" t="inlineStr"/>
@@ -20527,12 +20517,14 @@
       <c r="F200" s="5" t="inlineStr"/>
       <c r="G200" s="5" t="inlineStr"/>
       <c r="H200" s="5" t="inlineStr"/>
-      <c r="I200" s="5" t="inlineStr"/>
+      <c r="I200" s="5" t="n">
+        <v>0.9058</v>
+      </c>
       <c r="J200" s="5" t="n">
-        <v>0.9704</v>
+        <v>0.9106</v>
       </c>
       <c r="K200" s="5" t="n">
-        <v>0.9337</v>
+        <v>0.9048</v>
       </c>
       <c r="L200" s="5" t="inlineStr"/>
       <c r="M200" s="5" t="inlineStr"/>
@@ -21095,12 +21087,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>Junee Solar Farm</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -21124,12 +21116,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Sebastopol Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -21153,12 +21145,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Junee Solar Farm</t>
+          <t>Sebastopol Solar Farm</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -21632,7 +21624,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -21661,7 +21653,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -21724,13 +21716,11 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Williamsdale BESS</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
+          <t>WILLBESS</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v/>
       </c>
       <c r="D36" s="5" t="n">
         <v>0.9906</v>
@@ -21922,7 +21912,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -21951,7 +21941,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -21980,7 +21970,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update MLF data 2026-10-06 (audit close-out: unit types, battery lineage, retired units, DUALLOC capacities)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_mlf.xlsx
+++ b/outputs/NSW_mlf.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W201"/>
+  <dimension ref="A1:W194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -725,25 +725,27 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>White Rock Solar Farm</t>
+          <t>White Rock Wind Farm</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>22</v>
+        <v>175</v>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="H4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -786,27 +788,25 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>White Rock Wind Farm</t>
+          <t>White Rock Solar Farm</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>175</v>
+        <v>22</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -1748,12 +1748,12 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>West Wyalong Solar Farm</t>
+          <t>Junee Solar Farm</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1762,15 +1762,19 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>105</v>
+        <v>36</v>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr"/>
       <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr"/>
-      <c r="K21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="n">
+        <v>0.9645</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>0.8799</v>
+      </c>
       <c r="L21" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -1801,12 +1805,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Junee Solar Farm</t>
+          <t>Sebastopol Solar Farm</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1815,16 +1819,14 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>36</v>
+        <v>110</v>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
       <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr"/>
       <c r="H22" s="5" t="inlineStr"/>
       <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="n">
-        <v>0.9645</v>
-      </c>
+      <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="5" t="n">
         <v>0.8799</v>
       </c>
@@ -1858,12 +1860,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>West Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1872,7 +1874,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1911,12 +1913,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Sebastopol Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1925,7 +1927,7 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>110</v>
+        <v>62</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
@@ -1933,9 +1935,7 @@
       <c r="H24" s="5" t="inlineStr"/>
       <c r="I24" s="5" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr"/>
-      <c r="K24" s="5" t="n">
-        <v>0.8799</v>
-      </c>
+      <c r="K24" s="5" t="inlineStr"/>
       <c r="L24" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -2113,7 +2113,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -2166,7 +2166,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -2219,12 +2219,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>MULWASF1</t>
+          <t>CRWASF1</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Mulwala Solar Farm</t>
+          <t>Corowa Solar Farm</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2233,21 +2233,31 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr"/>
       <c r="H30" s="5" t="inlineStr"/>
       <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="inlineStr"/>
-      <c r="K30" s="5" t="inlineStr"/>
-      <c r="L30" s="5" t="inlineStr"/>
-      <c r="M30" s="5" t="inlineStr"/>
-      <c r="N30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="n">
+        <v>0.9497</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="M30" s="5" t="n">
+        <v>0.9365</v>
+      </c>
+      <c r="N30" s="5" t="n">
+        <v>0.8979</v>
+      </c>
       <c r="O30" s="5" t="inlineStr"/>
       <c r="P30" s="5" t="n">
-        <v>0.9345</v>
+        <v>0.9355</v>
       </c>
       <c r="Q30" s="5" t="inlineStr"/>
       <c r="R30" s="5" t="n">
@@ -2255,10 +2265,10 @@
       </c>
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="n">
-        <v>-0.0433</v>
+        <v>-0.0443</v>
       </c>
       <c r="U30" s="6" t="n">
-        <v>-4.63</v>
+        <v>-4.74</v>
       </c>
       <c r="V30" s="5" t="inlineStr"/>
       <c r="W30" s="6" t="inlineStr"/>
@@ -2266,12 +2276,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>CRWASF1</t>
+          <t>MULWASF1</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Corowa Solar Farm</t>
+          <t>Mulwala Solar Farm</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2280,31 +2290,21 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr"/>
       <c r="H31" s="5" t="inlineStr"/>
       <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="n">
-        <v>0.9497</v>
-      </c>
-      <c r="K31" s="5" t="n">
-        <v>0.8813</v>
-      </c>
-      <c r="L31" s="5" t="n">
-        <v>0.9242</v>
-      </c>
-      <c r="M31" s="5" t="n">
-        <v>0.9365</v>
-      </c>
-      <c r="N31" s="5" t="n">
-        <v>0.8979</v>
-      </c>
+      <c r="J31" s="5" t="inlineStr"/>
+      <c r="K31" s="5" t="inlineStr"/>
+      <c r="L31" s="5" t="inlineStr"/>
+      <c r="M31" s="5" t="inlineStr"/>
+      <c r="N31" s="5" t="inlineStr"/>
       <c r="O31" s="5" t="inlineStr"/>
       <c r="P31" s="5" t="n">
-        <v>0.9355</v>
+        <v>0.9345</v>
       </c>
       <c r="Q31" s="5" t="inlineStr"/>
       <c r="R31" s="5" t="n">
@@ -2312,10 +2312,10 @@
       </c>
       <c r="S31" s="5" t="inlineStr"/>
       <c r="T31" s="5" t="n">
-        <v>-0.0443</v>
+        <v>-0.0433</v>
       </c>
       <c r="U31" s="6" t="n">
-        <v>-4.74</v>
+        <v>-4.63</v>
       </c>
       <c r="V31" s="5" t="inlineStr"/>
       <c r="W31" s="6" t="inlineStr"/>
@@ -2781,7 +2781,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>NESBESS2</t>
+          <t>NESBESS1</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NESBESS1</t>
+          <t>NESBESS2</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -3013,7 +3013,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -3080,7 +3080,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -3147,7 +3147,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -3214,7 +3214,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -3399,12 +3399,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wellington Solar Farm </t>
+          <t>Nevertire Solar Farm</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3413,13 +3413,15 @@
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>216</v>
+        <v>132</v>
       </c>
       <c r="E50" s="5" t="inlineStr"/>
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr"/>
       <c r="H50" s="5" t="inlineStr"/>
-      <c r="I50" s="5" t="inlineStr"/>
+      <c r="I50" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="J50" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -3456,12 +3458,12 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Narromine Solar Farm</t>
+          <t>South Keswick Solar Farm</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3470,7 +3472,7 @@
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
       <c r="F51" s="5" t="inlineStr"/>
@@ -3519,12 +3521,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>NASF1</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Nevertire Solar Farm</t>
+          <t>Narromine Solar Farm</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3533,12 +3535,16 @@
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>132</v>
+        <v>10</v>
       </c>
       <c r="E52" s="5" t="inlineStr"/>
       <c r="F52" s="5" t="inlineStr"/>
-      <c r="G52" s="5" t="inlineStr"/>
-      <c r="H52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>0.9708</v>
+      </c>
       <c r="I52" s="5" t="n">
         <v>0.9582000000000001</v>
       </c>
@@ -3645,12 +3651,12 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>South Keswick Solar Farm</t>
+          <t xml:space="preserve">Wellington Solar Farm </t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -3659,19 +3665,13 @@
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>15</v>
+        <v>216</v>
       </c>
       <c r="E54" s="5" t="inlineStr"/>
       <c r="F54" s="5" t="inlineStr"/>
-      <c r="G54" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="H54" s="5" t="n">
-        <v>0.9708</v>
-      </c>
-      <c r="I54" s="5" t="n">
-        <v>0.9582000000000001</v>
-      </c>
+      <c r="G54" s="5" t="inlineStr"/>
+      <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="5" t="inlineStr"/>
       <c r="J54" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -3940,12 +3940,12 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>STUBSF2</t>
+          <t>STUBSF1</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Stubbo Solar Farm 2</t>
+          <t>Stubbo Solar Farm 1</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3954,7 +3954,7 @@
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="E59" s="5" t="inlineStr"/>
       <c r="F59" s="5" t="inlineStr"/>
@@ -3989,12 +3989,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>STUBSF1</t>
+          <t>STUBSF2</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Stubbo Solar Farm 1</t>
+          <t>Stubbo Solar Farm 2</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -4003,7 +4003,7 @@
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E60" s="5" t="inlineStr"/>
       <c r="F60" s="5" t="inlineStr"/>
@@ -4491,12 +4491,12 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Cullerin Range Wind Farm</t>
+          <t>Gunning Wind Farm</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>30</v>
+        <v>46.5</v>
       </c>
       <c r="E68" s="5" t="n">
         <v>0.9742</v>
@@ -4558,12 +4558,12 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Gunning Wind Farm</t>
+          <t>Cullerin Range Wind Farm</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -4572,7 +4572,7 @@
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>46.5</v>
+        <v>30</v>
       </c>
       <c r="E69" s="5" t="n">
         <v>0.9742</v>
@@ -5238,7 +5238,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>BW04</t>
+          <t>BW03</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>BW03</t>
+          <t>BW04</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -5372,7 +5372,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>BW02</t>
+          <t>BW01</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -5439,7 +5439,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>BW01</t>
+          <t>BW02</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -5506,26 +5506,30 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF2</t>
+          <t>GULLRSF1</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Gullen Range Wind Farm</t>
+          <t>Gullen Range Solar Farm</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D85" s="4" t="n">
-        <v>110</v>
+        <v>10</v>
       </c>
       <c r="E85" s="5" t="inlineStr"/>
       <c r="F85" s="5" t="inlineStr"/>
-      <c r="G85" s="5" t="inlineStr"/>
-      <c r="H85" s="5" t="inlineStr"/>
+      <c r="G85" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="H85" s="5" t="n">
+        <v>0.9959</v>
+      </c>
       <c r="I85" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -5565,7 +5569,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF1</t>
+          <t>GULLRWF2</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -5579,20 +5583,12 @@
         </is>
       </c>
       <c r="D86" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="E86" s="5" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="F86" s="5" t="n">
-        <v>0.9909</v>
-      </c>
-      <c r="G86" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="H86" s="5" t="n">
-        <v>0.9959</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="E86" s="5" t="inlineStr"/>
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="5" t="inlineStr"/>
+      <c r="H86" s="5" t="inlineStr"/>
       <c r="I86" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -5632,24 +5628,28 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>GULLRSF1</t>
+          <t>GULLRWF1</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Gullen Range Solar Farm</t>
+          <t>Gullen Range Wind Farm</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D87" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E87" s="5" t="inlineStr"/>
-      <c r="F87" s="5" t="inlineStr"/>
+        <v>165</v>
+      </c>
+      <c r="E87" s="5" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="F87" s="5" t="n">
+        <v>0.9909</v>
+      </c>
       <c r="G87" s="5" t="n">
         <v>1.001</v>
       </c>
@@ -6120,12 +6120,12 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Capital Wind Farm</t>
+          <t>Woodlawn Wind Farm</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -6134,7 +6134,7 @@
         </is>
       </c>
       <c r="D95" s="4" t="n">
-        <v>140</v>
+        <v>48.3</v>
       </c>
       <c r="E95" s="5" t="n">
         <v>0.9748</v>
@@ -6187,12 +6187,12 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Wind Farm</t>
+          <t>Capital Wind Farm</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -6201,7 +6201,7 @@
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>48.3</v>
+        <v>140</v>
       </c>
       <c r="E96" s="5" t="n">
         <v>0.9748</v>
@@ -6520,12 +6520,12 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MPNL1</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>MT PIPER POWER STATION</t>
+          <t>Mt Piper Power Station</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -6534,7 +6534,7 @@
         </is>
       </c>
       <c r="D101" s="4" t="n">
-        <v>25</v>
+        <v>700</v>
       </c>
       <c r="E101" s="5" t="n">
         <v>0.9744</v>
@@ -6654,12 +6654,12 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MPNL1</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Mt Piper Power Station</t>
+          <t>MT PIPER POWER STATION</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -6668,7 +6668,7 @@
         </is>
       </c>
       <c r="D103" s="4" t="n">
-        <v>700</v>
+        <v>25</v>
       </c>
       <c r="E103" s="5" t="n">
         <v>0.9744</v>
@@ -6878,8 +6878,12 @@
       <c r="I106" s="5" t="inlineStr"/>
       <c r="J106" s="5" t="inlineStr"/>
       <c r="K106" s="5" t="inlineStr"/>
-      <c r="L106" s="5" t="inlineStr"/>
-      <c r="M106" s="5" t="inlineStr"/>
+      <c r="L106" s="5" t="n">
+        <v>0.9058</v>
+      </c>
+      <c r="M106" s="5" t="n">
+        <v>0.9106</v>
+      </c>
       <c r="N106" s="5" t="n">
         <v>0.9048</v>
       </c>
@@ -6914,7 +6918,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -6922,7 +6926,7 @@
           <t>TUMUT2</t>
         </is>
       </c>
-      <c r="C107" s="3" t="inlineStr"/>
+      <c r="C107" s="3" t="n"/>
       <c r="D107" s="4" t="n">
         <v>72</v>
       </c>
@@ -6977,17 +6981,17 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
-        </is>
-      </c>
-      <c r="C108" s="3" t="inlineStr"/>
+          <t>TUMUT1</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="n"/>
       <c r="D108" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E108" s="5" t="n">
         <v>0.9768</v>
@@ -7040,17 +7044,17 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-2</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
-        </is>
-      </c>
-      <c r="C109" s="3" t="inlineStr"/>
+          <t>TUMUT1</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="n"/>
       <c r="D109" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E109" s="5" t="n">
         <v>0.9768</v>
@@ -7103,17 +7107,17 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
-        </is>
-      </c>
-      <c r="C110" s="3" t="inlineStr"/>
+          <t>TUMUT1</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="n"/>
       <c r="D110" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E110" s="5" t="n">
         <v>0.9768</v>
@@ -7166,17 +7170,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT2-2</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
-        </is>
-      </c>
-      <c r="C111" s="3" t="inlineStr"/>
+          <t>TUMUT2</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="n"/>
       <c r="D111" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E111" s="5" t="n">
         <v>0.9768</v>
@@ -7229,17 +7233,17 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
-        </is>
-      </c>
-      <c r="C112" s="3" t="inlineStr"/>
+          <t>TUMUT2</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="n"/>
       <c r="D112" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E112" s="5" t="n">
         <v>0.9768</v>
@@ -7292,17 +7296,17 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="inlineStr"/>
+          <t>TUMUT2</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="n"/>
       <c r="D113" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E113" s="5" t="n">
         <v>0.9768</v>
@@ -7363,7 +7367,7 @@
           <t>TUMUT1</t>
         </is>
       </c>
-      <c r="C114" s="3" t="inlineStr"/>
+      <c r="C114" s="3" t="n"/>
       <c r="D114" s="4" t="n">
         <v>82</v>
       </c>
@@ -7441,8 +7445,12 @@
       <c r="I115" s="5" t="inlineStr"/>
       <c r="J115" s="5" t="inlineStr"/>
       <c r="K115" s="5" t="inlineStr"/>
-      <c r="L115" s="5" t="inlineStr"/>
-      <c r="M115" s="5" t="inlineStr"/>
+      <c r="L115" s="5" t="n">
+        <v>0.9402</v>
+      </c>
+      <c r="M115" s="5" t="n">
+        <v>0.9089</v>
+      </c>
       <c r="N115" s="5" t="n">
         <v>0.9048</v>
       </c>
@@ -7544,7 +7552,9 @@
       <c r="J117" s="5" t="inlineStr"/>
       <c r="K117" s="5" t="inlineStr"/>
       <c r="L117" s="5" t="inlineStr"/>
-      <c r="M117" s="5" t="inlineStr"/>
+      <c r="M117" s="5" t="n">
+        <v>0.9704</v>
+      </c>
       <c r="N117" s="5" t="n">
         <v>0.9337</v>
       </c>
@@ -7705,7 +7715,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -7839,7 +7849,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -7930,7 +7940,9 @@
       <c r="J123" s="5" t="inlineStr"/>
       <c r="K123" s="5" t="inlineStr"/>
       <c r="L123" s="5" t="inlineStr"/>
-      <c r="M123" s="5" t="inlineStr"/>
+      <c r="M123" s="5" t="n">
+        <v>0.8671</v>
+      </c>
       <c r="N123" s="5" t="n">
         <v>0.8423</v>
       </c>
@@ -7965,12 +7977,12 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
+          <t>HEZ1</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>Eraring Power Station</t>
+          <t>Hunter Economic Zone</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -7979,41 +7991,29 @@
         </is>
       </c>
       <c r="D124" s="4" t="n">
-        <v>720</v>
-      </c>
-      <c r="E124" s="5" t="n">
-        <v>0.9856</v>
-      </c>
-      <c r="F124" s="5" t="n">
-        <v>0.9829</v>
-      </c>
-      <c r="G124" s="5" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="H124" s="5" t="n">
-        <v>0.9828</v>
-      </c>
-      <c r="I124" s="5" t="n">
-        <v>0.9836</v>
-      </c>
-      <c r="J124" s="5" t="n">
-        <v>0.9835</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="E124" s="5" t="inlineStr"/>
+      <c r="F124" s="5" t="inlineStr"/>
+      <c r="G124" s="5" t="inlineStr"/>
+      <c r="H124" s="5" t="inlineStr"/>
+      <c r="I124" s="5" t="inlineStr"/>
+      <c r="J124" s="5" t="inlineStr"/>
       <c r="K124" s="5" t="n">
-        <v>0.9849</v>
+        <v>0.9897</v>
       </c>
       <c r="L124" s="5" t="n">
-        <v>0.9865</v>
+        <v>0.992</v>
       </c>
       <c r="M124" s="5" t="n">
-        <v>0.9848</v>
+        <v>0.9899</v>
       </c>
       <c r="N124" s="5" t="n">
-        <v>0.9855</v>
+        <v>0.9896</v>
       </c>
       <c r="O124" s="5" t="inlineStr"/>
       <c r="P124" s="5" t="n">
-        <v>0.9846</v>
+        <v>0.9931</v>
       </c>
       <c r="Q124" s="5" t="inlineStr"/>
       <c r="R124" s="5" t="n">
@@ -8021,10 +8021,10 @@
       </c>
       <c r="S124" s="5" t="inlineStr"/>
       <c r="T124" s="5" t="n">
-        <v>-0.0015</v>
+        <v>-0.01</v>
       </c>
       <c r="U124" s="6" t="n">
-        <v>-0.15</v>
+        <v>-1.01</v>
       </c>
       <c r="V124" s="5" t="inlineStr"/>
       <c r="W124" s="6" t="inlineStr"/>
@@ -8032,7 +8032,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -8046,7 +8046,7 @@
         </is>
       </c>
       <c r="D125" s="4" t="n">
-        <v>720</v>
+        <v>41.5</v>
       </c>
       <c r="E125" s="5" t="n">
         <v>0.9856</v>
@@ -8099,7 +8099,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -8113,7 +8113,7 @@
         </is>
       </c>
       <c r="D126" s="4" t="n">
-        <v>41.5</v>
+        <v>720</v>
       </c>
       <c r="E126" s="5" t="n">
         <v>0.9856</v>
@@ -8166,12 +8166,12 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>HEZ1</t>
+          <t>ER01</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>Hunter Economic Zone</t>
+          <t>Eraring Power Station</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -8180,29 +8180,41 @@
         </is>
       </c>
       <c r="D127" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="E127" s="5" t="inlineStr"/>
-      <c r="F127" s="5" t="inlineStr"/>
-      <c r="G127" s="5" t="inlineStr"/>
-      <c r="H127" s="5" t="inlineStr"/>
-      <c r="I127" s="5" t="inlineStr"/>
-      <c r="J127" s="5" t="inlineStr"/>
+        <v>720</v>
+      </c>
+      <c r="E127" s="5" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="F127" s="5" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="G127" s="5" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="H127" s="5" t="n">
+        <v>0.9828</v>
+      </c>
+      <c r="I127" s="5" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="J127" s="5" t="n">
+        <v>0.9835</v>
+      </c>
       <c r="K127" s="5" t="n">
-        <v>0.9897</v>
+        <v>0.9849</v>
       </c>
       <c r="L127" s="5" t="n">
-        <v>0.992</v>
+        <v>0.9865</v>
       </c>
       <c r="M127" s="5" t="n">
-        <v>0.9899</v>
+        <v>0.9848</v>
       </c>
       <c r="N127" s="5" t="n">
-        <v>0.9896</v>
+        <v>0.9855</v>
       </c>
       <c r="O127" s="5" t="inlineStr"/>
       <c r="P127" s="5" t="n">
-        <v>0.9931</v>
+        <v>0.9846</v>
       </c>
       <c r="Q127" s="5" t="inlineStr"/>
       <c r="R127" s="5" t="n">
@@ -8210,10 +8222,10 @@
       </c>
       <c r="S127" s="5" t="inlineStr"/>
       <c r="T127" s="5" t="n">
-        <v>-0.01</v>
+        <v>-0.0015</v>
       </c>
       <c r="U127" s="6" t="n">
-        <v>-1.01</v>
+        <v>-0.15</v>
       </c>
       <c r="V127" s="5" t="inlineStr"/>
       <c r="W127" s="6" t="inlineStr"/>
@@ -8504,8 +8516,12 @@
       <c r="I132" s="5" t="inlineStr"/>
       <c r="J132" s="5" t="inlineStr"/>
       <c r="K132" s="5" t="inlineStr"/>
-      <c r="L132" s="5" t="inlineStr"/>
-      <c r="M132" s="5" t="inlineStr"/>
+      <c r="L132" s="5" t="n">
+        <v>0.9286</v>
+      </c>
+      <c r="M132" s="5" t="n">
+        <v>0.9089</v>
+      </c>
       <c r="N132" s="5" t="n">
         <v>0.8702</v>
       </c>
@@ -8607,7 +8623,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -8674,7 +8690,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -8741,7 +8757,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -8808,7 +8824,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -8875,7 +8891,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -9223,12 +9239,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>BROWNMT</t>
+          <t>JNDABNE1</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Brown Mountain Hydro Power Station</t>
+          <t>Jindabyne Small Hydro Power Station</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -9237,7 +9253,7 @@
         </is>
       </c>
       <c r="D144" s="4" t="n">
-        <v>5</v>
+        <v>1.1</v>
       </c>
       <c r="E144" s="5" t="n">
         <v>0.9762999999999999</v>
@@ -9290,12 +9306,12 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>JNDABNE1</t>
+          <t>BROWNMT</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Jindabyne Small Hydro Power Station</t>
+          <t>Brown Mountain Hydro Power Station</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -9304,7 +9320,7 @@
         </is>
       </c>
       <c r="D145" s="4" t="n">
-        <v>1.1</v>
+        <v>5</v>
       </c>
       <c r="E145" s="5" t="n">
         <v>0.9762999999999999</v>
@@ -9491,12 +9507,12 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>WESTILL1</t>
+          <t>SHOAL1</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>West Illawarra Leagues Club Plant</t>
+          <t>Shoalhaven Starches Cogeneration Plant</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -9505,32 +9521,16 @@
         </is>
       </c>
       <c r="D148" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E148" s="5" t="n">
-        <v>0.9916</v>
-      </c>
-      <c r="F148" s="5" t="n">
-        <v>0.9986</v>
-      </c>
-      <c r="G148" s="5" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="H148" s="5" t="n">
-        <v>1.0037</v>
-      </c>
-      <c r="I148" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="J148" s="5" t="n">
-        <v>0.9967</v>
-      </c>
-      <c r="K148" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="L148" s="5" t="n">
-        <v>0.9933999999999999</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E148" s="5" t="inlineStr"/>
+      <c r="F148" s="5" t="inlineStr"/>
+      <c r="G148" s="5" t="inlineStr"/>
+      <c r="H148" s="5" t="inlineStr"/>
+      <c r="I148" s="5" t="inlineStr"/>
+      <c r="J148" s="5" t="inlineStr"/>
+      <c r="K148" s="5" t="inlineStr"/>
+      <c r="L148" s="5" t="inlineStr"/>
       <c r="M148" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -9558,12 +9558,12 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>SHOAL1</t>
+          <t>WESTILL1</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Shoalhaven Starches Cogeneration Plant</t>
+          <t>West Illawarra Leagues Club Plant</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -9572,16 +9572,32 @@
         </is>
       </c>
       <c r="D149" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="E149" s="5" t="inlineStr"/>
-      <c r="F149" s="5" t="inlineStr"/>
-      <c r="G149" s="5" t="inlineStr"/>
-      <c r="H149" s="5" t="inlineStr"/>
-      <c r="I149" s="5" t="inlineStr"/>
-      <c r="J149" s="5" t="inlineStr"/>
-      <c r="K149" s="5" t="inlineStr"/>
-      <c r="L149" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E149" s="5" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="F149" s="5" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>1.0023</v>
+      </c>
+      <c r="H149" s="5" t="n">
+        <v>1.0037</v>
+      </c>
+      <c r="I149" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="J149" s="5" t="n">
+        <v>0.9967</v>
+      </c>
+      <c r="K149" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="L149" s="5" t="n">
+        <v>0.9933999999999999</v>
+      </c>
       <c r="M149" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -9766,8 +9782,12 @@
       <c r="I152" s="5" t="inlineStr"/>
       <c r="J152" s="5" t="inlineStr"/>
       <c r="K152" s="5" t="inlineStr"/>
-      <c r="L152" s="5" t="inlineStr"/>
-      <c r="M152" s="5" t="inlineStr"/>
+      <c r="L152" s="5" t="n">
+        <v>0.9752</v>
+      </c>
+      <c r="M152" s="5" t="n">
+        <v>0.979</v>
+      </c>
       <c r="N152" s="5" t="n">
         <v>0.9571</v>
       </c>
@@ -9802,12 +9822,12 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>Wyangala A Power Station</t>
+          <t>Wyangala B Power Station</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
@@ -9816,7 +9836,7 @@
         </is>
       </c>
       <c r="D153" s="4" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E153" s="5" t="n">
         <v>1.0099</v>
@@ -9869,12 +9889,12 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>Wyangala B Power Station</t>
+          <t>Wyangala A Power Station</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -9883,7 +9903,7 @@
         </is>
       </c>
       <c r="D154" s="4" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E154" s="5" t="n">
         <v>1.0099</v>
@@ -10279,7 +10299,7 @@
           <t>NSW1 Dummy Generator</t>
         </is>
       </c>
-      <c r="C160" s="3" t="inlineStr"/>
+      <c r="C160" s="3" t="n"/>
       <c r="D160" s="4" t="n">
         <v>3000</v>
       </c>
@@ -10602,12 +10622,12 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>WALGRV1</t>
+          <t>SMTHBES1</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Wallgrove BESS 1</t>
+          <t>Smithfield Battery Energy Storage System, Units 1 - 36</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -10616,7 +10636,7 @@
         </is>
       </c>
       <c r="D165" s="4" t="n">
-        <v>50</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="E165" s="5" t="inlineStr"/>
       <c r="F165" s="5" t="inlineStr"/>
@@ -10627,29 +10647,25 @@
       <c r="K165" s="5" t="inlineStr"/>
       <c r="L165" s="5" t="inlineStr"/>
       <c r="M165" s="5" t="inlineStr"/>
-      <c r="N165" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="O165" s="5" t="n">
-        <v>1.0009</v>
-      </c>
+      <c r="N165" s="5" t="inlineStr"/>
+      <c r="O165" s="5" t="inlineStr"/>
       <c r="P165" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0016</v>
       </c>
       <c r="Q165" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0017</v>
       </c>
       <c r="R165" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="S165" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0019</v>
       </c>
       <c r="T165" s="5" t="n">
-        <v>-0.0001</v>
+        <v>0.0001</v>
       </c>
       <c r="U165" s="6" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="V165" s="5" t="n">
         <v>0.0002</v>
@@ -10661,12 +10677,12 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>SMTHBES1</t>
+          <t>WALGRV1</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>Smithfield Battery Energy Storage System, Units 1 - 36</t>
+          <t>Wallgrove BESS 1</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -10675,7 +10691,7 @@
         </is>
       </c>
       <c r="D166" s="4" t="n">
-        <v>69.40000000000001</v>
+        <v>50</v>
       </c>
       <c r="E166" s="5" t="inlineStr"/>
       <c r="F166" s="5" t="inlineStr"/>
@@ -10683,28 +10699,38 @@
       <c r="H166" s="5" t="inlineStr"/>
       <c r="I166" s="5" t="inlineStr"/>
       <c r="J166" s="5" t="inlineStr"/>
-      <c r="K166" s="5" t="inlineStr"/>
-      <c r="L166" s="5" t="inlineStr"/>
-      <c r="M166" s="5" t="inlineStr"/>
-      <c r="N166" s="5" t="inlineStr"/>
-      <c r="O166" s="5" t="inlineStr"/>
+      <c r="K166" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="L166" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="M166" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="N166" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="O166" s="5" t="n">
+        <v>1.0009</v>
+      </c>
       <c r="P166" s="5" t="n">
-        <v>1.0016</v>
+        <v>1.0018</v>
       </c>
       <c r="Q166" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0015</v>
       </c>
       <c r="R166" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="S166" s="5" t="n">
-        <v>1.0019</v>
+        <v>1.0017</v>
       </c>
       <c r="T166" s="5" t="n">
-        <v>0.0001</v>
+        <v>-0.0001</v>
       </c>
       <c r="U166" s="6" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="V166" s="5" t="n">
         <v>0.0002</v>
@@ -10783,21 +10809,21 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Bioreactor Energy Generation Station</t>
+          <t>Taralga Wind Farm</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D168" s="4" t="n">
-        <v>7</v>
+        <v>106.8</v>
       </c>
       <c r="E168" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -10850,21 +10876,21 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>Taralga Wind Farm</t>
+          <t>Woodlawn Bioreactor Energy Generation Station</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D169" s="4" t="n">
-        <v>106.8</v>
+        <v>7</v>
       </c>
       <c r="E169" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -11035,7 +11061,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -11043,7 +11069,7 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C172" s="3" t="inlineStr"/>
+      <c r="C172" s="3" t="n"/>
       <c r="D172" s="4" t="n">
         <v>250</v>
       </c>
@@ -11098,7 +11124,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -11106,7 +11132,7 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C173" s="3" t="inlineStr"/>
+      <c r="C173" s="3" t="n"/>
       <c r="D173" s="4" t="n">
         <v>250</v>
       </c>
@@ -11161,7 +11187,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -11169,7 +11195,7 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C174" s="3" t="inlineStr"/>
+      <c r="C174" s="3" t="n"/>
       <c r="D174" s="4" t="n">
         <v>250</v>
       </c>
@@ -11224,7 +11250,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -11232,7 +11258,7 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C175" s="3" t="inlineStr"/>
+      <c r="C175" s="3" t="n"/>
       <c r="D175" s="4" t="n">
         <v>250</v>
       </c>
@@ -11287,7 +11313,7 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -11295,7 +11321,7 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C176" s="3" t="inlineStr"/>
+      <c r="C176" s="3" t="n"/>
       <c r="D176" s="4" t="n">
         <v>250</v>
       </c>
@@ -11350,7 +11376,7 @@
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -11358,7 +11384,7 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C177" s="3" t="inlineStr"/>
+      <c r="C177" s="3" t="n"/>
       <c r="D177" s="4" t="n">
         <v>250</v>
       </c>
@@ -11421,7 +11447,7 @@
           <t>Redbank Power Station</t>
         </is>
       </c>
-      <c r="C178" s="3" t="inlineStr"/>
+      <c r="C178" s="3" t="n"/>
       <c r="D178" s="4" t="n">
         <v>150</v>
       </c>
@@ -11507,7 +11533,7 @@
         </is>
       </c>
       <c r="D180" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E180" s="5" t="n">
         <v>1.0016</v>
@@ -11636,12 +11662,12 @@
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AGLSITA1</t>
+          <t>AGLNOW1</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>AGL KEMPS CREEK</t>
+          <t>West Nowra Landfill Gas Power Generation Facility</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
@@ -11652,24 +11678,26 @@
       <c r="D183" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E183" s="5" t="inlineStr"/>
+      <c r="E183" s="5" t="n">
+        <v>0.9916</v>
+      </c>
       <c r="F183" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9986</v>
       </c>
       <c r="G183" s="5" t="n">
-        <v>1.0022</v>
+        <v>1.0023</v>
       </c>
       <c r="H183" s="5" t="n">
-        <v>1.0024</v>
+        <v>1.0037</v>
       </c>
       <c r="I183" s="5" t="n">
-        <v>1.0009</v>
+        <v>0.9929</v>
       </c>
       <c r="J183" s="5" t="n">
-        <v>1.0012</v>
+        <v>0.9967</v>
       </c>
       <c r="K183" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9929</v>
       </c>
       <c r="L183" s="5" t="inlineStr"/>
       <c r="M183" s="5" t="inlineStr"/>
@@ -11687,12 +11715,12 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>West Nowra Landfill Gas Power Generation Facility</t>
+          <t>TERALBA POWER STATION</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
@@ -11701,28 +11729,28 @@
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>0.9916</v>
+        <v>0.9926</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9986</v>
+        <v>0.9907</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>1.0023</v>
+        <v>0.9892</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9901</v>
       </c>
       <c r="I184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="J184" s="5" t="n">
-        <v>0.9967</v>
+        <v>0.9907</v>
       </c>
       <c r="K184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9917</v>
       </c>
       <c r="L184" s="5" t="inlineStr"/>
       <c r="M184" s="5" t="inlineStr"/>
@@ -11740,42 +11768,42 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Kincumber Landfill Site</t>
+          <t>Liddell Power Station</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Fossil</t>
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9676</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9593</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9509</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9537</v>
       </c>
       <c r="I185" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9593</v>
       </c>
       <c r="J185" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9631</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9628</v>
       </c>
       <c r="L185" s="5" t="inlineStr"/>
       <c r="M185" s="5" t="inlineStr"/>
@@ -11793,42 +11821,42 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>Liddell Power Station</t>
+          <t>Kincumber Landfill Site</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Fossil</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D186" s="4" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="I186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="J186" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="K186" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="L186" s="5" t="inlineStr"/>
       <c r="M186" s="5" t="inlineStr"/>
@@ -11854,10 +11882,14 @@
           <t>Hunter Valley Gas Turbine</t>
         </is>
       </c>
-      <c r="C187" s="3" t="n">
-        <v/>
-      </c>
-      <c r="D187" s="3" t="inlineStr"/>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>Fossil</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>50</v>
+      </c>
       <c r="E187" s="5" t="n">
         <v>0.974</v>
       </c>
@@ -11895,12 +11927,12 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>WOYWOY1</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>TERALBA POWER STATION</t>
+          <t>Woy Woy Landfill Site</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -11909,28 +11941,28 @@
         </is>
       </c>
       <c r="D188" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>0.9926</v>
+        <v>1.0017</v>
       </c>
       <c r="F188" s="5" t="n">
-        <v>0.9907</v>
+        <v>1.0015</v>
       </c>
       <c r="G188" s="5" t="n">
-        <v>0.9892</v>
+        <v>1.0008</v>
       </c>
       <c r="H188" s="5" t="n">
-        <v>0.9901</v>
+        <v>1.0011</v>
       </c>
       <c r="I188" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>1.0036</v>
       </c>
       <c r="J188" s="5" t="n">
-        <v>0.9907</v>
+        <v>1.0019</v>
       </c>
       <c r="K188" s="5" t="n">
-        <v>0.9917</v>
+        <v>1.0037</v>
       </c>
       <c r="L188" s="5" t="inlineStr"/>
       <c r="M188" s="5" t="inlineStr"/>
@@ -11948,12 +11980,12 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
+          <t>AGLSITA1</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>Woy Woy Landfill Site</t>
+          <t>AGL KEMPS CREEK</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
@@ -11964,26 +11996,24 @@
       <c r="D189" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E189" s="5" t="n">
-        <v>1.0017</v>
-      </c>
+      <c r="E189" s="5" t="inlineStr"/>
       <c r="F189" s="5" t="n">
+        <v>1.0019</v>
+      </c>
+      <c r="G189" s="5" t="n">
+        <v>1.0022</v>
+      </c>
+      <c r="H189" s="5" t="n">
+        <v>1.0024</v>
+      </c>
+      <c r="I189" s="5" t="n">
+        <v>1.0009</v>
+      </c>
+      <c r="J189" s="5" t="n">
+        <v>1.0012</v>
+      </c>
+      <c r="K189" s="5" t="n">
         <v>1.0015</v>
-      </c>
-      <c r="G189" s="5" t="n">
-        <v>1.0008</v>
-      </c>
-      <c r="H189" s="5" t="n">
-        <v>1.0011</v>
-      </c>
-      <c r="I189" s="5" t="n">
-        <v>1.0036</v>
-      </c>
-      <c r="J189" s="5" t="n">
-        <v>1.0019</v>
-      </c>
-      <c r="K189" s="5" t="n">
-        <v>1.0037</v>
       </c>
       <c r="L189" s="5" t="inlineStr"/>
       <c r="M189" s="5" t="inlineStr"/>
@@ -12001,7 +12031,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD04</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -12056,7 +12086,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>LD04</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
@@ -12111,7 +12141,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -12166,21 +12196,21 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>QBYNBG1</t>
+          <t>MLLFGEF1</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>Queanbeyan BESS</t>
+          <t>Mugga Lane Landfill Gas To Energy Facility</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D193" s="4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E193" s="5" t="inlineStr"/>
       <c r="F193" s="5" t="inlineStr"/>
@@ -12188,15 +12218,17 @@
       <c r="H193" s="5" t="inlineStr"/>
       <c r="I193" s="5" t="inlineStr"/>
       <c r="J193" s="5" t="inlineStr"/>
-      <c r="K193" s="5" t="inlineStr"/>
+      <c r="K193" s="5" t="n">
+        <v>0.9683</v>
+      </c>
       <c r="L193" s="5" t="n">
-        <v>0.9752</v>
+        <v>0.9687</v>
       </c>
       <c r="M193" s="5" t="n">
-        <v>0.979</v>
+        <v>0.9663</v>
       </c>
       <c r="N193" s="5" t="n">
-        <v>0.9571</v>
+        <v>0.9567</v>
       </c>
       <c r="O193" s="5" t="inlineStr"/>
       <c r="P193" s="5" t="inlineStr"/>
@@ -12211,38 +12243,56 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>BHBG1</t>
+          <t>WESTCBT1</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>Broken Hill Battery Energy Storage System</t>
+          <t>Western Suburbs League Club (Campbelltown) Plant</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>Battery</t>
+          <t>Fossil</t>
         </is>
       </c>
       <c r="D194" s="4" t="n">
-        <v>66</v>
-      </c>
-      <c r="E194" s="5" t="inlineStr"/>
-      <c r="F194" s="5" t="inlineStr"/>
-      <c r="G194" s="5" t="inlineStr"/>
-      <c r="H194" s="5" t="inlineStr"/>
-      <c r="I194" s="5" t="inlineStr"/>
-      <c r="J194" s="5" t="inlineStr"/>
-      <c r="K194" s="5" t="inlineStr"/>
-      <c r="L194" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E194" s="5" t="n">
+        <v>0.9991</v>
+      </c>
+      <c r="F194" s="5" t="n">
+        <v>1.0005</v>
+      </c>
+      <c r="G194" s="5" t="n">
+        <v>1.0001</v>
+      </c>
+      <c r="H194" s="5" t="n">
+        <v>1.0006</v>
+      </c>
+      <c r="I194" s="5" t="n">
+        <v>0.9973</v>
+      </c>
+      <c r="J194" s="5" t="n">
+        <v>0.9983</v>
+      </c>
+      <c r="K194" s="5" t="n">
+        <v>0.9987</v>
+      </c>
+      <c r="L194" s="5" t="n">
+        <v>0.9976</v>
+      </c>
       <c r="M194" s="5" t="n">
-        <v>0.8671</v>
+        <v>0.9958</v>
       </c>
       <c r="N194" s="5" t="n">
-        <v>0.8423</v>
+        <v>0.9954</v>
       </c>
       <c r="O194" s="5" t="inlineStr"/>
-      <c r="P194" s="5" t="inlineStr"/>
+      <c r="P194" s="5" t="n">
+        <v>0.9961</v>
+      </c>
       <c r="Q194" s="5" t="inlineStr"/>
       <c r="R194" s="5" t="inlineStr"/>
       <c r="S194" s="5" t="inlineStr"/>
@@ -12250,339 +12300,6 @@
       <c r="U194" s="6" t="inlineStr"/>
       <c r="V194" s="5" t="inlineStr"/>
       <c r="W194" s="6" t="inlineStr"/>
-    </row>
-    <row r="195">
-      <c r="A195" s="3" t="inlineStr">
-        <is>
-          <t>CAPBES1G</t>
-        </is>
-      </c>
-      <c r="B195" s="3" t="inlineStr">
-        <is>
-          <t>Capital Battery</t>
-        </is>
-      </c>
-      <c r="C195" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="D195" s="4" t="n">
-        <v>125</v>
-      </c>
-      <c r="E195" s="5" t="inlineStr"/>
-      <c r="F195" s="5" t="inlineStr"/>
-      <c r="G195" s="5" t="inlineStr"/>
-      <c r="H195" s="5" t="inlineStr"/>
-      <c r="I195" s="5" t="inlineStr"/>
-      <c r="J195" s="5" t="inlineStr"/>
-      <c r="K195" s="5" t="inlineStr"/>
-      <c r="L195" s="5" t="inlineStr"/>
-      <c r="M195" s="5" t="n">
-        <v>0.9704</v>
-      </c>
-      <c r="N195" s="5" t="n">
-        <v>0.9337</v>
-      </c>
-      <c r="O195" s="5" t="inlineStr"/>
-      <c r="P195" s="5" t="inlineStr"/>
-      <c r="Q195" s="5" t="inlineStr"/>
-      <c r="R195" s="5" t="inlineStr"/>
-      <c r="S195" s="5" t="inlineStr"/>
-      <c r="T195" s="5" t="inlineStr"/>
-      <c r="U195" s="6" t="inlineStr"/>
-      <c r="V195" s="5" t="inlineStr"/>
-      <c r="W195" s="6" t="inlineStr"/>
-    </row>
-    <row r="196">
-      <c r="A196" s="3" t="inlineStr">
-        <is>
-          <t>WALGRVG1</t>
-        </is>
-      </c>
-      <c r="B196" s="3" t="inlineStr">
-        <is>
-          <t>Wallgrove BESS 1</t>
-        </is>
-      </c>
-      <c r="C196" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="D196" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E196" s="5" t="inlineStr"/>
-      <c r="F196" s="5" t="inlineStr"/>
-      <c r="G196" s="5" t="inlineStr"/>
-      <c r="H196" s="5" t="inlineStr"/>
-      <c r="I196" s="5" t="inlineStr"/>
-      <c r="J196" s="5" t="inlineStr"/>
-      <c r="K196" s="5" t="n">
-        <v>1.0011</v>
-      </c>
-      <c r="L196" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="M196" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="N196" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="O196" s="5" t="inlineStr"/>
-      <c r="P196" s="5" t="inlineStr"/>
-      <c r="Q196" s="5" t="inlineStr"/>
-      <c r="R196" s="5" t="inlineStr"/>
-      <c r="S196" s="5" t="inlineStr"/>
-      <c r="T196" s="5" t="inlineStr"/>
-      <c r="U196" s="6" t="inlineStr"/>
-      <c r="V196" s="5" t="inlineStr"/>
-      <c r="W196" s="6" t="inlineStr"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="3" t="inlineStr">
-        <is>
-          <t>DPNTBG1</t>
-        </is>
-      </c>
-      <c r="B197" s="3" t="inlineStr">
-        <is>
-          <t>Darlington Point Energy Storage System</t>
-        </is>
-      </c>
-      <c r="C197" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="D197" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="E197" s="5" t="inlineStr"/>
-      <c r="F197" s="5" t="inlineStr"/>
-      <c r="G197" s="5" t="inlineStr"/>
-      <c r="H197" s="5" t="inlineStr"/>
-      <c r="I197" s="5" t="inlineStr"/>
-      <c r="J197" s="5" t="inlineStr"/>
-      <c r="K197" s="5" t="inlineStr"/>
-      <c r="L197" s="5" t="n">
-        <v>0.9402</v>
-      </c>
-      <c r="M197" s="5" t="n">
-        <v>0.9089</v>
-      </c>
-      <c r="N197" s="5" t="n">
-        <v>0.9048</v>
-      </c>
-      <c r="O197" s="5" t="inlineStr"/>
-      <c r="P197" s="5" t="inlineStr"/>
-      <c r="Q197" s="5" t="inlineStr"/>
-      <c r="R197" s="5" t="inlineStr"/>
-      <c r="S197" s="5" t="inlineStr"/>
-      <c r="T197" s="5" t="inlineStr"/>
-      <c r="U197" s="6" t="inlineStr"/>
-      <c r="V197" s="5" t="inlineStr"/>
-      <c r="W197" s="6" t="inlineStr"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="3" t="inlineStr">
-        <is>
-          <t>MLLFGEF1</t>
-        </is>
-      </c>
-      <c r="B198" s="3" t="inlineStr">
-        <is>
-          <t>Mugga Lane Landfill Gas To Energy Facility</t>
-        </is>
-      </c>
-      <c r="C198" s="3" t="inlineStr">
-        <is>
-          <t>Other Renewable</t>
-        </is>
-      </c>
-      <c r="D198" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E198" s="5" t="inlineStr"/>
-      <c r="F198" s="5" t="inlineStr"/>
-      <c r="G198" s="5" t="inlineStr"/>
-      <c r="H198" s="5" t="inlineStr"/>
-      <c r="I198" s="5" t="inlineStr"/>
-      <c r="J198" s="5" t="inlineStr"/>
-      <c r="K198" s="5" t="n">
-        <v>0.9683</v>
-      </c>
-      <c r="L198" s="5" t="n">
-        <v>0.9687</v>
-      </c>
-      <c r="M198" s="5" t="n">
-        <v>0.9663</v>
-      </c>
-      <c r="N198" s="5" t="n">
-        <v>0.9567</v>
-      </c>
-      <c r="O198" s="5" t="inlineStr"/>
-      <c r="P198" s="5" t="inlineStr"/>
-      <c r="Q198" s="5" t="inlineStr"/>
-      <c r="R198" s="5" t="inlineStr"/>
-      <c r="S198" s="5" t="inlineStr"/>
-      <c r="T198" s="5" t="inlineStr"/>
-      <c r="U198" s="6" t="inlineStr"/>
-      <c r="V198" s="5" t="inlineStr"/>
-      <c r="W198" s="6" t="inlineStr"/>
-    </row>
-    <row r="199">
-      <c r="A199" s="3" t="inlineStr">
-        <is>
-          <t>RESS1G</t>
-        </is>
-      </c>
-      <c r="B199" s="3" t="inlineStr">
-        <is>
-          <t>Riverina BESS 1</t>
-        </is>
-      </c>
-      <c r="C199" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="D199" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="E199" s="5" t="inlineStr"/>
-      <c r="F199" s="5" t="inlineStr"/>
-      <c r="G199" s="5" t="inlineStr"/>
-      <c r="H199" s="5" t="inlineStr"/>
-      <c r="I199" s="5" t="inlineStr"/>
-      <c r="J199" s="5" t="inlineStr"/>
-      <c r="K199" s="5" t="inlineStr"/>
-      <c r="L199" s="5" t="n">
-        <v>0.9286</v>
-      </c>
-      <c r="M199" s="5" t="n">
-        <v>0.9089</v>
-      </c>
-      <c r="N199" s="5" t="n">
-        <v>0.8702</v>
-      </c>
-      <c r="O199" s="5" t="inlineStr"/>
-      <c r="P199" s="5" t="inlineStr"/>
-      <c r="Q199" s="5" t="inlineStr"/>
-      <c r="R199" s="5" t="inlineStr"/>
-      <c r="S199" s="5" t="inlineStr"/>
-      <c r="T199" s="5" t="inlineStr"/>
-      <c r="U199" s="6" t="inlineStr"/>
-      <c r="V199" s="5" t="inlineStr"/>
-      <c r="W199" s="6" t="inlineStr"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="3" t="inlineStr">
-        <is>
-          <t>RIVNBG2</t>
-        </is>
-      </c>
-      <c r="B200" s="3" t="inlineStr">
-        <is>
-          <t>Riverina Energy Storage System 2</t>
-        </is>
-      </c>
-      <c r="C200" s="3" t="inlineStr">
-        <is>
-          <t>Battery</t>
-        </is>
-      </c>
-      <c r="D200" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="E200" s="5" t="inlineStr"/>
-      <c r="F200" s="5" t="inlineStr"/>
-      <c r="G200" s="5" t="inlineStr"/>
-      <c r="H200" s="5" t="inlineStr"/>
-      <c r="I200" s="5" t="inlineStr"/>
-      <c r="J200" s="5" t="inlineStr"/>
-      <c r="K200" s="5" t="inlineStr"/>
-      <c r="L200" s="5" t="n">
-        <v>0.9058</v>
-      </c>
-      <c r="M200" s="5" t="n">
-        <v>0.9106</v>
-      </c>
-      <c r="N200" s="5" t="n">
-        <v>0.9048</v>
-      </c>
-      <c r="O200" s="5" t="inlineStr"/>
-      <c r="P200" s="5" t="inlineStr"/>
-      <c r="Q200" s="5" t="inlineStr"/>
-      <c r="R200" s="5" t="inlineStr"/>
-      <c r="S200" s="5" t="inlineStr"/>
-      <c r="T200" s="5" t="inlineStr"/>
-      <c r="U200" s="6" t="inlineStr"/>
-      <c r="V200" s="5" t="inlineStr"/>
-      <c r="W200" s="6" t="inlineStr"/>
-    </row>
-    <row r="201">
-      <c r="A201" s="3" t="inlineStr">
-        <is>
-          <t>WESTCBT1</t>
-        </is>
-      </c>
-      <c r="B201" s="3" t="inlineStr">
-        <is>
-          <t>Western Suburbs League Club (Campbelltown) Plant</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
-        <is>
-          <t>Fossil</t>
-        </is>
-      </c>
-      <c r="D201" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E201" s="5" t="n">
-        <v>0.9991</v>
-      </c>
-      <c r="F201" s="5" t="n">
-        <v>1.0005</v>
-      </c>
-      <c r="G201" s="5" t="n">
-        <v>1.0001</v>
-      </c>
-      <c r="H201" s="5" t="n">
-        <v>1.0006</v>
-      </c>
-      <c r="I201" s="5" t="n">
-        <v>0.9973</v>
-      </c>
-      <c r="J201" s="5" t="n">
-        <v>0.9983</v>
-      </c>
-      <c r="K201" s="5" t="n">
-        <v>0.9987</v>
-      </c>
-      <c r="L201" s="5" t="n">
-        <v>0.9976</v>
-      </c>
-      <c r="M201" s="5" t="n">
-        <v>0.9958</v>
-      </c>
-      <c r="N201" s="5" t="n">
-        <v>0.9954</v>
-      </c>
-      <c r="O201" s="5" t="inlineStr"/>
-      <c r="P201" s="5" t="n">
-        <v>0.9961</v>
-      </c>
-      <c r="Q201" s="5" t="inlineStr"/>
-      <c r="R201" s="5" t="inlineStr"/>
-      <c r="S201" s="5" t="inlineStr"/>
-      <c r="T201" s="5" t="inlineStr"/>
-      <c r="U201" s="6" t="inlineStr"/>
-      <c r="V201" s="5" t="inlineStr"/>
-      <c r="W201" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12595,7 +12312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P201"/>
+  <dimension ref="A1:P194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12775,12 +12492,14 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr"/>
       <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="E4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -12815,14 +12534,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="D5" s="5" t="inlineStr"/>
       <c r="E5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -13441,7 +13158,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr"/>
@@ -13449,8 +13166,12 @@
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="n">
+        <v>0.9645</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0.8799</v>
+      </c>
       <c r="I21" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -13473,7 +13194,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr"/>
@@ -13481,9 +13202,7 @@
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr"/>
       <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="5" t="n">
-        <v>0.9645</v>
-      </c>
+      <c r="G22" s="5" t="inlineStr"/>
       <c r="H22" s="5" t="n">
         <v>0.8799</v>
       </c>
@@ -13509,7 +13228,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr"/>
@@ -13541,7 +13260,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr"/>
@@ -13550,9 +13269,7 @@
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="5" t="n">
-        <v>0.8799</v>
-      </c>
+      <c r="H24" s="5" t="inlineStr"/>
       <c r="I24" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -13659,7 +13376,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr"/>
@@ -13691,7 +13408,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr"/>
@@ -13723,7 +13440,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>MULWASF1</t>
+          <t>CRWASF1</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr"/>
@@ -13731,14 +13448,24 @@
       <c r="D30" s="5" t="inlineStr"/>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr"/>
-      <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="inlineStr"/>
-      <c r="K30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="n">
+        <v>0.9497</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>0.9365</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>0.8979</v>
+      </c>
       <c r="L30" s="5" t="inlineStr"/>
       <c r="M30" s="5" t="n">
-        <v>0.9345</v>
+        <v>0.9355</v>
       </c>
       <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="n">
@@ -13749,7 +13476,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>CRWASF1</t>
+          <t>MULWASF1</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr"/>
@@ -13757,24 +13484,14 @@
       <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="5" t="n">
-        <v>0.9497</v>
-      </c>
-      <c r="H31" s="5" t="n">
-        <v>0.8813</v>
-      </c>
-      <c r="I31" s="5" t="n">
-        <v>0.9242</v>
-      </c>
-      <c r="J31" s="5" t="n">
-        <v>0.9365</v>
-      </c>
-      <c r="K31" s="5" t="n">
-        <v>0.8979</v>
-      </c>
+      <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="5" t="inlineStr"/>
+      <c r="I31" s="5" t="inlineStr"/>
+      <c r="J31" s="5" t="inlineStr"/>
+      <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="5" t="inlineStr"/>
       <c r="M31" s="5" t="n">
-        <v>0.9355</v>
+        <v>0.9345</v>
       </c>
       <c r="N31" s="5" t="inlineStr"/>
       <c r="O31" s="5" t="n">
@@ -14071,7 +13788,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>NESBESS2</t>
+          <t>NESBESS1</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr"/>
@@ -14101,7 +13818,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NESBESS1</t>
+          <t>NESBESS2</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr"/>
@@ -14211,7 +13928,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
@@ -14257,7 +13974,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
@@ -14303,7 +14020,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
@@ -14349,7 +14066,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
@@ -14471,14 +14188,16 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr"/>
       <c r="C50" s="5" t="inlineStr"/>
       <c r="D50" s="5" t="inlineStr"/>
       <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="G50" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -14507,7 +14226,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr"/>
@@ -14549,13 +14268,17 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>NASF1</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr"/>
       <c r="C52" s="5" t="inlineStr"/>
-      <c r="D52" s="5" t="inlineStr"/>
-      <c r="E52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>0.9708</v>
+      </c>
       <c r="F52" s="5" t="n">
         <v>0.9582000000000001</v>
       </c>
@@ -14633,20 +14356,14 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr"/>
       <c r="C54" s="5" t="inlineStr"/>
-      <c r="D54" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="E54" s="5" t="n">
-        <v>0.9708</v>
-      </c>
-      <c r="F54" s="5" t="n">
-        <v>0.9582000000000001</v>
-      </c>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="inlineStr"/>
       <c r="G54" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -14823,7 +14540,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>STUBSF2</t>
+          <t>STUBSF1</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr"/>
@@ -14851,7 +14568,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>STUBSF1</t>
+          <t>STUBSF2</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr"/>
@@ -15181,7 +14898,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B68" s="5" t="n">
@@ -15227,7 +14944,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B69" s="5" t="n">
@@ -15655,7 +15372,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>BW04</t>
+          <t>BW03</t>
         </is>
       </c>
       <c r="B81" s="5" t="n">
@@ -15701,7 +15418,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>BW03</t>
+          <t>BW04</t>
         </is>
       </c>
       <c r="B82" s="5" t="n">
@@ -15747,7 +15464,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>BW02</t>
+          <t>BW01</t>
         </is>
       </c>
       <c r="B83" s="5" t="n">
@@ -15793,7 +15510,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>BW01</t>
+          <t>BW02</t>
         </is>
       </c>
       <c r="B84" s="5" t="n">
@@ -15839,13 +15556,17 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF2</t>
+          <t>GULLRSF1</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr"/>
       <c r="C85" s="5" t="inlineStr"/>
-      <c r="D85" s="5" t="inlineStr"/>
-      <c r="E85" s="5" t="inlineStr"/>
+      <c r="D85" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="E85" s="5" t="n">
+        <v>0.9959</v>
+      </c>
       <c r="F85" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -15877,21 +15598,13 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF1</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="C86" s="5" t="n">
-        <v>0.9909</v>
-      </c>
-      <c r="D86" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="E86" s="5" t="n">
-        <v>0.9959</v>
-      </c>
+          <t>GULLRWF2</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr"/>
+      <c r="C86" s="5" t="inlineStr"/>
+      <c r="D86" s="5" t="inlineStr"/>
+      <c r="E86" s="5" t="inlineStr"/>
       <c r="F86" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -15923,11 +15636,15 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>GULLRSF1</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr"/>
-      <c r="C87" s="5" t="inlineStr"/>
+          <t>GULLRWF1</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="C87" s="5" t="n">
+        <v>0.9909</v>
+      </c>
       <c r="D87" s="5" t="n">
         <v>1.001</v>
       </c>
@@ -16239,7 +15956,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B95" s="5" t="n">
@@ -16285,7 +16002,7 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B96" s="5" t="n">
@@ -16513,7 +16230,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MPNL1</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B101" s="5" t="n">
@@ -16605,7 +16322,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MPNL1</t>
         </is>
       </c>
       <c r="B103" s="5" t="n">
@@ -16753,8 +16470,12 @@
       <c r="F106" s="5" t="inlineStr"/>
       <c r="G106" s="5" t="inlineStr"/>
       <c r="H106" s="5" t="inlineStr"/>
-      <c r="I106" s="5" t="inlineStr"/>
-      <c r="J106" s="5" t="inlineStr"/>
+      <c r="I106" s="5" t="n">
+        <v>0.9058</v>
+      </c>
+      <c r="J106" s="5" t="n">
+        <v>0.9106</v>
+      </c>
       <c r="K106" s="5" t="n">
         <v>0.9048</v>
       </c>
@@ -16777,7 +16498,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B107" s="5" t="n">
@@ -16823,7 +16544,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B108" s="5" t="n">
@@ -16869,7 +16590,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-2</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B109" s="5" t="n">
@@ -16915,7 +16636,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B110" s="5" t="n">
@@ -16961,7 +16682,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT2-2</t>
         </is>
       </c>
       <c r="B111" s="5" t="n">
@@ -17007,7 +16728,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B112" s="5" t="n">
@@ -17053,7 +16774,7 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B113" s="5" t="n">
@@ -17155,8 +16876,12 @@
       <c r="F115" s="5" t="inlineStr"/>
       <c r="G115" s="5" t="inlineStr"/>
       <c r="H115" s="5" t="inlineStr"/>
-      <c r="I115" s="5" t="inlineStr"/>
-      <c r="J115" s="5" t="inlineStr"/>
+      <c r="I115" s="5" t="n">
+        <v>0.9402</v>
+      </c>
+      <c r="J115" s="5" t="n">
+        <v>0.9089</v>
+      </c>
       <c r="K115" s="5" t="n">
         <v>0.9048</v>
       </c>
@@ -17216,7 +16941,9 @@
       <c r="G117" s="5" t="inlineStr"/>
       <c r="H117" s="5" t="inlineStr"/>
       <c r="I117" s="5" t="inlineStr"/>
-      <c r="J117" s="5" t="inlineStr"/>
+      <c r="J117" s="5" t="n">
+        <v>0.9704</v>
+      </c>
       <c r="K117" s="5" t="n">
         <v>0.9337</v>
       </c>
@@ -17319,7 +17046,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B120" s="5" t="n">
@@ -17411,7 +17138,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B122" s="5" t="n">
@@ -17468,7 +17195,9 @@
       <c r="G123" s="5" t="inlineStr"/>
       <c r="H123" s="5" t="inlineStr"/>
       <c r="I123" s="5" t="inlineStr"/>
-      <c r="J123" s="5" t="inlineStr"/>
+      <c r="J123" s="5" t="n">
+        <v>0.8671</v>
+      </c>
       <c r="K123" s="5" t="n">
         <v>0.8423</v>
       </c>
@@ -17491,42 +17220,30 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="n">
-        <v>0.9856</v>
-      </c>
-      <c r="C124" s="5" t="n">
-        <v>0.9829</v>
-      </c>
-      <c r="D124" s="5" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="E124" s="5" t="n">
-        <v>0.9828</v>
-      </c>
-      <c r="F124" s="5" t="n">
-        <v>0.9836</v>
-      </c>
-      <c r="G124" s="5" t="n">
-        <v>0.9835</v>
-      </c>
+          <t>HEZ1</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr"/>
+      <c r="C124" s="5" t="inlineStr"/>
+      <c r="D124" s="5" t="inlineStr"/>
+      <c r="E124" s="5" t="inlineStr"/>
+      <c r="F124" s="5" t="inlineStr"/>
+      <c r="G124" s="5" t="inlineStr"/>
       <c r="H124" s="5" t="n">
-        <v>0.9849</v>
+        <v>0.9897</v>
       </c>
       <c r="I124" s="5" t="n">
-        <v>0.9865</v>
+        <v>0.992</v>
       </c>
       <c r="J124" s="5" t="n">
-        <v>0.9848</v>
+        <v>0.9899</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>0.9855</v>
+        <v>0.9896</v>
       </c>
       <c r="L124" s="5" t="inlineStr"/>
       <c r="M124" s="5" t="n">
-        <v>0.9846</v>
+        <v>0.9931</v>
       </c>
       <c r="N124" s="5" t="inlineStr"/>
       <c r="O124" s="5" t="n">
@@ -17537,7 +17254,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B125" s="5" t="n">
@@ -17583,7 +17300,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B126" s="5" t="n">
@@ -17629,30 +17346,42 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>HEZ1</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="inlineStr"/>
-      <c r="C127" s="5" t="inlineStr"/>
-      <c r="D127" s="5" t="inlineStr"/>
-      <c r="E127" s="5" t="inlineStr"/>
-      <c r="F127" s="5" t="inlineStr"/>
-      <c r="G127" s="5" t="inlineStr"/>
+          <t>ER01</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="C127" s="5" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="D127" s="5" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E127" s="5" t="n">
+        <v>0.9828</v>
+      </c>
+      <c r="F127" s="5" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="G127" s="5" t="n">
+        <v>0.9835</v>
+      </c>
       <c r="H127" s="5" t="n">
-        <v>0.9897</v>
+        <v>0.9849</v>
       </c>
       <c r="I127" s="5" t="n">
-        <v>0.992</v>
+        <v>0.9865</v>
       </c>
       <c r="J127" s="5" t="n">
-        <v>0.9899</v>
+        <v>0.9848</v>
       </c>
       <c r="K127" s="5" t="n">
-        <v>0.9896</v>
+        <v>0.9855</v>
       </c>
       <c r="L127" s="5" t="inlineStr"/>
       <c r="M127" s="5" t="n">
-        <v>0.9931</v>
+        <v>0.9846</v>
       </c>
       <c r="N127" s="5" t="inlineStr"/>
       <c r="O127" s="5" t="n">
@@ -17845,8 +17574,12 @@
       <c r="F132" s="5" t="inlineStr"/>
       <c r="G132" s="5" t="inlineStr"/>
       <c r="H132" s="5" t="inlineStr"/>
-      <c r="I132" s="5" t="inlineStr"/>
-      <c r="J132" s="5" t="inlineStr"/>
+      <c r="I132" s="5" t="n">
+        <v>0.9286</v>
+      </c>
+      <c r="J132" s="5" t="n">
+        <v>0.9089</v>
+      </c>
       <c r="K132" s="5" t="n">
         <v>0.8702</v>
       </c>
@@ -17915,7 +17648,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B134" s="5" t="n">
@@ -17961,7 +17694,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B135" s="5" t="n">
@@ -18007,7 +17740,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B136" s="5" t="n">
@@ -18053,7 +17786,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B137" s="5" t="n">
@@ -18099,7 +17832,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B138" s="5" t="n">
@@ -18321,7 +18054,7 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>BROWNMT</t>
+          <t>JNDABNE1</t>
         </is>
       </c>
       <c r="B144" s="5" t="n">
@@ -18367,7 +18100,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>JNDABNE1</t>
+          <t>BROWNMT</t>
         </is>
       </c>
       <c r="B145" s="5" t="n">
@@ -18505,33 +18238,17 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>WESTILL1</t>
-        </is>
-      </c>
-      <c r="B148" s="5" t="n">
-        <v>0.9916</v>
-      </c>
-      <c r="C148" s="5" t="n">
-        <v>0.9986</v>
-      </c>
-      <c r="D148" s="5" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="E148" s="5" t="n">
-        <v>1.0037</v>
-      </c>
-      <c r="F148" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="G148" s="5" t="n">
-        <v>0.9967</v>
-      </c>
-      <c r="H148" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="I148" s="5" t="n">
-        <v>0.9933999999999999</v>
-      </c>
+          <t>SHOAL1</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr"/>
+      <c r="C148" s="5" t="inlineStr"/>
+      <c r="D148" s="5" t="inlineStr"/>
+      <c r="E148" s="5" t="inlineStr"/>
+      <c r="F148" s="5" t="inlineStr"/>
+      <c r="G148" s="5" t="inlineStr"/>
+      <c r="H148" s="5" t="inlineStr"/>
+      <c r="I148" s="5" t="inlineStr"/>
       <c r="J148" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -18551,17 +18268,33 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>SHOAL1</t>
-        </is>
-      </c>
-      <c r="B149" s="5" t="inlineStr"/>
-      <c r="C149" s="5" t="inlineStr"/>
-      <c r="D149" s="5" t="inlineStr"/>
-      <c r="E149" s="5" t="inlineStr"/>
-      <c r="F149" s="5" t="inlineStr"/>
-      <c r="G149" s="5" t="inlineStr"/>
-      <c r="H149" s="5" t="inlineStr"/>
-      <c r="I149" s="5" t="inlineStr"/>
+          <t>WESTILL1</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="C149" s="5" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="D149" s="5" t="n">
+        <v>1.0023</v>
+      </c>
+      <c r="E149" s="5" t="n">
+        <v>1.0037</v>
+      </c>
+      <c r="F149" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>0.9967</v>
+      </c>
+      <c r="H149" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="I149" s="5" t="n">
+        <v>0.9933999999999999</v>
+      </c>
       <c r="J149" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -18683,8 +18416,12 @@
       <c r="F152" s="5" t="inlineStr"/>
       <c r="G152" s="5" t="inlineStr"/>
       <c r="H152" s="5" t="inlineStr"/>
-      <c r="I152" s="5" t="inlineStr"/>
-      <c r="J152" s="5" t="inlineStr"/>
+      <c r="I152" s="5" t="n">
+        <v>0.9752</v>
+      </c>
+      <c r="J152" s="5" t="n">
+        <v>0.979</v>
+      </c>
       <c r="K152" s="5" t="n">
         <v>0.9571</v>
       </c>
@@ -18707,7 +18444,7 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B153" s="5" t="n">
@@ -18753,7 +18490,7 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B154" s="5" t="n">
@@ -19259,7 +18996,7 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>WALGRV1</t>
+          <t>SMTHBES1</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr"/>
@@ -19271,29 +19008,25 @@
       <c r="H165" s="5" t="inlineStr"/>
       <c r="I165" s="5" t="inlineStr"/>
       <c r="J165" s="5" t="inlineStr"/>
-      <c r="K165" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="L165" s="5" t="n">
-        <v>1.0009</v>
-      </c>
+      <c r="K165" s="5" t="inlineStr"/>
+      <c r="L165" s="5" t="inlineStr"/>
       <c r="M165" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0016</v>
       </c>
       <c r="N165" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0017</v>
       </c>
       <c r="O165" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="P165" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0019</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>SMTHBES1</t>
+          <t>WALGRV1</t>
         </is>
       </c>
       <c r="B166" s="5" t="inlineStr"/>
@@ -19302,22 +19035,32 @@
       <c r="E166" s="5" t="inlineStr"/>
       <c r="F166" s="5" t="inlineStr"/>
       <c r="G166" s="5" t="inlineStr"/>
-      <c r="H166" s="5" t="inlineStr"/>
-      <c r="I166" s="5" t="inlineStr"/>
-      <c r="J166" s="5" t="inlineStr"/>
-      <c r="K166" s="5" t="inlineStr"/>
-      <c r="L166" s="5" t="inlineStr"/>
+      <c r="H166" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="I166" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="J166" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="K166" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="L166" s="5" t="n">
+        <v>1.0009</v>
+      </c>
       <c r="M166" s="5" t="n">
-        <v>1.0016</v>
+        <v>1.0018</v>
       </c>
       <c r="N166" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0015</v>
       </c>
       <c r="O166" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="P166" s="5" t="n">
-        <v>1.0019</v>
+        <v>1.0017</v>
       </c>
     </row>
     <row r="167">
@@ -19369,7 +19112,7 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B168" s="5" t="n">
@@ -19415,7 +19158,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B169" s="5" t="n">
@@ -19537,7 +19280,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B172" s="5" t="n">
@@ -19583,7 +19326,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B173" s="5" t="n">
@@ -19629,7 +19372,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B174" s="5" t="n">
@@ -19675,7 +19418,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B175" s="5" t="n">
@@ -19721,7 +19464,7 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B176" s="5" t="n">
@@ -19767,7 +19510,7 @@
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B177" s="5" t="n">
@@ -19955,27 +19698,29 @@
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AGLSITA1</t>
-        </is>
-      </c>
-      <c r="B183" s="5" t="inlineStr"/>
+          <t>AGLNOW1</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="n">
+        <v>0.9916</v>
+      </c>
       <c r="C183" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9986</v>
       </c>
       <c r="D183" s="5" t="n">
-        <v>1.0022</v>
+        <v>1.0023</v>
       </c>
       <c r="E183" s="5" t="n">
-        <v>1.0024</v>
+        <v>1.0037</v>
       </c>
       <c r="F183" s="5" t="n">
-        <v>1.0009</v>
+        <v>0.9929</v>
       </c>
       <c r="G183" s="5" t="n">
-        <v>1.0012</v>
+        <v>0.9967</v>
       </c>
       <c r="H183" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9929</v>
       </c>
       <c r="I183" s="5" t="inlineStr"/>
       <c r="J183" s="5" t="inlineStr"/>
@@ -19989,29 +19734,29 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B184" s="5" t="n">
-        <v>0.9916</v>
+        <v>0.9926</v>
       </c>
       <c r="C184" s="5" t="n">
-        <v>0.9986</v>
+        <v>0.9907</v>
       </c>
       <c r="D184" s="5" t="n">
-        <v>1.0023</v>
+        <v>0.9892</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9901</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>0.9967</v>
+        <v>0.9907</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>0.9929</v>
+        <v>0.9917</v>
       </c>
       <c r="I184" s="5" t="inlineStr"/>
       <c r="J184" s="5" t="inlineStr"/>
@@ -20025,29 +19770,29 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B185" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9676</v>
       </c>
       <c r="C185" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9593</v>
       </c>
       <c r="D185" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9509</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9537</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9593</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9631</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9628</v>
       </c>
       <c r="I185" s="5" t="inlineStr"/>
       <c r="J185" s="5" t="inlineStr"/>
@@ -20061,29 +19806,29 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B186" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="C186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="D186" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="I186" s="5" t="inlineStr"/>
       <c r="J186" s="5" t="inlineStr"/>
@@ -20133,29 +19878,29 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>WOYWOY1</t>
         </is>
       </c>
       <c r="B188" s="5" t="n">
-        <v>0.9926</v>
+        <v>1.0017</v>
       </c>
       <c r="C188" s="5" t="n">
-        <v>0.9907</v>
+        <v>1.0015</v>
       </c>
       <c r="D188" s="5" t="n">
-        <v>0.9892</v>
+        <v>1.0008</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>0.9901</v>
+        <v>1.0011</v>
       </c>
       <c r="F188" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>1.0036</v>
       </c>
       <c r="G188" s="5" t="n">
-        <v>0.9907</v>
+        <v>1.0019</v>
       </c>
       <c r="H188" s="5" t="n">
-        <v>0.9917</v>
+        <v>1.0037</v>
       </c>
       <c r="I188" s="5" t="inlineStr"/>
       <c r="J188" s="5" t="inlineStr"/>
@@ -20169,29 +19914,27 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
-        </is>
-      </c>
-      <c r="B189" s="5" t="n">
-        <v>1.0017</v>
-      </c>
+          <t>AGLSITA1</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr"/>
       <c r="C189" s="5" t="n">
+        <v>1.0019</v>
+      </c>
+      <c r="D189" s="5" t="n">
+        <v>1.0022</v>
+      </c>
+      <c r="E189" s="5" t="n">
+        <v>1.0024</v>
+      </c>
+      <c r="F189" s="5" t="n">
+        <v>1.0009</v>
+      </c>
+      <c r="G189" s="5" t="n">
+        <v>1.0012</v>
+      </c>
+      <c r="H189" s="5" t="n">
         <v>1.0015</v>
-      </c>
-      <c r="D189" s="5" t="n">
-        <v>1.0008</v>
-      </c>
-      <c r="E189" s="5" t="n">
-        <v>1.0011</v>
-      </c>
-      <c r="F189" s="5" t="n">
-        <v>1.0036</v>
-      </c>
-      <c r="G189" s="5" t="n">
-        <v>1.0019</v>
-      </c>
-      <c r="H189" s="5" t="n">
-        <v>1.0037</v>
       </c>
       <c r="I189" s="5" t="inlineStr"/>
       <c r="J189" s="5" t="inlineStr"/>
@@ -20205,7 +19948,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD04</t>
         </is>
       </c>
       <c r="B190" s="5" t="n">
@@ -20243,7 +19986,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>LD04</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B191" s="5" t="n">
@@ -20281,7 +20024,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B192" s="5" t="n">
@@ -20319,7 +20062,7 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>QBYNBG1</t>
+          <t>MLLFGEF1</t>
         </is>
       </c>
       <c r="B193" s="5" t="inlineStr"/>
@@ -20328,15 +20071,17 @@
       <c r="E193" s="5" t="inlineStr"/>
       <c r="F193" s="5" t="inlineStr"/>
       <c r="G193" s="5" t="inlineStr"/>
-      <c r="H193" s="5" t="inlineStr"/>
+      <c r="H193" s="5" t="n">
+        <v>0.9683</v>
+      </c>
       <c r="I193" s="5" t="n">
-        <v>0.9752</v>
+        <v>0.9687</v>
       </c>
       <c r="J193" s="5" t="n">
-        <v>0.979</v>
+        <v>0.9663</v>
       </c>
       <c r="K193" s="5" t="n">
-        <v>0.9571</v>
+        <v>0.9567</v>
       </c>
       <c r="L193" s="5" t="inlineStr"/>
       <c r="M193" s="5" t="inlineStr"/>
@@ -20347,245 +20092,49 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>BHBG1</t>
-        </is>
-      </c>
-      <c r="B194" s="5" t="inlineStr"/>
-      <c r="C194" s="5" t="inlineStr"/>
-      <c r="D194" s="5" t="inlineStr"/>
-      <c r="E194" s="5" t="inlineStr"/>
-      <c r="F194" s="5" t="inlineStr"/>
-      <c r="G194" s="5" t="inlineStr"/>
-      <c r="H194" s="5" t="inlineStr"/>
-      <c r="I194" s="5" t="inlineStr"/>
+          <t>WESTCBT1</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="n">
+        <v>0.9991</v>
+      </c>
+      <c r="C194" s="5" t="n">
+        <v>1.0005</v>
+      </c>
+      <c r="D194" s="5" t="n">
+        <v>1.0001</v>
+      </c>
+      <c r="E194" s="5" t="n">
+        <v>1.0006</v>
+      </c>
+      <c r="F194" s="5" t="n">
+        <v>0.9973</v>
+      </c>
+      <c r="G194" s="5" t="n">
+        <v>0.9983</v>
+      </c>
+      <c r="H194" s="5" t="n">
+        <v>0.9987</v>
+      </c>
+      <c r="I194" s="5" t="n">
+        <v>0.9976</v>
+      </c>
       <c r="J194" s="5" t="n">
-        <v>0.8671</v>
+        <v>0.9958</v>
       </c>
       <c r="K194" s="5" t="n">
-        <v>0.8423</v>
+        <v>0.9954</v>
       </c>
       <c r="L194" s="5" t="inlineStr"/>
-      <c r="M194" s="5" t="inlineStr"/>
+      <c r="M194" s="5" t="n">
+        <v>0.9961</v>
+      </c>
       <c r="N194" s="5" t="inlineStr"/>
       <c r="O194" s="5" t="inlineStr"/>
       <c r="P194" s="5" t="inlineStr"/>
     </row>
-    <row r="195">
-      <c r="A195" s="3" t="inlineStr">
-        <is>
-          <t>CAPBES1G</t>
-        </is>
-      </c>
-      <c r="B195" s="5" t="inlineStr"/>
-      <c r="C195" s="5" t="inlineStr"/>
-      <c r="D195" s="5" t="inlineStr"/>
-      <c r="E195" s="5" t="inlineStr"/>
-      <c r="F195" s="5" t="inlineStr"/>
-      <c r="G195" s="5" t="inlineStr"/>
-      <c r="H195" s="5" t="inlineStr"/>
-      <c r="I195" s="5" t="inlineStr"/>
-      <c r="J195" s="5" t="n">
-        <v>0.9704</v>
-      </c>
-      <c r="K195" s="5" t="n">
-        <v>0.9337</v>
-      </c>
-      <c r="L195" s="5" t="inlineStr"/>
-      <c r="M195" s="5" t="inlineStr"/>
-      <c r="N195" s="5" t="inlineStr"/>
-      <c r="O195" s="5" t="inlineStr"/>
-      <c r="P195" s="5" t="inlineStr"/>
-    </row>
-    <row r="196">
-      <c r="A196" s="3" t="inlineStr">
-        <is>
-          <t>WALGRVG1</t>
-        </is>
-      </c>
-      <c r="B196" s="5" t="inlineStr"/>
-      <c r="C196" s="5" t="inlineStr"/>
-      <c r="D196" s="5" t="inlineStr"/>
-      <c r="E196" s="5" t="inlineStr"/>
-      <c r="F196" s="5" t="inlineStr"/>
-      <c r="G196" s="5" t="inlineStr"/>
-      <c r="H196" s="5" t="n">
-        <v>1.0011</v>
-      </c>
-      <c r="I196" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="J196" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="K196" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="L196" s="5" t="inlineStr"/>
-      <c r="M196" s="5" t="inlineStr"/>
-      <c r="N196" s="5" t="inlineStr"/>
-      <c r="O196" s="5" t="inlineStr"/>
-      <c r="P196" s="5" t="inlineStr"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="3" t="inlineStr">
-        <is>
-          <t>DPNTBG1</t>
-        </is>
-      </c>
-      <c r="B197" s="5" t="inlineStr"/>
-      <c r="C197" s="5" t="inlineStr"/>
-      <c r="D197" s="5" t="inlineStr"/>
-      <c r="E197" s="5" t="inlineStr"/>
-      <c r="F197" s="5" t="inlineStr"/>
-      <c r="G197" s="5" t="inlineStr"/>
-      <c r="H197" s="5" t="inlineStr"/>
-      <c r="I197" s="5" t="n">
-        <v>0.9402</v>
-      </c>
-      <c r="J197" s="5" t="n">
-        <v>0.9089</v>
-      </c>
-      <c r="K197" s="5" t="n">
-        <v>0.9048</v>
-      </c>
-      <c r="L197" s="5" t="inlineStr"/>
-      <c r="M197" s="5" t="inlineStr"/>
-      <c r="N197" s="5" t="inlineStr"/>
-      <c r="O197" s="5" t="inlineStr"/>
-      <c r="P197" s="5" t="inlineStr"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="3" t="inlineStr">
-        <is>
-          <t>MLLFGEF1</t>
-        </is>
-      </c>
-      <c r="B198" s="5" t="inlineStr"/>
-      <c r="C198" s="5" t="inlineStr"/>
-      <c r="D198" s="5" t="inlineStr"/>
-      <c r="E198" s="5" t="inlineStr"/>
-      <c r="F198" s="5" t="inlineStr"/>
-      <c r="G198" s="5" t="inlineStr"/>
-      <c r="H198" s="5" t="n">
-        <v>0.9683</v>
-      </c>
-      <c r="I198" s="5" t="n">
-        <v>0.9687</v>
-      </c>
-      <c r="J198" s="5" t="n">
-        <v>0.9663</v>
-      </c>
-      <c r="K198" s="5" t="n">
-        <v>0.9567</v>
-      </c>
-      <c r="L198" s="5" t="inlineStr"/>
-      <c r="M198" s="5" t="inlineStr"/>
-      <c r="N198" s="5" t="inlineStr"/>
-      <c r="O198" s="5" t="inlineStr"/>
-      <c r="P198" s="5" t="inlineStr"/>
-    </row>
-    <row r="199">
-      <c r="A199" s="3" t="inlineStr">
-        <is>
-          <t>RESS1G</t>
-        </is>
-      </c>
-      <c r="B199" s="5" t="inlineStr"/>
-      <c r="C199" s="5" t="inlineStr"/>
-      <c r="D199" s="5" t="inlineStr"/>
-      <c r="E199" s="5" t="inlineStr"/>
-      <c r="F199" s="5" t="inlineStr"/>
-      <c r="G199" s="5" t="inlineStr"/>
-      <c r="H199" s="5" t="inlineStr"/>
-      <c r="I199" s="5" t="n">
-        <v>0.9286</v>
-      </c>
-      <c r="J199" s="5" t="n">
-        <v>0.9089</v>
-      </c>
-      <c r="K199" s="5" t="n">
-        <v>0.8702</v>
-      </c>
-      <c r="L199" s="5" t="inlineStr"/>
-      <c r="M199" s="5" t="inlineStr"/>
-      <c r="N199" s="5" t="inlineStr"/>
-      <c r="O199" s="5" t="inlineStr"/>
-      <c r="P199" s="5" t="inlineStr"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="3" t="inlineStr">
-        <is>
-          <t>RIVNBG2</t>
-        </is>
-      </c>
-      <c r="B200" s="5" t="inlineStr"/>
-      <c r="C200" s="5" t="inlineStr"/>
-      <c r="D200" s="5" t="inlineStr"/>
-      <c r="E200" s="5" t="inlineStr"/>
-      <c r="F200" s="5" t="inlineStr"/>
-      <c r="G200" s="5" t="inlineStr"/>
-      <c r="H200" s="5" t="inlineStr"/>
-      <c r="I200" s="5" t="n">
-        <v>0.9058</v>
-      </c>
-      <c r="J200" s="5" t="n">
-        <v>0.9106</v>
-      </c>
-      <c r="K200" s="5" t="n">
-        <v>0.9048</v>
-      </c>
-      <c r="L200" s="5" t="inlineStr"/>
-      <c r="M200" s="5" t="inlineStr"/>
-      <c r="N200" s="5" t="inlineStr"/>
-      <c r="O200" s="5" t="inlineStr"/>
-      <c r="P200" s="5" t="inlineStr"/>
-    </row>
-    <row r="201">
-      <c r="A201" s="3" t="inlineStr">
-        <is>
-          <t>WESTCBT1</t>
-        </is>
-      </c>
-      <c r="B201" s="5" t="n">
-        <v>0.9991</v>
-      </c>
-      <c r="C201" s="5" t="n">
-        <v>1.0005</v>
-      </c>
-      <c r="D201" s="5" t="n">
-        <v>1.0001</v>
-      </c>
-      <c r="E201" s="5" t="n">
-        <v>1.0006</v>
-      </c>
-      <c r="F201" s="5" t="n">
-        <v>0.9973</v>
-      </c>
-      <c r="G201" s="5" t="n">
-        <v>0.9983</v>
-      </c>
-      <c r="H201" s="5" t="n">
-        <v>0.9987</v>
-      </c>
-      <c r="I201" s="5" t="n">
-        <v>0.9976</v>
-      </c>
-      <c r="J201" s="5" t="n">
-        <v>0.9958</v>
-      </c>
-      <c r="K201" s="5" t="n">
-        <v>0.9954</v>
-      </c>
-      <c r="L201" s="5" t="inlineStr"/>
-      <c r="M201" s="5" t="n">
-        <v>0.9961</v>
-      </c>
-      <c r="N201" s="5" t="inlineStr"/>
-      <c r="O201" s="5" t="inlineStr"/>
-      <c r="P201" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B201">
+  <conditionalFormatting sqref="B2:B194">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -20597,7 +20146,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C201">
+  <conditionalFormatting sqref="C2:C194">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -20609,7 +20158,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D201">
+  <conditionalFormatting sqref="D2:D194">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -20621,7 +20170,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E201">
+  <conditionalFormatting sqref="E2:E194">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -20633,7 +20182,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F201">
+  <conditionalFormatting sqref="F2:F194">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -20645,7 +20194,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G201">
+  <conditionalFormatting sqref="G2:G194">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -20657,7 +20206,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H201">
+  <conditionalFormatting sqref="H2:H194">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -20669,7 +20218,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I201">
+  <conditionalFormatting sqref="I2:I194">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -20681,7 +20230,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J201">
+  <conditionalFormatting sqref="J2:J194">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -20693,7 +20242,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K201">
+  <conditionalFormatting sqref="K2:K194">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -20705,7 +20254,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L201">
+  <conditionalFormatting sqref="M2:M194">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -20717,44 +20266,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M201">
+  <conditionalFormatting sqref="O2:O194">
     <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="00F8696B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="0063BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N201">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="00F8696B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="0063BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O201">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="00F8696B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="0063BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P201">
-    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -21095,12 +20608,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Junee Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -21124,12 +20637,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>Sebastopol Solar Farm</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -21153,12 +20666,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Sebastopol Solar Farm</t>
+          <t>Junee Solar Farm</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -21632,7 +21145,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -21661,7 +21174,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -21922,7 +21435,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -21951,7 +21464,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -21980,7 +21493,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update MLF data 2026-10-07
</commit_message>
<xml_diff>
--- a/outputs/NSW_mlf.xlsx
+++ b/outputs/NSW_mlf.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MLF Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Biggest Movers" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -725,27 +725,25 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>White Rock Wind Farm</t>
+          <t>White Rock Solar Farm</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>175</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -788,25 +786,27 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>White Rock Solar Farm</t>
+          <t>White Rock Wind Farm</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>22</v>
+        <v>175</v>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="H5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -1748,12 +1748,12 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Junee Solar Farm</t>
+          <t>West Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1762,19 +1762,15 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr"/>
       <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="n">
-        <v>0.9645</v>
-      </c>
-      <c r="K21" s="5" t="n">
-        <v>0.8799</v>
-      </c>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -1805,12 +1801,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Sebastopol Solar Farm</t>
+          <t>Junee Solar Farm</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1819,14 +1815,16 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>110</v>
+        <v>36</v>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
       <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr"/>
       <c r="H22" s="5" t="inlineStr"/>
       <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="n">
+        <v>0.9645</v>
+      </c>
       <c r="K22" s="5" t="n">
         <v>0.8799</v>
       </c>
@@ -1860,12 +1858,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>West Wyalong Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1874,7 +1872,7 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1913,12 +1911,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>Sebastopol Solar Farm</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1927,7 +1925,7 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>62</v>
+        <v>110</v>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
@@ -1935,7 +1933,9 @@
       <c r="H24" s="5" t="inlineStr"/>
       <c r="I24" s="5" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr"/>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="n">
+        <v>0.8799</v>
+      </c>
       <c r="L24" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -2113,7 +2113,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -2166,7 +2166,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -2219,12 +2219,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>CRWASF1</t>
+          <t>MULWASF1</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Corowa Solar Farm</t>
+          <t>Mulwala Solar Farm</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2233,31 +2233,21 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr"/>
       <c r="H30" s="5" t="inlineStr"/>
       <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="n">
-        <v>0.9497</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>0.8813</v>
-      </c>
-      <c r="L30" s="5" t="n">
-        <v>0.9242</v>
-      </c>
-      <c r="M30" s="5" t="n">
-        <v>0.9365</v>
-      </c>
-      <c r="N30" s="5" t="n">
-        <v>0.8979</v>
-      </c>
+      <c r="J30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr"/>
+      <c r="M30" s="5" t="inlineStr"/>
+      <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr"/>
       <c r="P30" s="5" t="n">
-        <v>0.9355</v>
+        <v>0.9345</v>
       </c>
       <c r="Q30" s="5" t="inlineStr"/>
       <c r="R30" s="5" t="n">
@@ -2265,10 +2255,10 @@
       </c>
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="n">
-        <v>-0.0443</v>
+        <v>-0.0433</v>
       </c>
       <c r="U30" s="6" t="n">
-        <v>-4.74</v>
+        <v>-4.63</v>
       </c>
       <c r="V30" s="5" t="inlineStr"/>
       <c r="W30" s="6" t="inlineStr"/>
@@ -2276,12 +2266,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>MULWASF1</t>
+          <t>CRWASF1</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Mulwala Solar Farm</t>
+          <t>Corowa Solar Farm</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2290,21 +2280,31 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr"/>
       <c r="H31" s="5" t="inlineStr"/>
       <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
-      <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr"/>
-      <c r="M31" s="5" t="inlineStr"/>
-      <c r="N31" s="5" t="inlineStr"/>
+      <c r="J31" s="5" t="n">
+        <v>0.9497</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>0.9365</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>0.8979</v>
+      </c>
       <c r="O31" s="5" t="inlineStr"/>
       <c r="P31" s="5" t="n">
-        <v>0.9345</v>
+        <v>0.9355</v>
       </c>
       <c r="Q31" s="5" t="inlineStr"/>
       <c r="R31" s="5" t="n">
@@ -2312,10 +2312,10 @@
       </c>
       <c r="S31" s="5" t="inlineStr"/>
       <c r="T31" s="5" t="n">
-        <v>-0.0433</v>
+        <v>-0.0443</v>
       </c>
       <c r="U31" s="6" t="n">
-        <v>-4.63</v>
+        <v>-4.74</v>
       </c>
       <c r="V31" s="5" t="inlineStr"/>
       <c r="W31" s="6" t="inlineStr"/>
@@ -2781,7 +2781,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>NESBESS1</t>
+          <t>NESBESS2</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NESBESS2</t>
+          <t>NESBESS1</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -3013,7 +3013,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -3080,7 +3080,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -3147,7 +3147,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -3214,7 +3214,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -3399,12 +3399,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Nevertire Solar Farm</t>
+          <t xml:space="preserve">Wellington Solar Farm </t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3413,15 +3413,13 @@
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>132</v>
+        <v>216</v>
       </c>
       <c r="E50" s="5" t="inlineStr"/>
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr"/>
       <c r="H50" s="5" t="inlineStr"/>
-      <c r="I50" s="5" t="n">
-        <v>0.9582000000000001</v>
-      </c>
+      <c r="I50" s="5" t="inlineStr"/>
       <c r="J50" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -3458,12 +3456,12 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
+          <t>NASF1</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>South Keswick Solar Farm</t>
+          <t>Narromine Solar Farm</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3472,7 +3470,7 @@
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
       <c r="F51" s="5" t="inlineStr"/>
@@ -3521,12 +3519,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Narromine Solar Farm</t>
+          <t>Nevertire Solar Farm</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3535,16 +3533,12 @@
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>10</v>
+        <v>132</v>
       </c>
       <c r="E52" s="5" t="inlineStr"/>
       <c r="F52" s="5" t="inlineStr"/>
-      <c r="G52" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="H52" s="5" t="n">
-        <v>0.9708</v>
-      </c>
+      <c r="G52" s="5" t="inlineStr"/>
+      <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="n">
         <v>0.9582000000000001</v>
       </c>
@@ -3651,12 +3645,12 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wellington Solar Farm </t>
+          <t>South Keswick Solar Farm</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -3665,13 +3659,19 @@
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>216</v>
+        <v>15</v>
       </c>
       <c r="E54" s="5" t="inlineStr"/>
       <c r="F54" s="5" t="inlineStr"/>
-      <c r="G54" s="5" t="inlineStr"/>
-      <c r="H54" s="5" t="inlineStr"/>
-      <c r="I54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="H54" s="5" t="n">
+        <v>0.9708</v>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="J54" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -3940,12 +3940,12 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>STUBSF1</t>
+          <t>STUBSF2</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Stubbo Solar Farm 1</t>
+          <t>Stubbo Solar Farm 2</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3954,7 +3954,7 @@
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E59" s="5" t="inlineStr"/>
       <c r="F59" s="5" t="inlineStr"/>
@@ -3989,12 +3989,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>STUBSF2</t>
+          <t>STUBSF1</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Stubbo Solar Farm 2</t>
+          <t>Stubbo Solar Farm 1</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -4003,7 +4003,7 @@
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="E60" s="5" t="inlineStr"/>
       <c r="F60" s="5" t="inlineStr"/>
@@ -4491,12 +4491,12 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Gunning Wind Farm</t>
+          <t>Cullerin Range Wind Farm</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>46.5</v>
+        <v>30</v>
       </c>
       <c r="E68" s="5" t="n">
         <v>0.9742</v>
@@ -4558,12 +4558,12 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Cullerin Range Wind Farm</t>
+          <t>Gunning Wind Farm</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -4572,7 +4572,7 @@
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>30</v>
+        <v>46.5</v>
       </c>
       <c r="E69" s="5" t="n">
         <v>0.9742</v>
@@ -5238,7 +5238,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>BW03</t>
+          <t>BW04</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>BW04</t>
+          <t>BW03</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -5372,7 +5372,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>BW01</t>
+          <t>BW02</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -5439,7 +5439,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>BW02</t>
+          <t>BW01</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -5506,30 +5506,26 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>GULLRSF1</t>
+          <t>GULLRWF2</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Gullen Range Solar Farm</t>
+          <t>Gullen Range Wind Farm</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D85" s="4" t="n">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="E85" s="5" t="inlineStr"/>
       <c r="F85" s="5" t="inlineStr"/>
-      <c r="G85" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="H85" s="5" t="n">
-        <v>0.9959</v>
-      </c>
+      <c r="G85" s="5" t="inlineStr"/>
+      <c r="H85" s="5" t="inlineStr"/>
       <c r="I85" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -5569,7 +5565,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF2</t>
+          <t>GULLRWF1</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -5583,12 +5579,20 @@
         </is>
       </c>
       <c r="D86" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="E86" s="5" t="inlineStr"/>
-      <c r="F86" s="5" t="inlineStr"/>
-      <c r="G86" s="5" t="inlineStr"/>
-      <c r="H86" s="5" t="inlineStr"/>
+        <v>165</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="F86" s="5" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="G86" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="H86" s="5" t="n">
+        <v>0.9959</v>
+      </c>
       <c r="I86" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -5628,28 +5632,24 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF1</t>
+          <t>GULLRSF1</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Gullen Range Wind Farm</t>
+          <t>Gullen Range Solar Farm</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="D87" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="E87" s="5" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="F87" s="5" t="n">
-        <v>0.9909</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E87" s="5" t="inlineStr"/>
+      <c r="F87" s="5" t="inlineStr"/>
       <c r="G87" s="5" t="n">
         <v>1.001</v>
       </c>
@@ -6120,12 +6120,12 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Wind Farm</t>
+          <t>Capital Wind Farm</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -6134,7 +6134,7 @@
         </is>
       </c>
       <c r="D95" s="4" t="n">
-        <v>48.3</v>
+        <v>140</v>
       </c>
       <c r="E95" s="5" t="n">
         <v>0.9748</v>
@@ -6187,12 +6187,12 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Capital Wind Farm</t>
+          <t>Woodlawn Wind Farm</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -6201,7 +6201,7 @@
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>140</v>
+        <v>48.3</v>
       </c>
       <c r="E96" s="5" t="n">
         <v>0.9748</v>
@@ -6520,12 +6520,12 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MPNL1</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Mt Piper Power Station</t>
+          <t>MT PIPER POWER STATION</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -6534,7 +6534,7 @@
         </is>
       </c>
       <c r="D101" s="4" t="n">
-        <v>700</v>
+        <v>25</v>
       </c>
       <c r="E101" s="5" t="n">
         <v>0.9744</v>
@@ -6654,12 +6654,12 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>MPNL1</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>MT PIPER POWER STATION</t>
+          <t>Mt Piper Power Station</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -6668,7 +6668,7 @@
         </is>
       </c>
       <c r="D103" s="4" t="n">
-        <v>25</v>
+        <v>700</v>
       </c>
       <c r="E103" s="5" t="n">
         <v>0.9744</v>
@@ -6918,7 +6918,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -6926,7 +6926,9 @@
           <t>TUMUT2</t>
         </is>
       </c>
-      <c r="C107" s="3" t="n"/>
+      <c r="C107" s="3" t="n">
+        <v/>
+      </c>
       <c r="D107" s="4" t="n">
         <v>72</v>
       </c>
@@ -6981,17 +6983,19 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
-        </is>
-      </c>
-      <c r="C108" s="3" t="n"/>
+          <t>TUMUT2</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="n">
+        <v/>
+      </c>
       <c r="D108" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E108" s="5" t="n">
         <v>0.9768</v>
@@ -7044,17 +7048,19 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-2</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
-        </is>
-      </c>
-      <c r="C109" s="3" t="n"/>
+          <t>TUMUT2</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="n">
+        <v/>
+      </c>
       <c r="D109" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E109" s="5" t="n">
         <v>0.9768</v>
@@ -7107,17 +7113,19 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1</t>
-        </is>
-      </c>
-      <c r="C110" s="3" t="n"/>
+          <t>TUMUT2</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="n">
+        <v/>
+      </c>
       <c r="D110" s="4" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E110" s="5" t="n">
         <v>0.9768</v>
@@ -7170,17 +7178,19 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-2</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
-        </is>
-      </c>
-      <c r="C111" s="3" t="n"/>
+          <t>TUMUT1</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="n">
+        <v/>
+      </c>
       <c r="D111" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E111" s="5" t="n">
         <v>0.9768</v>
@@ -7233,17 +7243,19 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
-        </is>
-      </c>
-      <c r="C112" s="3" t="n"/>
+          <t>TUMUT1</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="n">
+        <v/>
+      </c>
       <c r="D112" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E112" s="5" t="n">
         <v>0.9768</v>
@@ -7296,17 +7308,19 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="n"/>
+          <t>TUMUT1</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="n">
+        <v/>
+      </c>
       <c r="D113" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E113" s="5" t="n">
         <v>0.9768</v>
@@ -7367,7 +7381,9 @@
           <t>TUMUT1</t>
         </is>
       </c>
-      <c r="C114" s="3" t="n"/>
+      <c r="C114" s="3" t="n">
+        <v/>
+      </c>
       <c r="D114" s="4" t="n">
         <v>82</v>
       </c>
@@ -7715,7 +7731,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -7849,7 +7865,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -7977,12 +7993,12 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>HEZ1</t>
+          <t>ER01</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>Hunter Economic Zone</t>
+          <t>Eraring Power Station</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -7991,29 +8007,41 @@
         </is>
       </c>
       <c r="D124" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="E124" s="5" t="inlineStr"/>
-      <c r="F124" s="5" t="inlineStr"/>
-      <c r="G124" s="5" t="inlineStr"/>
-      <c r="H124" s="5" t="inlineStr"/>
-      <c r="I124" s="5" t="inlineStr"/>
-      <c r="J124" s="5" t="inlineStr"/>
+        <v>720</v>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="F124" s="5" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="G124" s="5" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="H124" s="5" t="n">
+        <v>0.9828</v>
+      </c>
+      <c r="I124" s="5" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="J124" s="5" t="n">
+        <v>0.9835</v>
+      </c>
       <c r="K124" s="5" t="n">
-        <v>0.9897</v>
+        <v>0.9849</v>
       </c>
       <c r="L124" s="5" t="n">
-        <v>0.992</v>
+        <v>0.9865</v>
       </c>
       <c r="M124" s="5" t="n">
-        <v>0.9899</v>
+        <v>0.9848</v>
       </c>
       <c r="N124" s="5" t="n">
-        <v>0.9896</v>
+        <v>0.9855</v>
       </c>
       <c r="O124" s="5" t="inlineStr"/>
       <c r="P124" s="5" t="n">
-        <v>0.9931</v>
+        <v>0.9846</v>
       </c>
       <c r="Q124" s="5" t="inlineStr"/>
       <c r="R124" s="5" t="n">
@@ -8021,10 +8049,10 @@
       </c>
       <c r="S124" s="5" t="inlineStr"/>
       <c r="T124" s="5" t="n">
-        <v>-0.01</v>
+        <v>-0.0015</v>
       </c>
       <c r="U124" s="6" t="n">
-        <v>-1.01</v>
+        <v>-0.15</v>
       </c>
       <c r="V124" s="5" t="inlineStr"/>
       <c r="W124" s="6" t="inlineStr"/>
@@ -8032,7 +8060,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -8046,7 +8074,7 @@
         </is>
       </c>
       <c r="D125" s="4" t="n">
-        <v>41.5</v>
+        <v>720</v>
       </c>
       <c r="E125" s="5" t="n">
         <v>0.9856</v>
@@ -8099,7 +8127,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -8113,7 +8141,7 @@
         </is>
       </c>
       <c r="D126" s="4" t="n">
-        <v>720</v>
+        <v>41.5</v>
       </c>
       <c r="E126" s="5" t="n">
         <v>0.9856</v>
@@ -8166,12 +8194,12 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
+          <t>HEZ1</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>Eraring Power Station</t>
+          <t>Hunter Economic Zone</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -8180,41 +8208,29 @@
         </is>
       </c>
       <c r="D127" s="4" t="n">
-        <v>720</v>
-      </c>
-      <c r="E127" s="5" t="n">
-        <v>0.9856</v>
-      </c>
-      <c r="F127" s="5" t="n">
-        <v>0.9829</v>
-      </c>
-      <c r="G127" s="5" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="H127" s="5" t="n">
-        <v>0.9828</v>
-      </c>
-      <c r="I127" s="5" t="n">
-        <v>0.9836</v>
-      </c>
-      <c r="J127" s="5" t="n">
-        <v>0.9835</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="E127" s="5" t="inlineStr"/>
+      <c r="F127" s="5" t="inlineStr"/>
+      <c r="G127" s="5" t="inlineStr"/>
+      <c r="H127" s="5" t="inlineStr"/>
+      <c r="I127" s="5" t="inlineStr"/>
+      <c r="J127" s="5" t="inlineStr"/>
       <c r="K127" s="5" t="n">
-        <v>0.9849</v>
+        <v>0.9897</v>
       </c>
       <c r="L127" s="5" t="n">
-        <v>0.9865</v>
+        <v>0.992</v>
       </c>
       <c r="M127" s="5" t="n">
-        <v>0.9848</v>
+        <v>0.9899</v>
       </c>
       <c r="N127" s="5" t="n">
-        <v>0.9855</v>
+        <v>0.9896</v>
       </c>
       <c r="O127" s="5" t="inlineStr"/>
       <c r="P127" s="5" t="n">
-        <v>0.9846</v>
+        <v>0.9931</v>
       </c>
       <c r="Q127" s="5" t="inlineStr"/>
       <c r="R127" s="5" t="n">
@@ -8222,10 +8238,10 @@
       </c>
       <c r="S127" s="5" t="inlineStr"/>
       <c r="T127" s="5" t="n">
-        <v>-0.0015</v>
+        <v>-0.01</v>
       </c>
       <c r="U127" s="6" t="n">
-        <v>-0.15</v>
+        <v>-1.01</v>
       </c>
       <c r="V127" s="5" t="inlineStr"/>
       <c r="W127" s="6" t="inlineStr"/>
@@ -8623,7 +8639,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -8690,7 +8706,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -8757,7 +8773,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -8824,7 +8840,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -8891,7 +8907,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -9239,12 +9255,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>JNDABNE1</t>
+          <t>BROWNMT</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Jindabyne Small Hydro Power Station</t>
+          <t>Brown Mountain Hydro Power Station</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -9253,7 +9269,7 @@
         </is>
       </c>
       <c r="D144" s="4" t="n">
-        <v>1.1</v>
+        <v>5</v>
       </c>
       <c r="E144" s="5" t="n">
         <v>0.9762999999999999</v>
@@ -9306,12 +9322,12 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>BROWNMT</t>
+          <t>JNDABNE1</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Brown Mountain Hydro Power Station</t>
+          <t>Jindabyne Small Hydro Power Station</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -9320,7 +9336,7 @@
         </is>
       </c>
       <c r="D145" s="4" t="n">
-        <v>5</v>
+        <v>1.1</v>
       </c>
       <c r="E145" s="5" t="n">
         <v>0.9762999999999999</v>
@@ -9507,12 +9523,12 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>SHOAL1</t>
+          <t>WESTILL1</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Shoalhaven Starches Cogeneration Plant</t>
+          <t>West Illawarra Leagues Club Plant</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -9521,16 +9537,32 @@
         </is>
       </c>
       <c r="D148" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="E148" s="5" t="inlineStr"/>
-      <c r="F148" s="5" t="inlineStr"/>
-      <c r="G148" s="5" t="inlineStr"/>
-      <c r="H148" s="5" t="inlineStr"/>
-      <c r="I148" s="5" t="inlineStr"/>
-      <c r="J148" s="5" t="inlineStr"/>
-      <c r="K148" s="5" t="inlineStr"/>
-      <c r="L148" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E148" s="5" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="F148" s="5" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="G148" s="5" t="n">
+        <v>1.0023</v>
+      </c>
+      <c r="H148" s="5" t="n">
+        <v>1.0037</v>
+      </c>
+      <c r="I148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="J148" s="5" t="n">
+        <v>0.9967</v>
+      </c>
+      <c r="K148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="L148" s="5" t="n">
+        <v>0.9933999999999999</v>
+      </c>
       <c r="M148" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -9558,12 +9590,12 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>WESTILL1</t>
+          <t>SHOAL1</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>West Illawarra Leagues Club Plant</t>
+          <t>Shoalhaven Starches Cogeneration Plant</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -9572,32 +9604,16 @@
         </is>
       </c>
       <c r="D149" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E149" s="5" t="n">
-        <v>0.9916</v>
-      </c>
-      <c r="F149" s="5" t="n">
-        <v>0.9986</v>
-      </c>
-      <c r="G149" s="5" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="H149" s="5" t="n">
-        <v>1.0037</v>
-      </c>
-      <c r="I149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="J149" s="5" t="n">
-        <v>0.9967</v>
-      </c>
-      <c r="K149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="L149" s="5" t="n">
-        <v>0.9933999999999999</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E149" s="5" t="inlineStr"/>
+      <c r="F149" s="5" t="inlineStr"/>
+      <c r="G149" s="5" t="inlineStr"/>
+      <c r="H149" s="5" t="inlineStr"/>
+      <c r="I149" s="5" t="inlineStr"/>
+      <c r="J149" s="5" t="inlineStr"/>
+      <c r="K149" s="5" t="inlineStr"/>
+      <c r="L149" s="5" t="inlineStr"/>
       <c r="M149" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -9822,12 +9838,12 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>Wyangala B Power Station</t>
+          <t>Wyangala A Power Station</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
@@ -9836,7 +9852,7 @@
         </is>
       </c>
       <c r="D153" s="4" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E153" s="5" t="n">
         <v>1.0099</v>
@@ -9889,12 +9905,12 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>Wyangala A Power Station</t>
+          <t>Wyangala B Power Station</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -9903,7 +9919,7 @@
         </is>
       </c>
       <c r="D154" s="4" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E154" s="5" t="n">
         <v>1.0099</v>
@@ -10299,7 +10315,9 @@
           <t>NSW1 Dummy Generator</t>
         </is>
       </c>
-      <c r="C160" s="3" t="n"/>
+      <c r="C160" s="3" t="n">
+        <v/>
+      </c>
       <c r="D160" s="4" t="n">
         <v>3000</v>
       </c>
@@ -10622,12 +10640,12 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>SMTHBES1</t>
+          <t>WALGRV1</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Smithfield Battery Energy Storage System, Units 1 - 36</t>
+          <t>Wallgrove BESS 1</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -10636,7 +10654,7 @@
         </is>
       </c>
       <c r="D165" s="4" t="n">
-        <v>69.40000000000001</v>
+        <v>50</v>
       </c>
       <c r="E165" s="5" t="inlineStr"/>
       <c r="F165" s="5" t="inlineStr"/>
@@ -10644,28 +10662,38 @@
       <c r="H165" s="5" t="inlineStr"/>
       <c r="I165" s="5" t="inlineStr"/>
       <c r="J165" s="5" t="inlineStr"/>
-      <c r="K165" s="5" t="inlineStr"/>
-      <c r="L165" s="5" t="inlineStr"/>
-      <c r="M165" s="5" t="inlineStr"/>
-      <c r="N165" s="5" t="inlineStr"/>
-      <c r="O165" s="5" t="inlineStr"/>
+      <c r="K165" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="L165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="M165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="N165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="O165" s="5" t="n">
+        <v>1.0009</v>
+      </c>
       <c r="P165" s="5" t="n">
-        <v>1.0016</v>
+        <v>1.0018</v>
       </c>
       <c r="Q165" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0015</v>
       </c>
       <c r="R165" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="S165" s="5" t="n">
-        <v>1.0019</v>
+        <v>1.0017</v>
       </c>
       <c r="T165" s="5" t="n">
-        <v>0.0001</v>
+        <v>-0.0001</v>
       </c>
       <c r="U165" s="6" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="V165" s="5" t="n">
         <v>0.0002</v>
@@ -10677,12 +10705,12 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>WALGRV1</t>
+          <t>SMTHBES1</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>Wallgrove BESS 1</t>
+          <t>Smithfield Battery Energy Storage System, Units 1 - 36</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -10691,7 +10719,7 @@
         </is>
       </c>
       <c r="D166" s="4" t="n">
-        <v>50</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="E166" s="5" t="inlineStr"/>
       <c r="F166" s="5" t="inlineStr"/>
@@ -10699,38 +10727,28 @@
       <c r="H166" s="5" t="inlineStr"/>
       <c r="I166" s="5" t="inlineStr"/>
       <c r="J166" s="5" t="inlineStr"/>
-      <c r="K166" s="5" t="n">
-        <v>1.0011</v>
-      </c>
-      <c r="L166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="M166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="N166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="O166" s="5" t="n">
-        <v>1.0009</v>
-      </c>
+      <c r="K166" s="5" t="inlineStr"/>
+      <c r="L166" s="5" t="inlineStr"/>
+      <c r="M166" s="5" t="inlineStr"/>
+      <c r="N166" s="5" t="inlineStr"/>
+      <c r="O166" s="5" t="inlineStr"/>
       <c r="P166" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0016</v>
       </c>
       <c r="Q166" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0017</v>
       </c>
       <c r="R166" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="S166" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0019</v>
       </c>
       <c r="T166" s="5" t="n">
-        <v>-0.0001</v>
+        <v>0.0001</v>
       </c>
       <c r="U166" s="6" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="V166" s="5" t="n">
         <v>0.0002</v>
@@ -10809,21 +10827,21 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>Taralga Wind Farm</t>
+          <t>Woodlawn Bioreactor Energy Generation Station</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D168" s="4" t="n">
-        <v>106.8</v>
+        <v>7</v>
       </c>
       <c r="E168" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -10876,21 +10894,21 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>Woodlawn Bioreactor Energy Generation Station</t>
+          <t>Taralga Wind Farm</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Wind</t>
         </is>
       </c>
       <c r="D169" s="4" t="n">
-        <v>7</v>
+        <v>106.8</v>
       </c>
       <c r="E169" s="5" t="n">
         <v>0.9844000000000001</v>
@@ -11061,7 +11079,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -11069,7 +11087,9 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C172" s="3" t="n"/>
+      <c r="C172" s="3" t="n">
+        <v/>
+      </c>
       <c r="D172" s="4" t="n">
         <v>250</v>
       </c>
@@ -11124,7 +11144,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -11132,7 +11152,9 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C173" s="3" t="n"/>
+      <c r="C173" s="3" t="n">
+        <v/>
+      </c>
       <c r="D173" s="4" t="n">
         <v>250</v>
       </c>
@@ -11187,7 +11209,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -11195,7 +11217,9 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C174" s="3" t="n"/>
+      <c r="C174" s="3" t="n">
+        <v/>
+      </c>
       <c r="D174" s="4" t="n">
         <v>250</v>
       </c>
@@ -11250,7 +11274,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -11258,7 +11282,9 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C175" s="3" t="n"/>
+      <c r="C175" s="3" t="n">
+        <v/>
+      </c>
       <c r="D175" s="4" t="n">
         <v>250</v>
       </c>
@@ -11313,7 +11339,7 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -11321,7 +11347,9 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C176" s="3" t="n"/>
+      <c r="C176" s="3" t="n">
+        <v/>
+      </c>
       <c r="D176" s="4" t="n">
         <v>250</v>
       </c>
@@ -11376,7 +11404,7 @@
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -11384,7 +11412,9 @@
           <t>TUMUT3</t>
         </is>
       </c>
-      <c r="C177" s="3" t="n"/>
+      <c r="C177" s="3" t="n">
+        <v/>
+      </c>
       <c r="D177" s="4" t="n">
         <v>250</v>
       </c>
@@ -11447,7 +11477,9 @@
           <t>Redbank Power Station</t>
         </is>
       </c>
-      <c r="C178" s="3" t="n"/>
+      <c r="C178" s="3" t="n">
+        <v/>
+      </c>
       <c r="D178" s="4" t="n">
         <v>150</v>
       </c>
@@ -11662,12 +11694,12 @@
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
+          <t>AGLSITA1</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>West Nowra Landfill Gas Power Generation Facility</t>
+          <t>AGL KEMPS CREEK</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
@@ -11678,26 +11710,24 @@
       <c r="D183" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E183" s="5" t="n">
-        <v>0.9916</v>
-      </c>
+      <c r="E183" s="5" t="inlineStr"/>
       <c r="F183" s="5" t="n">
-        <v>0.9986</v>
+        <v>1.0019</v>
       </c>
       <c r="G183" s="5" t="n">
-        <v>1.0023</v>
+        <v>1.0022</v>
       </c>
       <c r="H183" s="5" t="n">
-        <v>1.0037</v>
+        <v>1.0024</v>
       </c>
       <c r="I183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0009</v>
       </c>
       <c r="J183" s="5" t="n">
-        <v>0.9967</v>
+        <v>1.0012</v>
       </c>
       <c r="K183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0015</v>
       </c>
       <c r="L183" s="5" t="inlineStr"/>
       <c r="M183" s="5" t="inlineStr"/>
@@ -11715,12 +11745,12 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>AGLNOW1</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>TERALBA POWER STATION</t>
+          <t>West Nowra Landfill Gas Power Generation Facility</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
@@ -11729,28 +11759,28 @@
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>0.9926</v>
+        <v>0.9916</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9986</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>0.9892</v>
+        <v>1.0023</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>0.9901</v>
+        <v>1.0037</v>
       </c>
       <c r="I184" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9929</v>
       </c>
       <c r="J184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9967</v>
       </c>
       <c r="K184" s="5" t="n">
-        <v>0.9917</v>
+        <v>0.9929</v>
       </c>
       <c r="L184" s="5" t="inlineStr"/>
       <c r="M184" s="5" t="inlineStr"/>
@@ -11768,42 +11798,42 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Liddell Power Station</t>
+          <t>Kincumber Landfill Site</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>Fossil</t>
+          <t>Other Renewable</t>
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="I185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="J185" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="L185" s="5" t="inlineStr"/>
       <c r="M185" s="5" t="inlineStr"/>
@@ -11821,42 +11851,42 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>Kincumber Landfill Site</t>
+          <t>Liddell Power Station</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>Other Renewable</t>
+          <t>Fossil</t>
         </is>
       </c>
       <c r="D186" s="4" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9676</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9593</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9509</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9537</v>
       </c>
       <c r="I186" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9593</v>
       </c>
       <c r="J186" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9631</v>
       </c>
       <c r="K186" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9628</v>
       </c>
       <c r="L186" s="5" t="inlineStr"/>
       <c r="M186" s="5" t="inlineStr"/>
@@ -11927,12 +11957,12 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>Woy Woy Landfill Site</t>
+          <t>TERALBA POWER STATION</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -11941,28 +11971,28 @@
         </is>
       </c>
       <c r="D188" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9926</v>
       </c>
       <c r="F188" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9907</v>
       </c>
       <c r="G188" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9892</v>
       </c>
       <c r="H188" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9901</v>
       </c>
       <c r="I188" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="J188" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9907</v>
       </c>
       <c r="K188" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9917</v>
       </c>
       <c r="L188" s="5" t="inlineStr"/>
       <c r="M188" s="5" t="inlineStr"/>
@@ -11980,12 +12010,12 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>AGLSITA1</t>
+          <t>WOYWOY1</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>AGL KEMPS CREEK</t>
+          <t>Woy Woy Landfill Site</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
@@ -11996,24 +12026,26 @@
       <c r="D189" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E189" s="5" t="inlineStr"/>
+      <c r="E189" s="5" t="n">
+        <v>1.0017</v>
+      </c>
       <c r="F189" s="5" t="n">
+        <v>1.0015</v>
+      </c>
+      <c r="G189" s="5" t="n">
+        <v>1.0008</v>
+      </c>
+      <c r="H189" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="I189" s="5" t="n">
+        <v>1.0036</v>
+      </c>
+      <c r="J189" s="5" t="n">
         <v>1.0019</v>
       </c>
-      <c r="G189" s="5" t="n">
-        <v>1.0022</v>
-      </c>
-      <c r="H189" s="5" t="n">
-        <v>1.0024</v>
-      </c>
-      <c r="I189" s="5" t="n">
-        <v>1.0009</v>
-      </c>
-      <c r="J189" s="5" t="n">
-        <v>1.0012</v>
-      </c>
       <c r="K189" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0037</v>
       </c>
       <c r="L189" s="5" t="inlineStr"/>
       <c r="M189" s="5" t="inlineStr"/>
@@ -12031,7 +12063,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>LD04</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -12086,7 +12118,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD04</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
@@ -12141,7 +12173,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -12492,14 +12524,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>WRWF1</t>
+          <t>WRSF1</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr"/>
       <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="n">
-        <v>0.8468</v>
-      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -12534,12 +12564,14 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>WRSF1</t>
+          <t>WRWF1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr"/>
       <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="n">
+        <v>0.8468</v>
+      </c>
       <c r="E5" s="5" t="n">
         <v>0.8427</v>
       </c>
@@ -13158,7 +13190,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>WSTWYSF1</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr"/>
@@ -13166,12 +13198,8 @@
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="5" t="n">
-        <v>0.9645</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>0.8799</v>
-      </c>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
       <c r="I21" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -13194,7 +13222,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr"/>
@@ -13202,7 +13230,9 @@
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr"/>
       <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="n">
+        <v>0.9645</v>
+      </c>
       <c r="H22" s="5" t="n">
         <v>0.8799</v>
       </c>
@@ -13228,7 +13258,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>WSTWYSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr"/>
@@ -13260,7 +13290,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr"/>
@@ -13269,7 +13299,9 @@
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="n">
+        <v>0.8799</v>
+      </c>
       <c r="I24" s="5" t="n">
         <v>0.9059</v>
       </c>
@@ -13376,7 +13408,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF2</t>
+          <t>NEWENSF1</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr"/>
@@ -13408,7 +13440,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>NEWENSF1</t>
+          <t>NEWENSF2</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr"/>
@@ -13440,7 +13472,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>CRWASF1</t>
+          <t>MULWASF1</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr"/>
@@ -13448,24 +13480,14 @@
       <c r="D30" s="5" t="inlineStr"/>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="n">
-        <v>0.9497</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>0.8813</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>0.9242</v>
-      </c>
-      <c r="J30" s="5" t="n">
-        <v>0.9365</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>0.8979</v>
-      </c>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="inlineStr"/>
       <c r="L30" s="5" t="inlineStr"/>
       <c r="M30" s="5" t="n">
-        <v>0.9355</v>
+        <v>0.9345</v>
       </c>
       <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="n">
@@ -13476,7 +13498,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>MULWASF1</t>
+          <t>CRWASF1</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr"/>
@@ -13484,14 +13506,24 @@
       <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr"/>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
-      <c r="K31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="n">
+        <v>0.9497</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0.9242</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0.9365</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.8979</v>
+      </c>
       <c r="L31" s="5" t="inlineStr"/>
       <c r="M31" s="5" t="n">
-        <v>0.9345</v>
+        <v>0.9355</v>
       </c>
       <c r="N31" s="5" t="inlineStr"/>
       <c r="O31" s="5" t="n">
@@ -13788,7 +13820,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>NESBESS1</t>
+          <t>NESBESS2</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr"/>
@@ -13818,7 +13850,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NESBESS2</t>
+          <t>NESBESS1</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr"/>
@@ -13928,7 +13960,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ14</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
@@ -13974,7 +14006,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ13</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
@@ -14020,7 +14052,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>URANQ13</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
@@ -14066,7 +14098,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>URANQ14</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
@@ -14188,16 +14220,14 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>NEVERSF1</t>
+          <t>WELLSF1</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr"/>
       <c r="C50" s="5" t="inlineStr"/>
       <c r="D50" s="5" t="inlineStr"/>
       <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="n">
-        <v>0.9582000000000001</v>
-      </c>
+      <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -14226,7 +14256,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>SKSF1</t>
+          <t>NASF1</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr"/>
@@ -14268,17 +14298,13 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>NASF1</t>
+          <t>NEVERSF1</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr"/>
       <c r="C52" s="5" t="inlineStr"/>
-      <c r="D52" s="5" t="n">
-        <v>0.9714</v>
-      </c>
-      <c r="E52" s="5" t="n">
-        <v>0.9708</v>
-      </c>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr"/>
       <c r="F52" s="5" t="n">
         <v>0.9582000000000001</v>
       </c>
@@ -14356,14 +14382,20 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>WELLSF1</t>
+          <t>SKSF1</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr"/>
       <c r="C54" s="5" t="inlineStr"/>
-      <c r="D54" s="5" t="inlineStr"/>
-      <c r="E54" s="5" t="inlineStr"/>
-      <c r="F54" s="5" t="inlineStr"/>
+      <c r="D54" s="5" t="n">
+        <v>0.9714</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>0.9708</v>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>0.9582000000000001</v>
+      </c>
       <c r="G54" s="5" t="n">
         <v>0.9471000000000001</v>
       </c>
@@ -14540,7 +14572,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>STUBSF1</t>
+          <t>STUBSF2</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr"/>
@@ -14568,7 +14600,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>STUBSF2</t>
+          <t>STUBSF1</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr"/>
@@ -14898,7 +14930,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>GUNNING1</t>
+          <t>CULLRGWF</t>
         </is>
       </c>
       <c r="B68" s="5" t="n">
@@ -14944,7 +14976,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>CULLRGWF</t>
+          <t>GUNNING1</t>
         </is>
       </c>
       <c r="B69" s="5" t="n">
@@ -15372,7 +15404,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>BW03</t>
+          <t>BW04</t>
         </is>
       </c>
       <c r="B81" s="5" t="n">
@@ -15418,7 +15450,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>BW04</t>
+          <t>BW03</t>
         </is>
       </c>
       <c r="B82" s="5" t="n">
@@ -15464,7 +15496,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>BW01</t>
+          <t>BW02</t>
         </is>
       </c>
       <c r="B83" s="5" t="n">
@@ -15510,7 +15542,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>BW02</t>
+          <t>BW01</t>
         </is>
       </c>
       <c r="B84" s="5" t="n">
@@ -15556,17 +15588,13 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>GULLRSF1</t>
+          <t>GULLRWF2</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr"/>
       <c r="C85" s="5" t="inlineStr"/>
-      <c r="D85" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="E85" s="5" t="n">
-        <v>0.9959</v>
-      </c>
+      <c r="D85" s="5" t="inlineStr"/>
+      <c r="E85" s="5" t="inlineStr"/>
       <c r="F85" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -15598,13 +15626,21 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF2</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="inlineStr"/>
-      <c r="C86" s="5" t="inlineStr"/>
-      <c r="D86" s="5" t="inlineStr"/>
-      <c r="E86" s="5" t="inlineStr"/>
+          <t>GULLRWF1</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="C86" s="5" t="n">
+        <v>0.9909</v>
+      </c>
+      <c r="D86" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v>0.9959</v>
+      </c>
       <c r="F86" s="5" t="n">
         <v>0.9694</v>
       </c>
@@ -15636,15 +15672,11 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>GULLRWF1</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="C87" s="5" t="n">
-        <v>0.9909</v>
-      </c>
+          <t>GULLRSF1</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr"/>
+      <c r="C87" s="5" t="inlineStr"/>
       <c r="D87" s="5" t="n">
         <v>1.001</v>
       </c>
@@ -15956,7 +15988,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>WOODLWN1</t>
+          <t>CAPTL_WF</t>
         </is>
       </c>
       <c r="B95" s="5" t="n">
@@ -16002,7 +16034,7 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>CAPTL_WF</t>
+          <t>WOODLWN1</t>
         </is>
       </c>
       <c r="B96" s="5" t="n">
@@ -16230,7 +16262,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>MP1</t>
+          <t>MPNL1</t>
         </is>
       </c>
       <c r="B101" s="5" t="n">
@@ -16322,7 +16354,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>MPNL1</t>
+          <t>MP1</t>
         </is>
       </c>
       <c r="B103" s="5" t="n">
@@ -16498,7 +16530,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-1</t>
+          <t>TUMUT2-4</t>
         </is>
       </c>
       <c r="B107" s="5" t="n">
@@ -16544,7 +16576,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-4</t>
+          <t>TUMUT2-3</t>
         </is>
       </c>
       <c r="B108" s="5" t="n">
@@ -16590,7 +16622,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-2</t>
+          <t>TUMUT2-2</t>
         </is>
       </c>
       <c r="B109" s="5" t="n">
@@ -16636,7 +16668,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>TUMUT1-3</t>
+          <t>TUMUT2-1</t>
         </is>
       </c>
       <c r="B110" s="5" t="n">
@@ -16682,7 +16714,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-2</t>
+          <t>TUMUT1-4</t>
         </is>
       </c>
       <c r="B111" s="5" t="n">
@@ -16728,7 +16760,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-4</t>
+          <t>TUMUT1-3</t>
         </is>
       </c>
       <c r="B112" s="5" t="n">
@@ -16774,7 +16806,7 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>TUMUT2-3</t>
+          <t>TUMUT1-2</t>
         </is>
       </c>
       <c r="B113" s="5" t="n">
@@ -17046,7 +17078,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>CG3</t>
+          <t>CG2</t>
         </is>
       </c>
       <c r="B120" s="5" t="n">
@@ -17138,7 +17170,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>CG2</t>
+          <t>CG3</t>
         </is>
       </c>
       <c r="B122" s="5" t="n">
@@ -17220,30 +17252,42 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>HEZ1</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="inlineStr"/>
-      <c r="C124" s="5" t="inlineStr"/>
-      <c r="D124" s="5" t="inlineStr"/>
-      <c r="E124" s="5" t="inlineStr"/>
-      <c r="F124" s="5" t="inlineStr"/>
-      <c r="G124" s="5" t="inlineStr"/>
+          <t>ER01</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="C124" s="5" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="D124" s="5" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>0.9828</v>
+      </c>
+      <c r="F124" s="5" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="G124" s="5" t="n">
+        <v>0.9835</v>
+      </c>
       <c r="H124" s="5" t="n">
-        <v>0.9897</v>
+        <v>0.9849</v>
       </c>
       <c r="I124" s="5" t="n">
-        <v>0.992</v>
+        <v>0.9865</v>
       </c>
       <c r="J124" s="5" t="n">
-        <v>0.9899</v>
+        <v>0.9848</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>0.9896</v>
+        <v>0.9855</v>
       </c>
       <c r="L124" s="5" t="inlineStr"/>
       <c r="M124" s="5" t="n">
-        <v>0.9931</v>
+        <v>0.9846</v>
       </c>
       <c r="N124" s="5" t="inlineStr"/>
       <c r="O124" s="5" t="n">
@@ -17254,7 +17298,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>ERGT01</t>
+          <t>ER02</t>
         </is>
       </c>
       <c r="B125" s="5" t="n">
@@ -17300,7 +17344,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>ER02</t>
+          <t>ERGT01</t>
         </is>
       </c>
       <c r="B126" s="5" t="n">
@@ -17346,42 +17390,30 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>ER01</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="n">
-        <v>0.9856</v>
-      </c>
-      <c r="C127" s="5" t="n">
-        <v>0.9829</v>
-      </c>
-      <c r="D127" s="5" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="E127" s="5" t="n">
-        <v>0.9828</v>
-      </c>
-      <c r="F127" s="5" t="n">
-        <v>0.9836</v>
-      </c>
-      <c r="G127" s="5" t="n">
-        <v>0.9835</v>
-      </c>
+          <t>HEZ1</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr"/>
+      <c r="C127" s="5" t="inlineStr"/>
+      <c r="D127" s="5" t="inlineStr"/>
+      <c r="E127" s="5" t="inlineStr"/>
+      <c r="F127" s="5" t="inlineStr"/>
+      <c r="G127" s="5" t="inlineStr"/>
       <c r="H127" s="5" t="n">
-        <v>0.9849</v>
+        <v>0.9897</v>
       </c>
       <c r="I127" s="5" t="n">
-        <v>0.9865</v>
+        <v>0.992</v>
       </c>
       <c r="J127" s="5" t="n">
-        <v>0.9848</v>
+        <v>0.9899</v>
       </c>
       <c r="K127" s="5" t="n">
-        <v>0.9855</v>
+        <v>0.9896</v>
       </c>
       <c r="L127" s="5" t="inlineStr"/>
       <c r="M127" s="5" t="n">
-        <v>0.9846</v>
+        <v>0.9931</v>
       </c>
       <c r="N127" s="5" t="inlineStr"/>
       <c r="O127" s="5" t="n">
@@ -17648,7 +17680,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>VP5</t>
+          <t>VP6</t>
         </is>
       </c>
       <c r="B134" s="5" t="n">
@@ -17694,7 +17726,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>VP6</t>
+          <t>VP5</t>
         </is>
       </c>
       <c r="B135" s="5" t="n">
@@ -17740,7 +17772,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B136" s="5" t="n">
@@ -17786,7 +17818,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B137" s="5" t="n">
@@ -17832,7 +17864,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B138" s="5" t="n">
@@ -18054,7 +18086,7 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>JNDABNE1</t>
+          <t>BROWNMT</t>
         </is>
       </c>
       <c r="B144" s="5" t="n">
@@ -18100,7 +18132,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>BROWNMT</t>
+          <t>JNDABNE1</t>
         </is>
       </c>
       <c r="B145" s="5" t="n">
@@ -18238,17 +18270,33 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>SHOAL1</t>
-        </is>
-      </c>
-      <c r="B148" s="5" t="inlineStr"/>
-      <c r="C148" s="5" t="inlineStr"/>
-      <c r="D148" s="5" t="inlineStr"/>
-      <c r="E148" s="5" t="inlineStr"/>
-      <c r="F148" s="5" t="inlineStr"/>
-      <c r="G148" s="5" t="inlineStr"/>
-      <c r="H148" s="5" t="inlineStr"/>
-      <c r="I148" s="5" t="inlineStr"/>
+          <t>WESTILL1</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="C148" s="5" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="D148" s="5" t="n">
+        <v>1.0023</v>
+      </c>
+      <c r="E148" s="5" t="n">
+        <v>1.0037</v>
+      </c>
+      <c r="F148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="G148" s="5" t="n">
+        <v>0.9967</v>
+      </c>
+      <c r="H148" s="5" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="I148" s="5" t="n">
+        <v>0.9933999999999999</v>
+      </c>
       <c r="J148" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -18268,33 +18316,17 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>WESTILL1</t>
-        </is>
-      </c>
-      <c r="B149" s="5" t="n">
-        <v>0.9916</v>
-      </c>
-      <c r="C149" s="5" t="n">
-        <v>0.9986</v>
-      </c>
-      <c r="D149" s="5" t="n">
-        <v>1.0023</v>
-      </c>
-      <c r="E149" s="5" t="n">
-        <v>1.0037</v>
-      </c>
-      <c r="F149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="G149" s="5" t="n">
-        <v>0.9967</v>
-      </c>
-      <c r="H149" s="5" t="n">
-        <v>0.9929</v>
-      </c>
-      <c r="I149" s="5" t="n">
-        <v>0.9933999999999999</v>
-      </c>
+          <t>SHOAL1</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr"/>
+      <c r="C149" s="5" t="inlineStr"/>
+      <c r="D149" s="5" t="inlineStr"/>
+      <c r="E149" s="5" t="inlineStr"/>
+      <c r="F149" s="5" t="inlineStr"/>
+      <c r="G149" s="5" t="inlineStr"/>
+      <c r="H149" s="5" t="inlineStr"/>
+      <c r="I149" s="5" t="inlineStr"/>
       <c r="J149" s="5" t="n">
         <v>0.9888</v>
       </c>
@@ -18444,7 +18476,7 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>WYANGALB</t>
+          <t>WYANGALA</t>
         </is>
       </c>
       <c r="B153" s="5" t="n">
@@ -18490,7 +18522,7 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>WYANGALA</t>
+          <t>WYANGALB</t>
         </is>
       </c>
       <c r="B154" s="5" t="n">
@@ -18996,7 +19028,7 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>SMTHBES1</t>
+          <t>WALGRV1</t>
         </is>
       </c>
       <c r="B165" s="5" t="inlineStr"/>
@@ -19005,28 +19037,38 @@
       <c r="E165" s="5" t="inlineStr"/>
       <c r="F165" s="5" t="inlineStr"/>
       <c r="G165" s="5" t="inlineStr"/>
-      <c r="H165" s="5" t="inlineStr"/>
-      <c r="I165" s="5" t="inlineStr"/>
-      <c r="J165" s="5" t="inlineStr"/>
-      <c r="K165" s="5" t="inlineStr"/>
-      <c r="L165" s="5" t="inlineStr"/>
+      <c r="H165" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="I165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="J165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="K165" s="5" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="L165" s="5" t="n">
+        <v>1.0009</v>
+      </c>
       <c r="M165" s="5" t="n">
-        <v>1.0016</v>
+        <v>1.0018</v>
       </c>
       <c r="N165" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0015</v>
       </c>
       <c r="O165" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="P165" s="5" t="n">
-        <v>1.0019</v>
+        <v>1.0017</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>WALGRV1</t>
+          <t>SMTHBES1</t>
         </is>
       </c>
       <c r="B166" s="5" t="inlineStr"/>
@@ -19035,32 +19077,22 @@
       <c r="E166" s="5" t="inlineStr"/>
       <c r="F166" s="5" t="inlineStr"/>
       <c r="G166" s="5" t="inlineStr"/>
-      <c r="H166" s="5" t="n">
-        <v>1.0011</v>
-      </c>
-      <c r="I166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="J166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="K166" s="5" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="L166" s="5" t="n">
-        <v>1.0009</v>
-      </c>
+      <c r="H166" s="5" t="inlineStr"/>
+      <c r="I166" s="5" t="inlineStr"/>
+      <c r="J166" s="5" t="inlineStr"/>
+      <c r="K166" s="5" t="inlineStr"/>
+      <c r="L166" s="5" t="inlineStr"/>
       <c r="M166" s="5" t="n">
-        <v>1.0018</v>
+        <v>1.0016</v>
       </c>
       <c r="N166" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0017</v>
       </c>
       <c r="O166" s="5" t="n">
         <v>1.0017</v>
       </c>
       <c r="P166" s="5" t="n">
-        <v>1.0017</v>
+        <v>1.0019</v>
       </c>
     </row>
     <row r="167">
@@ -19112,7 +19144,7 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>TARALGA1</t>
+          <t>WDLNGN01</t>
         </is>
       </c>
       <c r="B168" s="5" t="n">
@@ -19158,7 +19190,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>WDLNGN01</t>
+          <t>TARALGA1</t>
         </is>
       </c>
       <c r="B169" s="5" t="n">
@@ -19280,7 +19312,7 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-1</t>
+          <t>TUMUT3-6</t>
         </is>
       </c>
       <c r="B172" s="5" t="n">
@@ -19326,7 +19358,7 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-2</t>
+          <t>TUMUT3-5</t>
         </is>
       </c>
       <c r="B173" s="5" t="n">
@@ -19372,7 +19404,7 @@
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-3</t>
+          <t>TUMUT3-4</t>
         </is>
       </c>
       <c r="B174" s="5" t="n">
@@ -19418,7 +19450,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-5</t>
+          <t>TUMUT3-3</t>
         </is>
       </c>
       <c r="B175" s="5" t="n">
@@ -19464,7 +19496,7 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-6</t>
+          <t>TUMUT3-2</t>
         </is>
       </c>
       <c r="B176" s="5" t="n">
@@ -19510,7 +19542,7 @@
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>TUMUT3-4</t>
+          <t>TUMUT3-1</t>
         </is>
       </c>
       <c r="B177" s="5" t="n">
@@ -19698,29 +19730,27 @@
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AGLNOW1</t>
-        </is>
-      </c>
-      <c r="B183" s="5" t="n">
-        <v>0.9916</v>
-      </c>
+          <t>AGLSITA1</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr"/>
       <c r="C183" s="5" t="n">
-        <v>0.9986</v>
+        <v>1.0019</v>
       </c>
       <c r="D183" s="5" t="n">
-        <v>1.0023</v>
+        <v>1.0022</v>
       </c>
       <c r="E183" s="5" t="n">
-        <v>1.0037</v>
+        <v>1.0024</v>
       </c>
       <c r="F183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0009</v>
       </c>
       <c r="G183" s="5" t="n">
-        <v>0.9967</v>
+        <v>1.0012</v>
       </c>
       <c r="H183" s="5" t="n">
-        <v>0.9929</v>
+        <v>1.0015</v>
       </c>
       <c r="I183" s="5" t="inlineStr"/>
       <c r="J183" s="5" t="inlineStr"/>
@@ -19734,29 +19764,29 @@
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>TERALBA</t>
+          <t>AGLNOW1</t>
         </is>
       </c>
       <c r="B184" s="5" t="n">
-        <v>0.9926</v>
+        <v>0.9916</v>
       </c>
       <c r="C184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9986</v>
       </c>
       <c r="D184" s="5" t="n">
-        <v>0.9892</v>
+        <v>1.0023</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>0.9901</v>
+        <v>1.0037</v>
       </c>
       <c r="F184" s="5" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9929</v>
       </c>
       <c r="G184" s="5" t="n">
-        <v>0.9907</v>
+        <v>0.9967</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>0.9917</v>
+        <v>0.9929</v>
       </c>
       <c r="I184" s="5" t="inlineStr"/>
       <c r="J184" s="5" t="inlineStr"/>
@@ -19770,29 +19800,29 @@
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>LD03</t>
+          <t>KINCUM1</t>
         </is>
       </c>
       <c r="B185" s="5" t="n">
-        <v>0.9676</v>
+        <v>1.0017</v>
       </c>
       <c r="C185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0015</v>
       </c>
       <c r="D185" s="5" t="n">
-        <v>0.9509</v>
+        <v>1.0008</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>0.9537</v>
+        <v>1.0011</v>
       </c>
       <c r="F185" s="5" t="n">
-        <v>0.9593</v>
+        <v>1.0036</v>
       </c>
       <c r="G185" s="5" t="n">
-        <v>0.9631</v>
+        <v>1.0019</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>0.9628</v>
+        <v>1.0037</v>
       </c>
       <c r="I185" s="5" t="inlineStr"/>
       <c r="J185" s="5" t="inlineStr"/>
@@ -19806,29 +19836,29 @@
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>KINCUM1</t>
+          <t>LD03</t>
         </is>
       </c>
       <c r="B186" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9676</v>
       </c>
       <c r="C186" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9593</v>
       </c>
       <c r="D186" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9509</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9537</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9593</v>
       </c>
       <c r="G186" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9631</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9628</v>
       </c>
       <c r="I186" s="5" t="inlineStr"/>
       <c r="J186" s="5" t="inlineStr"/>
@@ -19878,29 +19908,29 @@
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>WOYWOY1</t>
+          <t>TERALBA</t>
         </is>
       </c>
       <c r="B188" s="5" t="n">
-        <v>1.0017</v>
+        <v>0.9926</v>
       </c>
       <c r="C188" s="5" t="n">
-        <v>1.0015</v>
+        <v>0.9907</v>
       </c>
       <c r="D188" s="5" t="n">
-        <v>1.0008</v>
+        <v>0.9892</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>1.0011</v>
+        <v>0.9901</v>
       </c>
       <c r="F188" s="5" t="n">
-        <v>1.0036</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="G188" s="5" t="n">
-        <v>1.0019</v>
+        <v>0.9907</v>
       </c>
       <c r="H188" s="5" t="n">
-        <v>1.0037</v>
+        <v>0.9917</v>
       </c>
       <c r="I188" s="5" t="inlineStr"/>
       <c r="J188" s="5" t="inlineStr"/>
@@ -19914,27 +19944,29 @@
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>AGLSITA1</t>
-        </is>
-      </c>
-      <c r="B189" s="5" t="inlineStr"/>
+          <t>WOYWOY1</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="n">
+        <v>1.0017</v>
+      </c>
       <c r="C189" s="5" t="n">
+        <v>1.0015</v>
+      </c>
+      <c r="D189" s="5" t="n">
+        <v>1.0008</v>
+      </c>
+      <c r="E189" s="5" t="n">
+        <v>1.0011</v>
+      </c>
+      <c r="F189" s="5" t="n">
+        <v>1.0036</v>
+      </c>
+      <c r="G189" s="5" t="n">
         <v>1.0019</v>
       </c>
-      <c r="D189" s="5" t="n">
-        <v>1.0022</v>
-      </c>
-      <c r="E189" s="5" t="n">
-        <v>1.0024</v>
-      </c>
-      <c r="F189" s="5" t="n">
-        <v>1.0009</v>
-      </c>
-      <c r="G189" s="5" t="n">
-        <v>1.0012</v>
-      </c>
       <c r="H189" s="5" t="n">
-        <v>1.0015</v>
+        <v>1.0037</v>
       </c>
       <c r="I189" s="5" t="inlineStr"/>
       <c r="J189" s="5" t="inlineStr"/>
@@ -19948,7 +19980,7 @@
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>LD04</t>
+          <t>LD01</t>
         </is>
       </c>
       <c r="B190" s="5" t="n">
@@ -19986,7 +20018,7 @@
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>LD02</t>
+          <t>LD04</t>
         </is>
       </c>
       <c r="B191" s="5" t="n">
@@ -20024,7 +20056,7 @@
     <row r="192">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>LD01</t>
+          <t>LD02</t>
         </is>
       </c>
       <c r="B192" s="5" t="n">
@@ -20608,12 +20640,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>WYASF1</t>
+          <t>JUNEESF1</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Wyalong Solar Farm</t>
+          <t>Junee Solar Farm</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -20637,12 +20669,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>SEBSF1</t>
+          <t>WYASF1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Sebastopol Solar Farm</t>
+          <t>Wyalong Solar Farm</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -20666,12 +20698,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>JUNEESF1</t>
+          <t>SEBSF1</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Junee Solar Farm</t>
+          <t>Sebastopol Solar Farm</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -21145,7 +21177,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>URANQ11</t>
+          <t>URANQ12</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -21174,7 +21206,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>URANQ12</t>
+          <t>URANQ11</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -21435,7 +21467,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL1</t>
+          <t>TUMT3NL3</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -21464,7 +21496,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL3</t>
+          <t>TUMT3NL2</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -21493,7 +21525,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>TUMT3NL2</t>
+          <t>TUMT3NL1</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">

</xml_diff>